<commit_message>
Actualizacion nocturna 10 nov
</commit_message>
<xml_diff>
--- a/Totales Docentes.xlsx
+++ b/Totales Docentes.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="60">
   <si>
     <t>Docente</t>
   </si>
@@ -109,6 +109,9 @@
   </si>
   <si>
     <t>Jiménez Nieto Enrique</t>
+  </si>
+  <si>
+    <t>Martínez Cruz Norma</t>
   </si>
   <si>
     <t>Martínez López Miguel Ángel</t>
@@ -550,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="50.7109375" customWidth="1"/>
@@ -593,16 +596,16 @@
         <v>130</v>
       </c>
       <c r="C2">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="D2">
-        <v>23.08</v>
+        <v>10</v>
       </c>
       <c r="E2">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="F2">
-        <v>76.92</v>
+        <v>90</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -611,7 +614,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>9</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -622,16 +625,16 @@
         <v>172</v>
       </c>
       <c r="C3">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>27.33</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>125</v>
+        <v>172</v>
       </c>
       <c r="F3">
-        <v>72.67</v>
+        <v>100</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -640,7 +643,7 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>9.699999999999999</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -651,25 +654,25 @@
         <v>203</v>
       </c>
       <c r="C4">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>37.93</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>126</v>
+        <v>160</v>
       </c>
       <c r="F4">
-        <v>62.07</v>
+        <v>78.81999999999999</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>21.18</v>
       </c>
       <c r="I4">
-        <v>8.4</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -709,10 +712,10 @@
         <v>74</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <v>1.35</v>
+        <v>0</v>
       </c>
       <c r="E6">
         <v>56</v>
@@ -721,13 +724,13 @@
         <v>75.68000000000001</v>
       </c>
       <c r="G6">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H6">
-        <v>22.97</v>
+        <v>24.32</v>
       </c>
       <c r="I6">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -764,7 +767,7 @@
         <v>15</v>
       </c>
       <c r="B8">
-        <v>169</v>
+        <v>148</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -773,16 +776,16 @@
         <v>0</v>
       </c>
       <c r="E8">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="F8">
-        <v>62.13</v>
+        <v>62.84</v>
       </c>
       <c r="G8">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="H8">
-        <v>37.87</v>
+        <v>37.16</v>
       </c>
       <c r="I8">
         <v>6.7</v>
@@ -796,25 +799,25 @@
         <v>99</v>
       </c>
       <c r="C9">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="D9">
-        <v>48.48</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="F9">
-        <v>51.52</v>
+        <v>66.67</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>33.33</v>
       </c>
       <c r="I9">
-        <v>9.1</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -825,16 +828,16 @@
         <v>176</v>
       </c>
       <c r="C10">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>31.25</v>
+        <v>0</v>
       </c>
       <c r="E10">
-        <v>121</v>
+        <v>176</v>
       </c>
       <c r="F10">
-        <v>68.75</v>
+        <v>100</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -843,7 +846,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>8.300000000000001</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -854,25 +857,25 @@
         <v>102</v>
       </c>
       <c r="C11">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="D11">
-        <v>27.45</v>
+        <v>0</v>
       </c>
       <c r="E11">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="F11">
-        <v>72.55</v>
+        <v>83.33</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="I11">
-        <v>8.300000000000001</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -883,25 +886,25 @@
         <v>51</v>
       </c>
       <c r="C12">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D12">
-        <v>39.22</v>
+        <v>0</v>
       </c>
       <c r="E12">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="F12">
-        <v>60.78</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>17.65</v>
       </c>
       <c r="I12">
-        <v>7.7</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -912,25 +915,25 @@
         <v>159</v>
       </c>
       <c r="C13">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="D13">
-        <v>26.42</v>
+        <v>15.72</v>
       </c>
       <c r="E13">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="F13">
-        <v>69.81</v>
+        <v>74.84</v>
       </c>
       <c r="G13">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="H13">
-        <v>3.77</v>
+        <v>9.43</v>
       </c>
       <c r="I13">
-        <v>8</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -941,25 +944,25 @@
         <v>189</v>
       </c>
       <c r="C14">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D14">
-        <v>12.17</v>
+        <v>9.52</v>
       </c>
       <c r="E14">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="F14">
-        <v>77.78</v>
+        <v>79.89</v>
       </c>
       <c r="G14">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H14">
-        <v>10.05</v>
+        <v>10.58</v>
       </c>
       <c r="I14">
-        <v>8</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -999,16 +1002,16 @@
         <v>211</v>
       </c>
       <c r="C16">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D16">
-        <v>18.96</v>
+        <v>12.8</v>
       </c>
       <c r="E16">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="F16">
-        <v>81.04000000000001</v>
+        <v>87.2</v>
       </c>
       <c r="G16">
         <v>0</v>
@@ -1017,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="I16">
-        <v>8.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -1028,16 +1031,16 @@
         <v>177</v>
       </c>
       <c r="C17">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="D17">
-        <v>27.68</v>
+        <v>19.21</v>
       </c>
       <c r="E17">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="F17">
-        <v>72.31999999999999</v>
+        <v>80.79000000000001</v>
       </c>
       <c r="G17">
         <v>0</v>
@@ -1046,7 +1049,7 @@
         <v>0</v>
       </c>
       <c r="I17">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1057,25 +1060,25 @@
         <v>146</v>
       </c>
       <c r="C18">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="D18">
-        <v>19.18</v>
+        <v>0.68</v>
       </c>
       <c r="E18">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="F18">
-        <v>80.81999999999999</v>
+        <v>83.56</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>15.75</v>
       </c>
       <c r="I18">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -1086,16 +1089,16 @@
         <v>228</v>
       </c>
       <c r="C19">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D19">
-        <v>9.210000000000001</v>
+        <v>7.89</v>
       </c>
       <c r="E19">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F19">
-        <v>71.93000000000001</v>
+        <v>73.25</v>
       </c>
       <c r="G19">
         <v>43</v>
@@ -1144,16 +1147,16 @@
         <v>120</v>
       </c>
       <c r="C21">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D21">
-        <v>35.83</v>
+        <v>35</v>
       </c>
       <c r="E21">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F21">
-        <v>64.17</v>
+        <v>65</v>
       </c>
       <c r="G21">
         <v>0</v>
@@ -1173,25 +1176,25 @@
         <v>211</v>
       </c>
       <c r="C22">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>20.85</v>
+        <v>0</v>
       </c>
       <c r="E22">
-        <v>167</v>
+        <v>195</v>
       </c>
       <c r="F22">
-        <v>79.15000000000001</v>
+        <v>92.42</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>7.58</v>
       </c>
       <c r="I22">
-        <v>7.4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -1228,28 +1231,28 @@
         <v>31</v>
       </c>
       <c r="B24">
-        <v>82</v>
+        <v>21</v>
       </c>
       <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
         <v>12</v>
       </c>
-      <c r="D24">
-        <v>14.63</v>
-      </c>
-      <c r="E24">
-        <v>66</v>
-      </c>
       <c r="F24">
-        <v>80.48999999999999</v>
+        <v>57.14</v>
       </c>
       <c r="G24">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H24">
-        <v>4.88</v>
+        <v>42.86</v>
       </c>
       <c r="I24">
-        <v>8.6</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1257,28 +1260,28 @@
         <v>32</v>
       </c>
       <c r="B25">
-        <v>104</v>
+        <v>82</v>
       </c>
       <c r="C25">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D25">
-        <v>0</v>
+        <v>14.63</v>
       </c>
       <c r="E25">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F25">
-        <v>64.42</v>
+        <v>80.48999999999999</v>
       </c>
       <c r="G25">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="H25">
-        <v>35.58</v>
+        <v>4.88</v>
       </c>
       <c r="I25">
-        <v>6.4</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -1286,28 +1289,28 @@
         <v>33</v>
       </c>
       <c r="B26">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C26">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="D26">
-        <v>48.15</v>
+        <v>0</v>
       </c>
       <c r="E26">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="F26">
-        <v>51.85</v>
+        <v>64.42</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="H26">
-        <v>0</v>
+        <v>35.58</v>
       </c>
       <c r="I26">
-        <v>8.6</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1315,28 +1318,28 @@
         <v>34</v>
       </c>
       <c r="B27">
-        <v>71</v>
+        <v>108</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="D27">
-        <v>0</v>
+        <v>39.81</v>
       </c>
       <c r="E27">
         <v>60</v>
       </c>
       <c r="F27">
-        <v>84.51000000000001</v>
+        <v>55.56</v>
       </c>
       <c r="G27">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="H27">
-        <v>15.49</v>
+        <v>4.63</v>
       </c>
       <c r="I27">
-        <v>7.8</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1344,28 +1347,28 @@
         <v>35</v>
       </c>
       <c r="B28">
-        <v>137</v>
+        <v>71</v>
       </c>
       <c r="C28">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="D28">
-        <v>26.28</v>
+        <v>0</v>
       </c>
       <c r="E28">
-        <v>101</v>
+        <v>60</v>
       </c>
       <c r="F28">
-        <v>73.72</v>
+        <v>84.51000000000001</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H28">
-        <v>0</v>
+        <v>15.49</v>
       </c>
       <c r="I28">
-        <v>10</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1373,19 +1376,19 @@
         <v>36</v>
       </c>
       <c r="B29">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="C29">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D29">
-        <v>22.22</v>
+        <v>10.95</v>
       </c>
       <c r="E29">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F29">
-        <v>77.78</v>
+        <v>89.05</v>
       </c>
       <c r="G29">
         <v>0</v>
@@ -1394,7 +1397,7 @@
         <v>0</v>
       </c>
       <c r="I29">
-        <v>8.1</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -1402,28 +1405,28 @@
         <v>37</v>
       </c>
       <c r="B30">
-        <v>24</v>
+        <v>153</v>
       </c>
       <c r="C30">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>9.15</v>
       </c>
       <c r="E30">
-        <v>24</v>
+        <v>135</v>
       </c>
       <c r="F30">
-        <v>100</v>
+        <v>88.23999999999999</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H30">
-        <v>0</v>
+        <v>2.61</v>
       </c>
       <c r="I30">
-        <v>8.800000000000001</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -1431,28 +1434,28 @@
         <v>38</v>
       </c>
       <c r="B31">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="C31">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="D31">
-        <v>23.15</v>
+        <v>0</v>
       </c>
       <c r="E31">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="F31">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H31">
-        <v>1.85</v>
+        <v>0</v>
       </c>
       <c r="I31">
-        <v>8.1</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -1460,28 +1463,28 @@
         <v>39</v>
       </c>
       <c r="B32">
-        <v>247</v>
+        <v>108</v>
       </c>
       <c r="C32">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="D32">
-        <v>31.17</v>
+        <v>16.67</v>
       </c>
       <c r="E32">
-        <v>170</v>
+        <v>82</v>
       </c>
       <c r="F32">
-        <v>68.83</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H32">
-        <v>0</v>
+        <v>7.41</v>
       </c>
       <c r="I32">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -1489,28 +1492,28 @@
         <v>40</v>
       </c>
       <c r="B33">
-        <v>222</v>
+        <v>247</v>
       </c>
       <c r="C33">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="D33">
-        <v>21.62</v>
+        <v>0.4</v>
       </c>
       <c r="E33">
-        <v>174</v>
+        <v>188</v>
       </c>
       <c r="F33">
-        <v>78.38</v>
+        <v>76.11</v>
       </c>
       <c r="G33">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="H33">
-        <v>0</v>
+        <v>23.48</v>
       </c>
       <c r="I33">
-        <v>7.6</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -1521,25 +1524,25 @@
         <v>222</v>
       </c>
       <c r="C34">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="D34">
-        <v>10.36</v>
+        <v>0.9</v>
       </c>
       <c r="E34">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="F34">
-        <v>85.59</v>
+        <v>82.88</v>
       </c>
       <c r="G34">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="H34">
-        <v>4.05</v>
+        <v>16.22</v>
       </c>
       <c r="I34">
-        <v>8.199999999999999</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -1547,28 +1550,28 @@
         <v>42</v>
       </c>
       <c r="B35">
-        <v>162</v>
+        <v>222</v>
       </c>
       <c r="C35">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="D35">
-        <v>25.31</v>
+        <v>3.15</v>
       </c>
       <c r="E35">
-        <v>75</v>
+        <v>192</v>
       </c>
       <c r="F35">
-        <v>46.3</v>
+        <v>86.48999999999999</v>
       </c>
       <c r="G35">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="H35">
-        <v>28.4</v>
+        <v>10.36</v>
       </c>
       <c r="I35">
-        <v>6.6</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -1576,28 +1579,28 @@
         <v>43</v>
       </c>
       <c r="B36">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="C36">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D36">
-        <v>26.39</v>
+        <v>25.31</v>
       </c>
       <c r="E36">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="F36">
-        <v>70.14</v>
+        <v>46.3</v>
       </c>
       <c r="G36">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="H36">
-        <v>3.47</v>
+        <v>28.4</v>
       </c>
       <c r="I36">
-        <v>7.6</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -1605,7 +1608,7 @@
         <v>44</v>
       </c>
       <c r="B37">
-        <v>65</v>
+        <v>144</v>
       </c>
       <c r="C37">
         <v>0</v>
@@ -1614,19 +1617,19 @@
         <v>0</v>
       </c>
       <c r="E37">
-        <v>65</v>
+        <v>111</v>
       </c>
       <c r="F37">
-        <v>100</v>
+        <v>77.08</v>
       </c>
       <c r="G37">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>22.92</v>
       </c>
       <c r="I37">
-        <v>8.1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -1634,19 +1637,19 @@
         <v>45</v>
       </c>
       <c r="B38">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C38">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="D38">
-        <v>24.66</v>
+        <v>0</v>
       </c>
       <c r="E38">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="F38">
-        <v>75.34</v>
+        <v>100</v>
       </c>
       <c r="G38">
         <v>0</v>
@@ -1655,7 +1658,7 @@
         <v>0</v>
       </c>
       <c r="I38">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -1663,28 +1666,28 @@
         <v>46</v>
       </c>
       <c r="B39">
-        <v>143</v>
+        <v>73</v>
       </c>
       <c r="C39">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="D39">
-        <v>47.55</v>
+        <v>0</v>
       </c>
       <c r="E39">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="F39">
-        <v>52.45</v>
+        <v>86.3</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H39">
-        <v>0</v>
+        <v>13.7</v>
       </c>
       <c r="I39">
-        <v>7.4</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -1692,28 +1695,28 @@
         <v>47</v>
       </c>
       <c r="B40">
-        <v>203</v>
+        <v>143</v>
       </c>
       <c r="C40">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D40">
-        <v>0.99</v>
+        <v>0</v>
       </c>
       <c r="E40">
-        <v>167</v>
+        <v>96</v>
       </c>
       <c r="F40">
-        <v>82.27</v>
+        <v>67.13</v>
       </c>
       <c r="G40">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="H40">
-        <v>16.75</v>
+        <v>32.87</v>
       </c>
       <c r="I40">
-        <v>7.1</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -1721,28 +1724,28 @@
         <v>48</v>
       </c>
       <c r="B41">
-        <v>72</v>
+        <v>203</v>
       </c>
       <c r="C41">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="D41">
-        <v>31.94</v>
+        <v>0.99</v>
       </c>
       <c r="E41">
-        <v>49</v>
+        <v>167</v>
       </c>
       <c r="F41">
-        <v>68.06</v>
+        <v>82.27</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="H41">
-        <v>0</v>
+        <v>16.75</v>
       </c>
       <c r="I41">
-        <v>7.5</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -1750,28 +1753,28 @@
         <v>49</v>
       </c>
       <c r="B42">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="C42">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="D42">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E42">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="F42">
-        <v>70</v>
+        <v>79.17</v>
       </c>
       <c r="G42">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H42">
-        <v>0</v>
+        <v>20.83</v>
       </c>
       <c r="I42">
-        <v>8.300000000000001</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -1779,25 +1782,25 @@
         <v>50</v>
       </c>
       <c r="B43">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C43">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D43">
-        <v>42.42</v>
+        <v>0</v>
       </c>
       <c r="E43">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F43">
-        <v>57.58</v>
+        <v>75</v>
       </c>
       <c r="G43">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H43">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I43">
         <v>7.4</v>
@@ -1808,19 +1811,19 @@
         <v>51</v>
       </c>
       <c r="B44">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="C44">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D44">
-        <v>28.81</v>
+        <v>42.42</v>
       </c>
       <c r="E44">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="F44">
-        <v>71.19</v>
+        <v>57.58</v>
       </c>
       <c r="G44">
         <v>0</v>
@@ -1829,7 +1832,7 @@
         <v>0</v>
       </c>
       <c r="I44">
-        <v>8.800000000000001</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -1837,28 +1840,28 @@
         <v>52</v>
       </c>
       <c r="B45">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="C45">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D45">
-        <v>2.78</v>
+        <v>0</v>
       </c>
       <c r="E45">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="F45">
-        <v>50</v>
+        <v>84.75</v>
       </c>
       <c r="G45">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="H45">
-        <v>47.22</v>
+        <v>15.25</v>
       </c>
       <c r="I45">
-        <v>6.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -1866,28 +1869,28 @@
         <v>53</v>
       </c>
       <c r="B46">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="C46">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="D46">
-        <v>40.22</v>
+        <v>2.78</v>
       </c>
       <c r="E46">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="F46">
-        <v>59.78</v>
+        <v>50</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="H46">
-        <v>0</v>
+        <v>47.22</v>
       </c>
       <c r="I46">
-        <v>8.5</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -1895,28 +1898,28 @@
         <v>54</v>
       </c>
       <c r="B47">
-        <v>158</v>
+        <v>92</v>
       </c>
       <c r="C47">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D47">
-        <v>1.27</v>
+        <v>16.3</v>
       </c>
       <c r="E47">
-        <v>108</v>
+        <v>77</v>
       </c>
       <c r="F47">
-        <v>68.34999999999999</v>
+        <v>83.7</v>
       </c>
       <c r="G47">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="H47">
-        <v>30.38</v>
+        <v>0</v>
       </c>
       <c r="I47">
-        <v>7.1</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -1924,28 +1927,28 @@
         <v>55</v>
       </c>
       <c r="B48">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="C48">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="D48">
-        <v>31.76</v>
+        <v>1.27</v>
       </c>
       <c r="E48">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="F48">
-        <v>67.56999999999999</v>
+        <v>68.34999999999999</v>
       </c>
       <c r="G48">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="H48">
-        <v>0.68</v>
+        <v>30.38</v>
       </c>
       <c r="I48">
-        <v>6.8</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -1953,28 +1956,28 @@
         <v>56</v>
       </c>
       <c r="B49">
-        <v>90</v>
+        <v>148</v>
       </c>
       <c r="C49">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D49">
-        <v>44.44</v>
+        <v>20.95</v>
       </c>
       <c r="E49">
-        <v>50</v>
+        <v>116</v>
       </c>
       <c r="F49">
-        <v>55.56</v>
+        <v>78.38</v>
       </c>
       <c r="G49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H49">
-        <v>0</v>
+        <v>0.68</v>
       </c>
       <c r="I49">
-        <v>8.6</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -1982,7 +1985,7 @@
         <v>57</v>
       </c>
       <c r="B50">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="C50">
         <v>0</v>
@@ -1991,19 +1994,19 @@
         <v>0</v>
       </c>
       <c r="E50">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="F50">
-        <v>87.5</v>
+        <v>75.56</v>
       </c>
       <c r="G50">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="H50">
-        <v>12.5</v>
+        <v>24.44</v>
       </c>
       <c r="I50">
-        <v>8.699999999999999</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -2011,27 +2014,56 @@
         <v>58</v>
       </c>
       <c r="B51">
+        <v>104</v>
+      </c>
+      <c r="C51">
+        <v>0</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51">
+        <v>91</v>
+      </c>
+      <c r="F51">
+        <v>87.5</v>
+      </c>
+      <c r="G51">
+        <v>13</v>
+      </c>
+      <c r="H51">
+        <v>12.5</v>
+      </c>
+      <c r="I51">
+        <v>8.699999999999999</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52">
         <v>108</v>
       </c>
-      <c r="C51">
-        <v>2</v>
-      </c>
-      <c r="D51">
-        <v>1.85</v>
-      </c>
-      <c r="E51">
+      <c r="C52">
+        <v>0</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52">
         <v>88</v>
       </c>
-      <c r="F51">
+      <c r="F52">
         <v>81.48</v>
       </c>
-      <c r="G51">
-        <v>18</v>
-      </c>
-      <c r="H51">
-        <v>16.67</v>
-      </c>
-      <c r="I51">
+      <c r="G52">
+        <v>20</v>
+      </c>
+      <c r="H52">
+        <v>18.52</v>
+      </c>
+      <c r="I52">
         <v>7.6</v>
       </c>
     </row>
@@ -2042,7 +2074,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="50.7109375" customWidth="1"/>
@@ -2085,22 +2117,25 @@
         <v>130</v>
       </c>
       <c r="C2">
-        <v>130</v>
+        <v>13</v>
       </c>
       <c r="D2">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>117</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="G2">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <v>76.92</v>
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>8.4</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2111,22 +2146,25 @@
         <v>172</v>
       </c>
       <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
         <v>172</v>
       </c>
-      <c r="D3">
+      <c r="F3">
         <v>100</v>
       </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
       <c r="G3">
-        <v>125</v>
+        <v>0</v>
       </c>
       <c r="H3">
-        <v>72.67</v>
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>9.1</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2137,22 +2175,25 @@
         <v>203</v>
       </c>
       <c r="C4">
-        <v>203</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>78.81999999999999</v>
       </c>
       <c r="G4">
-        <v>126</v>
+        <v>43</v>
       </c>
       <c r="H4">
-        <v>62.07</v>
+        <v>21.18</v>
+      </c>
+      <c r="I4">
+        <v>7.5</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2189,22 +2230,25 @@
         <v>74</v>
       </c>
       <c r="C6">
-        <v>74</v>
+        <v>8</v>
       </c>
       <c r="D6">
-        <v>100</v>
+        <v>10.81</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>78.38</v>
       </c>
       <c r="G6">
-        <v>73</v>
+        <v>16</v>
       </c>
       <c r="H6">
-        <v>98.65000000000001</v>
+        <v>21.62</v>
+      </c>
+      <c r="I6">
+        <v>7.7</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2215,22 +2259,25 @@
         <v>91</v>
       </c>
       <c r="C7">
-        <v>91</v>
+        <v>1</v>
       </c>
       <c r="D7">
-        <v>100</v>
+        <v>1.1</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>59.34</v>
       </c>
       <c r="G7">
-        <v>91</v>
+        <v>37</v>
       </c>
       <c r="H7">
-        <v>100</v>
+        <v>40.66</v>
+      </c>
+      <c r="I7">
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2238,25 +2285,28 @@
         <v>15</v>
       </c>
       <c r="B8">
-        <v>169</v>
+        <v>148</v>
       </c>
       <c r="C8">
-        <v>169</v>
+        <v>21</v>
       </c>
       <c r="D8">
-        <v>100</v>
+        <v>14.19</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>68.92</v>
       </c>
       <c r="G8">
-        <v>169</v>
+        <v>46</v>
       </c>
       <c r="H8">
-        <v>100</v>
+        <v>31.08</v>
+      </c>
+      <c r="I8">
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2267,22 +2317,25 @@
         <v>99</v>
       </c>
       <c r="C9">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="D9">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>64.65000000000001</v>
       </c>
       <c r="G9">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="H9">
-        <v>51.52</v>
+        <v>35.35</v>
+      </c>
+      <c r="I9">
+        <v>7.3</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2293,22 +2346,25 @@
         <v>176</v>
       </c>
       <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
         <v>176</v>
       </c>
-      <c r="D10">
+      <c r="F10">
         <v>100</v>
       </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
       <c r="G10">
-        <v>121</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>68.75</v>
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>7.9</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -2319,22 +2375,25 @@
         <v>102</v>
       </c>
       <c r="C11">
-        <v>102</v>
+        <v>0</v>
       </c>
       <c r="D11">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>81.37</v>
       </c>
       <c r="G11">
-        <v>74</v>
+        <v>19</v>
       </c>
       <c r="H11">
-        <v>72.55</v>
+        <v>18.63</v>
+      </c>
+      <c r="I11">
+        <v>7.3</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -2345,22 +2404,25 @@
         <v>51</v>
       </c>
       <c r="C12">
-        <v>51</v>
+        <v>11</v>
       </c>
       <c r="D12">
-        <v>100</v>
+        <v>21.57</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>78.43000000000001</v>
       </c>
       <c r="G12">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="H12">
-        <v>60.78</v>
+        <v>21.57</v>
+      </c>
+      <c r="I12">
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -2371,22 +2433,25 @@
         <v>159</v>
       </c>
       <c r="C13">
-        <v>159</v>
+        <v>41</v>
       </c>
       <c r="D13">
-        <v>100</v>
+        <v>25.79</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>59.75</v>
       </c>
       <c r="G13">
-        <v>117</v>
+        <v>39</v>
       </c>
       <c r="H13">
-        <v>73.58</v>
+        <v>24.53</v>
+      </c>
+      <c r="I13">
+        <v>7.3</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -2397,22 +2462,25 @@
         <v>189</v>
       </c>
       <c r="C14">
-        <v>189</v>
+        <v>21</v>
       </c>
       <c r="D14">
-        <v>100</v>
+        <v>11.11</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>156</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>82.54000000000001</v>
       </c>
       <c r="G14">
-        <v>166</v>
+        <v>15</v>
       </c>
       <c r="H14">
-        <v>87.83</v>
+        <v>7.94</v>
+      </c>
+      <c r="I14">
+        <v>7.7</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -2423,22 +2491,25 @@
         <v>96</v>
       </c>
       <c r="C15">
-        <v>96</v>
+        <v>30</v>
       </c>
       <c r="D15">
-        <v>100</v>
+        <v>31.25</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>68.75</v>
       </c>
       <c r="G15">
-        <v>96</v>
+        <v>30</v>
       </c>
       <c r="H15">
-        <v>100</v>
+        <v>31.25</v>
+      </c>
+      <c r="I15">
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -2449,25 +2520,28 @@
         <v>211</v>
       </c>
       <c r="C16">
-        <v>211</v>
+        <v>45</v>
       </c>
       <c r="D16">
-        <v>100</v>
+        <v>21.33</v>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>166</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>78.67</v>
       </c>
       <c r="G16">
-        <v>171</v>
+        <v>18</v>
       </c>
       <c r="H16">
-        <v>81.04000000000001</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
+        <v>8.529999999999999</v>
+      </c>
+      <c r="I16">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -2475,25 +2549,28 @@
         <v>177</v>
       </c>
       <c r="C17">
-        <v>177</v>
+        <v>46</v>
       </c>
       <c r="D17">
-        <v>100</v>
+        <v>25.99</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>131</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>74.01000000000001</v>
       </c>
       <c r="G17">
-        <v>128</v>
+        <v>12</v>
       </c>
       <c r="H17">
-        <v>72.31999999999999</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
+        <v>6.78</v>
+      </c>
+      <c r="I17">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>25</v>
       </c>
@@ -2501,25 +2578,28 @@
         <v>146</v>
       </c>
       <c r="C18">
-        <v>146</v>
+        <v>36</v>
       </c>
       <c r="D18">
-        <v>100</v>
+        <v>24.66</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>103</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>70.55</v>
       </c>
       <c r="G18">
-        <v>118</v>
+        <v>42</v>
       </c>
       <c r="H18">
-        <v>80.81999999999999</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
+        <v>28.77</v>
+      </c>
+      <c r="I18">
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -2527,25 +2607,28 @@
         <v>228</v>
       </c>
       <c r="C19">
-        <v>228</v>
+        <v>140</v>
       </c>
       <c r="D19">
-        <v>100</v>
+        <v>61.4</v>
       </c>
       <c r="E19">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>36.84</v>
       </c>
       <c r="G19">
-        <v>207</v>
+        <v>126</v>
       </c>
       <c r="H19">
-        <v>90.79000000000001</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
+        <v>55.26</v>
+      </c>
+      <c r="I19">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -2571,7 +2654,7 @@
         <v>95.7</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:9">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -2579,25 +2662,28 @@
         <v>120</v>
       </c>
       <c r="C21">
-        <v>120</v>
+        <v>59</v>
       </c>
       <c r="D21">
-        <v>100</v>
+        <v>49.17</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>50.83</v>
       </c>
       <c r="G21">
-        <v>77</v>
+        <v>17</v>
       </c>
       <c r="H21">
-        <v>64.17</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
+        <v>14.17</v>
+      </c>
+      <c r="I21">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -2605,25 +2691,28 @@
         <v>211</v>
       </c>
       <c r="C22">
-        <v>211</v>
+        <v>41</v>
       </c>
       <c r="D22">
-        <v>100</v>
+        <v>19.43</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>79.62</v>
       </c>
       <c r="G22">
-        <v>167</v>
+        <v>43</v>
       </c>
       <c r="H22">
-        <v>79.15000000000001</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
+        <v>20.38</v>
+      </c>
+      <c r="I22">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -2649,41 +2738,44 @@
         <v>73.33</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:9">
       <c r="A24" t="s">
         <v>31</v>
       </c>
       <c r="B24">
-        <v>82</v>
+        <v>21</v>
       </c>
       <c r="C24">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="D24">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>76.19</v>
       </c>
       <c r="G24">
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="H24">
-        <v>85.37</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8">
+        <v>23.81</v>
+      </c>
+      <c r="I24">
+        <v>8.300000000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
       <c r="A25" t="s">
         <v>32</v>
       </c>
       <c r="B25">
-        <v>104</v>
+        <v>82</v>
       </c>
       <c r="C25">
-        <v>104</v>
+        <v>82</v>
       </c>
       <c r="D25">
         <v>100</v>
@@ -2695,221 +2787,245 @@
         <v>0</v>
       </c>
       <c r="G25">
-        <v>104</v>
+        <v>70</v>
       </c>
       <c r="H25">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
+        <v>85.37</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
       <c r="A26" t="s">
         <v>33</v>
       </c>
       <c r="B26">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C26">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="D26">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="G26">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="H26">
-        <v>51.85</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8">
+        <v>25</v>
+      </c>
+      <c r="I26">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
       <c r="A27" t="s">
         <v>34</v>
       </c>
       <c r="B27">
-        <v>71</v>
+        <v>108</v>
       </c>
       <c r="C27">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D27">
-        <v>100</v>
+        <v>62.04</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>37.96</v>
       </c>
       <c r="G27">
-        <v>71</v>
+        <v>24</v>
       </c>
       <c r="H27">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8">
+        <v>22.22</v>
+      </c>
+      <c r="I27">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
       <c r="A28" t="s">
         <v>35</v>
       </c>
       <c r="B28">
-        <v>137</v>
+        <v>71</v>
       </c>
       <c r="C28">
-        <v>137</v>
+        <v>0</v>
       </c>
       <c r="D28">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E28">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="F28">
-        <v>0</v>
+        <v>81.69</v>
       </c>
       <c r="G28">
-        <v>101</v>
+        <v>13</v>
       </c>
       <c r="H28">
-        <v>73.72</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8">
+        <v>18.31</v>
+      </c>
+      <c r="I28">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
       <c r="A29" t="s">
         <v>36</v>
       </c>
       <c r="B29">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="C29">
-        <v>153</v>
+        <v>36</v>
       </c>
       <c r="D29">
-        <v>100</v>
+        <v>26.28</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>73.72</v>
       </c>
       <c r="G29">
-        <v>119</v>
+        <v>21</v>
       </c>
       <c r="H29">
-        <v>77.78</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8">
+        <v>15.33</v>
+      </c>
+      <c r="I29">
+        <v>8.699999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
       <c r="A30" t="s">
         <v>37</v>
       </c>
       <c r="B30">
-        <v>24</v>
+        <v>153</v>
       </c>
       <c r="C30">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D30">
-        <v>100</v>
+        <v>18.95</v>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>122</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>79.73999999999999</v>
       </c>
       <c r="G30">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="H30">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8">
+        <v>11.11</v>
+      </c>
+      <c r="I30">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
       <c r="A31" t="s">
         <v>38</v>
       </c>
       <c r="B31">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="C31">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>24</v>
+      </c>
+      <c r="F31">
         <v>100</v>
       </c>
-      <c r="E31">
-        <v>0</v>
-      </c>
-      <c r="F31">
-        <v>0</v>
-      </c>
       <c r="G31">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="H31">
-        <v>76.84999999999999</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I31">
+        <v>9.199999999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
       <c r="A32" t="s">
         <v>39</v>
       </c>
       <c r="B32">
-        <v>247</v>
+        <v>108</v>
       </c>
       <c r="C32">
-        <v>247</v>
+        <v>33</v>
       </c>
       <c r="D32">
-        <v>100</v>
+        <v>30.56</v>
       </c>
       <c r="E32">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F32">
-        <v>0</v>
+        <v>69.44</v>
       </c>
       <c r="G32">
-        <v>170</v>
+        <v>15</v>
       </c>
       <c r="H32">
-        <v>68.83</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8">
+        <v>13.89</v>
+      </c>
+      <c r="I32">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
       <c r="A33" t="s">
         <v>40</v>
       </c>
       <c r="B33">
-        <v>222</v>
+        <v>247</v>
       </c>
       <c r="C33">
-        <v>222</v>
+        <v>1</v>
       </c>
       <c r="D33">
-        <v>100</v>
+        <v>0.4</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>182</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>73.68000000000001</v>
       </c>
       <c r="G33">
-        <v>174</v>
+        <v>64</v>
       </c>
       <c r="H33">
-        <v>78.38</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8">
+        <v>25.91</v>
+      </c>
+      <c r="I33">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
       <c r="A34" t="s">
         <v>41</v>
       </c>
@@ -2917,59 +3033,65 @@
         <v>222</v>
       </c>
       <c r="C34">
-        <v>222</v>
+        <v>5</v>
       </c>
       <c r="D34">
-        <v>100</v>
+        <v>2.25</v>
       </c>
       <c r="E34">
-        <v>0</v>
+        <v>183</v>
       </c>
       <c r="F34">
-        <v>0</v>
+        <v>82.43000000000001</v>
       </c>
       <c r="G34">
-        <v>199</v>
+        <v>37</v>
       </c>
       <c r="H34">
-        <v>89.64</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8">
+        <v>16.67</v>
+      </c>
+      <c r="I34">
+        <v>7.4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
       <c r="A35" t="s">
         <v>42</v>
       </c>
       <c r="B35">
-        <v>162</v>
+        <v>222</v>
       </c>
       <c r="C35">
-        <v>162</v>
+        <v>35</v>
       </c>
       <c r="D35">
-        <v>100</v>
+        <v>15.77</v>
       </c>
       <c r="E35">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="F35">
-        <v>0</v>
+        <v>72.52</v>
       </c>
       <c r="G35">
-        <v>121</v>
+        <v>54</v>
       </c>
       <c r="H35">
-        <v>74.69</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8">
+        <v>24.32</v>
+      </c>
+      <c r="I35">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
       <c r="A36" t="s">
         <v>43</v>
       </c>
       <c r="B36">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="C36">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="D36">
         <v>100</v>
@@ -2981,125 +3103,137 @@
         <v>0</v>
       </c>
       <c r="G36">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="H36">
-        <v>73.61</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8">
+        <v>74.69</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
       <c r="A37" t="s">
         <v>44</v>
       </c>
       <c r="B37">
-        <v>65</v>
+        <v>144</v>
       </c>
       <c r="C37">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D37">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E37">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="F37">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G37">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="H37">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
+        <v>50</v>
+      </c>
+      <c r="I37">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
       <c r="A38" t="s">
         <v>45</v>
       </c>
       <c r="B38">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C38">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>65</v>
+      </c>
+      <c r="F38">
         <v>100</v>
       </c>
-      <c r="E38">
-        <v>0</v>
-      </c>
-      <c r="F38">
-        <v>0</v>
-      </c>
       <c r="G38">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="H38">
-        <v>75.34</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
       <c r="A39" t="s">
         <v>46</v>
       </c>
       <c r="B39">
-        <v>143</v>
+        <v>73</v>
       </c>
       <c r="C39">
-        <v>143</v>
+        <v>12</v>
       </c>
       <c r="D39">
-        <v>100</v>
+        <v>16.44</v>
       </c>
       <c r="E39">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="F39">
-        <v>0</v>
+        <v>79.45</v>
       </c>
       <c r="G39">
-        <v>75</v>
+        <v>15</v>
       </c>
       <c r="H39">
-        <v>52.45</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8">
+        <v>20.55</v>
+      </c>
+      <c r="I39">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
       <c r="A40" t="s">
         <v>47</v>
       </c>
       <c r="B40">
-        <v>203</v>
+        <v>143</v>
       </c>
       <c r="C40">
-        <v>203</v>
+        <v>68</v>
       </c>
       <c r="D40">
-        <v>100</v>
+        <v>47.55</v>
       </c>
       <c r="E40">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F40">
-        <v>0</v>
+        <v>48.95</v>
       </c>
       <c r="G40">
-        <v>201</v>
+        <v>73</v>
       </c>
       <c r="H40">
-        <v>99.01000000000001</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8">
+        <v>51.05</v>
+      </c>
+      <c r="I40">
+        <v>6.9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
       <c r="A41" t="s">
         <v>48</v>
       </c>
       <c r="B41">
-        <v>72</v>
+        <v>203</v>
       </c>
       <c r="C41">
-        <v>72</v>
+        <v>203</v>
       </c>
       <c r="D41">
         <v>100</v>
@@ -3111,73 +3245,79 @@
         <v>0</v>
       </c>
       <c r="G41">
-        <v>49</v>
+        <v>201</v>
       </c>
       <c r="H41">
-        <v>68.06</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8">
+        <v>99.01000000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
       <c r="A42" t="s">
         <v>49</v>
       </c>
       <c r="B42">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="C42">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D42">
-        <v>100</v>
+        <v>41.67</v>
       </c>
       <c r="E42">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="F42">
-        <v>0</v>
+        <v>58.33</v>
       </c>
       <c r="G42">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H42">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8">
+        <v>41.67</v>
+      </c>
+      <c r="I42">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
       <c r="A43" t="s">
         <v>50</v>
       </c>
       <c r="B43">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C43">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="D43">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="E43">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F43">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="G43">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="H43">
-        <v>57.58</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8">
+        <v>25</v>
+      </c>
+      <c r="I43">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
       <c r="A44" t="s">
         <v>51</v>
       </c>
       <c r="B44">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="C44">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="D44">
         <v>100</v>
@@ -3189,47 +3329,50 @@
         <v>0</v>
       </c>
       <c r="G44">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="H44">
-        <v>71.19</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8">
+        <v>57.58</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
       <c r="A45" t="s">
         <v>52</v>
       </c>
       <c r="B45">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="C45">
-        <v>72</v>
+        <v>9</v>
       </c>
       <c r="D45">
-        <v>100</v>
+        <v>15.25</v>
       </c>
       <c r="E45">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F45">
-        <v>0</v>
+        <v>84.75</v>
       </c>
       <c r="G45">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="H45">
-        <v>97.22</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8">
+        <v>15.25</v>
+      </c>
+      <c r="I45">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
       <c r="A46" t="s">
         <v>53</v>
       </c>
       <c r="B46">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="C46">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="D46">
         <v>100</v>
@@ -3241,47 +3384,50 @@
         <v>0</v>
       </c>
       <c r="G46">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="H46">
-        <v>59.78</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8">
+        <v>97.22</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9">
       <c r="A47" t="s">
         <v>54</v>
       </c>
       <c r="B47">
-        <v>158</v>
+        <v>92</v>
       </c>
       <c r="C47">
-        <v>158</v>
+        <v>19</v>
       </c>
       <c r="D47">
-        <v>100</v>
+        <v>20.65</v>
       </c>
       <c r="E47">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="F47">
-        <v>0</v>
+        <v>79.34999999999999</v>
       </c>
       <c r="G47">
-        <v>156</v>
+        <v>4</v>
       </c>
       <c r="H47">
-        <v>98.73</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8">
+        <v>4.35</v>
+      </c>
+      <c r="I47">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
       <c r="A48" t="s">
         <v>55</v>
       </c>
       <c r="B48">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="C48">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="D48">
         <v>100</v>
@@ -3293,88 +3439,126 @@
         <v>0</v>
       </c>
       <c r="G48">
-        <v>101</v>
+        <v>156</v>
       </c>
       <c r="H48">
-        <v>68.23999999999999</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8">
+        <v>98.73</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
       <c r="A49" t="s">
         <v>56</v>
       </c>
       <c r="B49">
-        <v>90</v>
+        <v>148</v>
       </c>
       <c r="C49">
-        <v>90</v>
+        <v>33</v>
       </c>
       <c r="D49">
-        <v>100</v>
+        <v>22.3</v>
       </c>
       <c r="E49">
-        <v>0</v>
+        <v>115</v>
       </c>
       <c r="F49">
-        <v>0</v>
+        <v>77.7</v>
       </c>
       <c r="G49">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="H49">
-        <v>55.56</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8">
+        <v>1.35</v>
+      </c>
+      <c r="I49">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
       <c r="A50" t="s">
         <v>57</v>
       </c>
       <c r="B50">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="C50">
-        <v>104</v>
+        <v>47</v>
       </c>
       <c r="D50">
-        <v>100</v>
+        <v>52.22</v>
       </c>
       <c r="E50">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="F50">
-        <v>0</v>
+        <v>47.78</v>
       </c>
       <c r="G50">
-        <v>104</v>
+        <v>47</v>
       </c>
       <c r="H50">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8">
+        <v>52.22</v>
+      </c>
+      <c r="I50">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9">
       <c r="A51" t="s">
         <v>58</v>
       </c>
       <c r="B51">
+        <v>104</v>
+      </c>
+      <c r="C51">
+        <v>0</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51">
+        <v>92</v>
+      </c>
+      <c r="F51">
+        <v>88.45999999999999</v>
+      </c>
+      <c r="G51">
+        <v>12</v>
+      </c>
+      <c r="H51">
+        <v>11.54</v>
+      </c>
+      <c r="I51">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52">
         <v>108</v>
       </c>
-      <c r="C51">
-        <v>108</v>
-      </c>
-      <c r="D51">
-        <v>100</v>
-      </c>
-      <c r="E51">
-        <v>0</v>
-      </c>
-      <c r="F51">
-        <v>0</v>
-      </c>
-      <c r="G51">
-        <v>106</v>
-      </c>
-      <c r="H51">
-        <v>98.15000000000001</v>
+      <c r="C52">
+        <v>6</v>
+      </c>
+      <c r="D52">
+        <v>5.56</v>
+      </c>
+      <c r="E52">
+        <v>82</v>
+      </c>
+      <c r="F52">
+        <v>75.93000000000001</v>
+      </c>
+      <c r="G52">
+        <v>26</v>
+      </c>
+      <c r="H52">
+        <v>24.07</v>
+      </c>
+      <c r="I52">
+        <v>7.4</v>
       </c>
     </row>
   </sheetData>
@@ -3384,7 +3568,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="50.7109375" customWidth="1"/>
@@ -3427,16 +3611,16 @@
         <v>130</v>
       </c>
       <c r="C2">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="D2">
-        <v>23.08</v>
+        <v>10</v>
       </c>
       <c r="E2">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="F2">
-        <v>76.92</v>
+        <v>90</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -3445,7 +3629,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>9</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -3456,16 +3640,16 @@
         <v>172</v>
       </c>
       <c r="C3">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>27.33</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>125</v>
+        <v>172</v>
       </c>
       <c r="F3">
-        <v>72.67</v>
+        <v>100</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -3474,7 +3658,7 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>9.699999999999999</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -3485,25 +3669,25 @@
         <v>203</v>
       </c>
       <c r="C4">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>37.93</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>126</v>
+        <v>160</v>
       </c>
       <c r="F4">
-        <v>62.07</v>
+        <v>78.81999999999999</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>21.18</v>
       </c>
       <c r="I4">
-        <v>8.4</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -3543,25 +3727,25 @@
         <v>74</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <v>1.35</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F6">
-        <v>75.68000000000001</v>
+        <v>83.78</v>
       </c>
       <c r="G6">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H6">
-        <v>22.97</v>
+        <v>16.22</v>
       </c>
       <c r="I6">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -3578,19 +3762,19 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F7">
-        <v>57.14</v>
+        <v>59.34</v>
       </c>
       <c r="G7">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H7">
-        <v>42.86</v>
+        <v>40.66</v>
       </c>
       <c r="I7">
-        <v>7</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -3598,7 +3782,7 @@
         <v>15</v>
       </c>
       <c r="B8">
-        <v>169</v>
+        <v>148</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -3607,19 +3791,19 @@
         <v>0</v>
       </c>
       <c r="E8">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="F8">
-        <v>62.13</v>
+        <v>77.03</v>
       </c>
       <c r="G8">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="H8">
-        <v>37.87</v>
+        <v>22.97</v>
       </c>
       <c r="I8">
-        <v>6.7</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -3630,25 +3814,25 @@
         <v>99</v>
       </c>
       <c r="C9">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="D9">
-        <v>48.48</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="F9">
-        <v>51.52</v>
+        <v>64.65000000000001</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>35.35</v>
       </c>
       <c r="I9">
-        <v>9.1</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -3659,16 +3843,16 @@
         <v>176</v>
       </c>
       <c r="C10">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>31.25</v>
+        <v>0</v>
       </c>
       <c r="E10">
-        <v>121</v>
+        <v>176</v>
       </c>
       <c r="F10">
-        <v>68.75</v>
+        <v>100</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -3677,7 +3861,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>8.300000000000001</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -3688,25 +3872,25 @@
         <v>102</v>
       </c>
       <c r="C11">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="D11">
-        <v>27.45</v>
+        <v>0</v>
       </c>
       <c r="E11">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="F11">
-        <v>72.55</v>
+        <v>81.37</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>18.63</v>
       </c>
       <c r="I11">
-        <v>8.300000000000001</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -3717,25 +3901,25 @@
         <v>51</v>
       </c>
       <c r="C12">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D12">
-        <v>39.22</v>
+        <v>0</v>
       </c>
       <c r="E12">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="F12">
-        <v>60.78</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>17.65</v>
       </c>
       <c r="I12">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -3746,25 +3930,25 @@
         <v>159</v>
       </c>
       <c r="C13">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="D13">
-        <v>26.42</v>
+        <v>15.72</v>
       </c>
       <c r="E13">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="F13">
-        <v>69.81</v>
+        <v>67.92</v>
       </c>
       <c r="G13">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="H13">
-        <v>3.77</v>
+        <v>16.35</v>
       </c>
       <c r="I13">
-        <v>8</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -3775,25 +3959,25 @@
         <v>189</v>
       </c>
       <c r="C14">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D14">
-        <v>12.17</v>
+        <v>9.52</v>
       </c>
       <c r="E14">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="F14">
-        <v>77.78</v>
+        <v>83.06999999999999</v>
       </c>
       <c r="G14">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H14">
-        <v>10.05</v>
+        <v>7.41</v>
       </c>
       <c r="I14">
-        <v>8</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -3810,19 +3994,19 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F15">
-        <v>71.88</v>
+        <v>76.04000000000001</v>
       </c>
       <c r="G15">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H15">
-        <v>28.13</v>
+        <v>23.96</v>
       </c>
       <c r="I15">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -3833,16 +4017,16 @@
         <v>211</v>
       </c>
       <c r="C16">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D16">
-        <v>18.96</v>
+        <v>12.8</v>
       </c>
       <c r="E16">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="F16">
-        <v>81.04000000000001</v>
+        <v>87.2</v>
       </c>
       <c r="G16">
         <v>0</v>
@@ -3851,7 +4035,7 @@
         <v>0</v>
       </c>
       <c r="I16">
-        <v>8.300000000000001</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -3862,16 +4046,16 @@
         <v>177</v>
       </c>
       <c r="C17">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="D17">
-        <v>27.68</v>
+        <v>19.21</v>
       </c>
       <c r="E17">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="F17">
-        <v>72.31999999999999</v>
+        <v>80.79000000000001</v>
       </c>
       <c r="G17">
         <v>0</v>
@@ -3880,7 +4064,7 @@
         <v>0</v>
       </c>
       <c r="I17">
-        <v>6.8</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -3891,22 +4075,22 @@
         <v>146</v>
       </c>
       <c r="C18">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="D18">
-        <v>19.18</v>
+        <v>0.68</v>
       </c>
       <c r="E18">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="F18">
-        <v>80.81999999999999</v>
+        <v>83.56</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>15.75</v>
       </c>
       <c r="I18">
         <v>6.8</v>
@@ -3920,25 +4104,25 @@
         <v>228</v>
       </c>
       <c r="C19">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D19">
-        <v>9.210000000000001</v>
+        <v>7.89</v>
       </c>
       <c r="E19">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="F19">
-        <v>71.93000000000001</v>
+        <v>75</v>
       </c>
       <c r="G19">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="H19">
-        <v>18.86</v>
+        <v>17.11</v>
       </c>
       <c r="I19">
-        <v>7.6</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -3978,16 +4162,16 @@
         <v>120</v>
       </c>
       <c r="C21">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D21">
-        <v>35.83</v>
+        <v>35</v>
       </c>
       <c r="E21">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F21">
-        <v>64.17</v>
+        <v>65</v>
       </c>
       <c r="G21">
         <v>0</v>
@@ -3996,7 +4180,7 @@
         <v>0</v>
       </c>
       <c r="I21">
-        <v>8.5</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -4007,22 +4191,22 @@
         <v>211</v>
       </c>
       <c r="C22">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>20.85</v>
+        <v>0</v>
       </c>
       <c r="E22">
-        <v>167</v>
+        <v>195</v>
       </c>
       <c r="F22">
-        <v>79.15000000000001</v>
+        <v>92.42</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>7.58</v>
       </c>
       <c r="I22">
         <v>7.4</v>
@@ -4062,28 +4246,28 @@
         <v>31</v>
       </c>
       <c r="B24">
-        <v>82</v>
+        <v>21</v>
       </c>
       <c r="C24">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="D24">
-        <v>14.63</v>
+        <v>0</v>
       </c>
       <c r="E24">
-        <v>66</v>
+        <v>16</v>
       </c>
       <c r="F24">
-        <v>80.48999999999999</v>
+        <v>76.19</v>
       </c>
       <c r="G24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H24">
-        <v>4.88</v>
+        <v>23.81</v>
       </c>
       <c r="I24">
-        <v>8.6</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -4091,28 +4275,28 @@
         <v>32</v>
       </c>
       <c r="B25">
-        <v>104</v>
+        <v>82</v>
       </c>
       <c r="C25">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D25">
-        <v>0</v>
+        <v>14.63</v>
       </c>
       <c r="E25">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F25">
-        <v>64.42</v>
+        <v>80.48999999999999</v>
       </c>
       <c r="G25">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="H25">
-        <v>35.58</v>
+        <v>4.88</v>
       </c>
       <c r="I25">
-        <v>6.4</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -4120,28 +4304,28 @@
         <v>33</v>
       </c>
       <c r="B26">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C26">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="D26">
-        <v>48.15</v>
+        <v>0</v>
       </c>
       <c r="E26">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="F26">
-        <v>51.85</v>
+        <v>75</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="H26">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I26">
-        <v>8.6</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -4149,28 +4333,28 @@
         <v>34</v>
       </c>
       <c r="B27">
-        <v>71</v>
+        <v>108</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="D27">
-        <v>0</v>
+        <v>39.81</v>
       </c>
       <c r="E27">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="F27">
-        <v>84.51000000000001</v>
+        <v>60.19</v>
       </c>
       <c r="G27">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H27">
-        <v>15.49</v>
+        <v>0</v>
       </c>
       <c r="I27">
-        <v>7.8</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -4178,28 +4362,28 @@
         <v>35</v>
       </c>
       <c r="B28">
-        <v>137</v>
+        <v>71</v>
       </c>
       <c r="C28">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="D28">
-        <v>26.28</v>
+        <v>0</v>
       </c>
       <c r="E28">
-        <v>101</v>
+        <v>58</v>
       </c>
       <c r="F28">
-        <v>73.72</v>
+        <v>81.69</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H28">
-        <v>0</v>
+        <v>18.31</v>
       </c>
       <c r="I28">
-        <v>10</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -4207,19 +4391,19 @@
         <v>36</v>
       </c>
       <c r="B29">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="C29">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D29">
-        <v>22.22</v>
+        <v>10.95</v>
       </c>
       <c r="E29">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F29">
-        <v>77.78</v>
+        <v>89.05</v>
       </c>
       <c r="G29">
         <v>0</v>
@@ -4228,7 +4412,7 @@
         <v>0</v>
       </c>
       <c r="I29">
-        <v>8.1</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -4236,28 +4420,28 @@
         <v>37</v>
       </c>
       <c r="B30">
-        <v>24</v>
+        <v>153</v>
       </c>
       <c r="C30">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>9.15</v>
       </c>
       <c r="E30">
-        <v>24</v>
+        <v>135</v>
       </c>
       <c r="F30">
-        <v>100</v>
+        <v>88.23999999999999</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H30">
-        <v>0</v>
+        <v>2.61</v>
       </c>
       <c r="I30">
-        <v>8.800000000000001</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -4265,28 +4449,28 @@
         <v>38</v>
       </c>
       <c r="B31">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="C31">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="D31">
-        <v>23.15</v>
+        <v>0</v>
       </c>
       <c r="E31">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="F31">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H31">
-        <v>1.85</v>
+        <v>0</v>
       </c>
       <c r="I31">
-        <v>8.1</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -4294,28 +4478,28 @@
         <v>39</v>
       </c>
       <c r="B32">
-        <v>247</v>
+        <v>108</v>
       </c>
       <c r="C32">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="D32">
-        <v>31.17</v>
+        <v>16.67</v>
       </c>
       <c r="E32">
-        <v>170</v>
+        <v>88</v>
       </c>
       <c r="F32">
-        <v>68.83</v>
+        <v>81.48</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H32">
-        <v>0</v>
+        <v>1.85</v>
       </c>
       <c r="I32">
-        <v>7.8</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -4323,28 +4507,28 @@
         <v>40</v>
       </c>
       <c r="B33">
-        <v>222</v>
+        <v>247</v>
       </c>
       <c r="C33">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="D33">
-        <v>21.62</v>
+        <v>0.4</v>
       </c>
       <c r="E33">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="F33">
-        <v>78.38</v>
+        <v>73.68000000000001</v>
       </c>
       <c r="G33">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="H33">
-        <v>0</v>
+        <v>25.91</v>
       </c>
       <c r="I33">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -4355,25 +4539,25 @@
         <v>222</v>
       </c>
       <c r="C34">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="D34">
-        <v>10.36</v>
+        <v>0.9</v>
       </c>
       <c r="E34">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="F34">
-        <v>85.59</v>
+        <v>83.78</v>
       </c>
       <c r="G34">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="H34">
-        <v>4.05</v>
+        <v>15.32</v>
       </c>
       <c r="I34">
-        <v>8.199999999999999</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -4381,28 +4565,28 @@
         <v>42</v>
       </c>
       <c r="B35">
-        <v>162</v>
+        <v>222</v>
       </c>
       <c r="C35">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="D35">
-        <v>25.31</v>
+        <v>3.15</v>
       </c>
       <c r="E35">
-        <v>75</v>
+        <v>189</v>
       </c>
       <c r="F35">
-        <v>46.3</v>
+        <v>85.14</v>
       </c>
       <c r="G35">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="H35">
-        <v>28.4</v>
+        <v>11.71</v>
       </c>
       <c r="I35">
-        <v>6.6</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -4410,28 +4594,28 @@
         <v>43</v>
       </c>
       <c r="B36">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="C36">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D36">
-        <v>26.39</v>
+        <v>25.31</v>
       </c>
       <c r="E36">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="F36">
-        <v>70.14</v>
+        <v>46.3</v>
       </c>
       <c r="G36">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="H36">
-        <v>3.47</v>
+        <v>28.4</v>
       </c>
       <c r="I36">
-        <v>7.6</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -4439,7 +4623,7 @@
         <v>44</v>
       </c>
       <c r="B37">
-        <v>65</v>
+        <v>144</v>
       </c>
       <c r="C37">
         <v>0</v>
@@ -4448,19 +4632,19 @@
         <v>0</v>
       </c>
       <c r="E37">
-        <v>65</v>
+        <v>113</v>
       </c>
       <c r="F37">
-        <v>100</v>
+        <v>78.47</v>
       </c>
       <c r="G37">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>21.53</v>
       </c>
       <c r="I37">
-        <v>8.1</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -4468,19 +4652,19 @@
         <v>45</v>
       </c>
       <c r="B38">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C38">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="D38">
-        <v>24.66</v>
+        <v>0</v>
       </c>
       <c r="E38">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="F38">
-        <v>75.34</v>
+        <v>100</v>
       </c>
       <c r="G38">
         <v>0</v>
@@ -4489,7 +4673,7 @@
         <v>0</v>
       </c>
       <c r="I38">
-        <v>6.7</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -4497,28 +4681,28 @@
         <v>46</v>
       </c>
       <c r="B39">
-        <v>143</v>
+        <v>73</v>
       </c>
       <c r="C39">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="D39">
-        <v>47.55</v>
+        <v>0</v>
       </c>
       <c r="E39">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="F39">
-        <v>52.45</v>
+        <v>86.3</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H39">
-        <v>0</v>
+        <v>13.7</v>
       </c>
       <c r="I39">
-        <v>7.4</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -4526,28 +4710,28 @@
         <v>47</v>
       </c>
       <c r="B40">
-        <v>203</v>
+        <v>143</v>
       </c>
       <c r="C40">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D40">
-        <v>0.99</v>
+        <v>0</v>
       </c>
       <c r="E40">
-        <v>167</v>
+        <v>96</v>
       </c>
       <c r="F40">
-        <v>82.27</v>
+        <v>67.13</v>
       </c>
       <c r="G40">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="H40">
-        <v>16.75</v>
+        <v>32.87</v>
       </c>
       <c r="I40">
-        <v>7.1</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -4555,28 +4739,28 @@
         <v>48</v>
       </c>
       <c r="B41">
-        <v>72</v>
+        <v>203</v>
       </c>
       <c r="C41">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="D41">
-        <v>31.94</v>
+        <v>0.99</v>
       </c>
       <c r="E41">
-        <v>49</v>
+        <v>167</v>
       </c>
       <c r="F41">
-        <v>68.06</v>
+        <v>82.27</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="H41">
-        <v>0</v>
+        <v>16.75</v>
       </c>
       <c r="I41">
-        <v>7.5</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -4584,28 +4768,28 @@
         <v>49</v>
       </c>
       <c r="B42">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="C42">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="D42">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E42">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="F42">
-        <v>70</v>
+        <v>81.94</v>
       </c>
       <c r="G42">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H42">
-        <v>0</v>
+        <v>18.06</v>
       </c>
       <c r="I42">
-        <v>8.300000000000001</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -4613,25 +4797,25 @@
         <v>50</v>
       </c>
       <c r="B43">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C43">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D43">
-        <v>42.42</v>
+        <v>0</v>
       </c>
       <c r="E43">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F43">
-        <v>57.58</v>
+        <v>75</v>
       </c>
       <c r="G43">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H43">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I43">
         <v>7.4</v>
@@ -4642,19 +4826,19 @@
         <v>51</v>
       </c>
       <c r="B44">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="C44">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D44">
-        <v>28.81</v>
+        <v>42.42</v>
       </c>
       <c r="E44">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="F44">
-        <v>71.19</v>
+        <v>57.58</v>
       </c>
       <c r="G44">
         <v>0</v>
@@ -4663,7 +4847,7 @@
         <v>0</v>
       </c>
       <c r="I44">
-        <v>8.800000000000001</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -4671,28 +4855,28 @@
         <v>52</v>
       </c>
       <c r="B45">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="C45">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D45">
-        <v>2.78</v>
+        <v>0</v>
       </c>
       <c r="E45">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="F45">
-        <v>50</v>
+        <v>84.75</v>
       </c>
       <c r="G45">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="H45">
-        <v>47.22</v>
+        <v>15.25</v>
       </c>
       <c r="I45">
-        <v>6.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -4700,28 +4884,28 @@
         <v>53</v>
       </c>
       <c r="B46">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="C46">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="D46">
-        <v>40.22</v>
+        <v>2.78</v>
       </c>
       <c r="E46">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="F46">
-        <v>59.78</v>
+        <v>50</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="H46">
-        <v>0</v>
+        <v>47.22</v>
       </c>
       <c r="I46">
-        <v>8.5</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -4729,28 +4913,28 @@
         <v>54</v>
       </c>
       <c r="B47">
-        <v>158</v>
+        <v>92</v>
       </c>
       <c r="C47">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D47">
-        <v>1.27</v>
+        <v>16.3</v>
       </c>
       <c r="E47">
-        <v>108</v>
+        <v>77</v>
       </c>
       <c r="F47">
-        <v>68.34999999999999</v>
+        <v>83.7</v>
       </c>
       <c r="G47">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="H47">
-        <v>30.38</v>
+        <v>0</v>
       </c>
       <c r="I47">
-        <v>7.1</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -4758,28 +4942,28 @@
         <v>55</v>
       </c>
       <c r="B48">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="C48">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="D48">
-        <v>31.76</v>
+        <v>1.27</v>
       </c>
       <c r="E48">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="F48">
-        <v>67.56999999999999</v>
+        <v>68.34999999999999</v>
       </c>
       <c r="G48">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="H48">
-        <v>0.68</v>
+        <v>30.38</v>
       </c>
       <c r="I48">
-        <v>6.8</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -4787,28 +4971,28 @@
         <v>56</v>
       </c>
       <c r="B49">
-        <v>90</v>
+        <v>148</v>
       </c>
       <c r="C49">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D49">
-        <v>44.44</v>
+        <v>20.95</v>
       </c>
       <c r="E49">
-        <v>50</v>
+        <v>116</v>
       </c>
       <c r="F49">
-        <v>55.56</v>
+        <v>78.38</v>
       </c>
       <c r="G49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H49">
-        <v>0</v>
+        <v>0.68</v>
       </c>
       <c r="I49">
-        <v>8.6</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -4816,7 +5000,7 @@
         <v>57</v>
       </c>
       <c r="B50">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="C50">
         <v>0</v>
@@ -4825,19 +5009,19 @@
         <v>0</v>
       </c>
       <c r="E50">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="F50">
-        <v>87.5</v>
+        <v>77.78</v>
       </c>
       <c r="G50">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="H50">
-        <v>12.5</v>
+        <v>22.22</v>
       </c>
       <c r="I50">
-        <v>8.800000000000001</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -4845,28 +5029,57 @@
         <v>58</v>
       </c>
       <c r="B51">
+        <v>104</v>
+      </c>
+      <c r="C51">
+        <v>0</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51">
+        <v>92</v>
+      </c>
+      <c r="F51">
+        <v>88.45999999999999</v>
+      </c>
+      <c r="G51">
+        <v>12</v>
+      </c>
+      <c r="H51">
+        <v>11.54</v>
+      </c>
+      <c r="I51">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52">
         <v>108</v>
       </c>
-      <c r="C51">
-        <v>2</v>
-      </c>
-      <c r="D51">
-        <v>1.85</v>
-      </c>
-      <c r="E51">
-        <v>88</v>
-      </c>
-      <c r="F51">
-        <v>81.48</v>
-      </c>
-      <c r="G51">
-        <v>18</v>
-      </c>
-      <c r="H51">
-        <v>16.67</v>
-      </c>
-      <c r="I51">
-        <v>7.7</v>
+      <c r="C52">
+        <v>0</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52">
+        <v>83</v>
+      </c>
+      <c r="F52">
+        <v>76.84999999999999</v>
+      </c>
+      <c r="G52">
+        <v>25</v>
+      </c>
+      <c r="H52">
+        <v>23.15</v>
+      </c>
+      <c r="I52">
+        <v>7.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion 10 Mar Mañana
</commit_message>
<xml_diff>
--- a/Totales Docentes.xlsx
+++ b/Totales Docentes.xlsx
@@ -596,16 +596,16 @@
         <v>90</v>
       </c>
       <c r="C2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D2">
-        <v>21.11</v>
+        <v>20</v>
       </c>
       <c r="E2">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F2">
-        <v>78.89</v>
+        <v>80</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -683,22 +683,25 @@
         <v>123</v>
       </c>
       <c r="C5">
-        <v>123</v>
+        <v>27</v>
       </c>
       <c r="D5">
-        <v>100</v>
+        <v>21.95</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>73.98</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>4.07</v>
+      </c>
+      <c r="I5">
+        <v>7.7</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -738,25 +741,25 @@
         <v>95</v>
       </c>
       <c r="C7">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="D7">
-        <v>41.05</v>
+        <v>2.11</v>
       </c>
       <c r="E7">
-        <v>56</v>
+        <v>90</v>
       </c>
       <c r="F7">
-        <v>58.95</v>
+        <v>94.73999999999999</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>3.16</v>
       </c>
       <c r="I7">
-        <v>8.699999999999999</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -851,22 +854,22 @@
         <v>147</v>
       </c>
       <c r="C11">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="D11">
-        <v>35.37</v>
+        <v>15.65</v>
       </c>
       <c r="E11">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="F11">
-        <v>51.02</v>
+        <v>63.95</v>
       </c>
       <c r="G11">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H11">
-        <v>13.61</v>
+        <v>20.41</v>
       </c>
       <c r="I11">
         <v>7.4</v>
@@ -880,22 +883,25 @@
         <v>176</v>
       </c>
       <c r="C12">
-        <v>176</v>
+        <v>110</v>
       </c>
       <c r="D12">
-        <v>100</v>
+        <v>62.5</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>37.5</v>
       </c>
       <c r="G12">
         <v>0</v>
       </c>
       <c r="H12">
         <v>0</v>
+      </c>
+      <c r="I12">
+        <v>7.4</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -906,22 +912,25 @@
         <v>187</v>
       </c>
       <c r="C13">
-        <v>187</v>
+        <v>2</v>
       </c>
       <c r="D13">
-        <v>100</v>
+        <v>1.07</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>185</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>98.93000000000001</v>
       </c>
       <c r="G13">
         <v>0</v>
       </c>
       <c r="H13">
         <v>0</v>
+      </c>
+      <c r="I13">
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -932,22 +941,25 @@
         <v>69</v>
       </c>
       <c r="C14">
-        <v>69</v>
+        <v>13</v>
       </c>
       <c r="D14">
-        <v>100</v>
+        <v>18.84</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>81.16</v>
       </c>
       <c r="G14">
         <v>0</v>
       </c>
       <c r="H14">
         <v>0</v>
+      </c>
+      <c r="I14">
+        <v>7.6</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -1045,22 +1057,25 @@
         <v>262</v>
       </c>
       <c r="C18">
-        <v>262</v>
+        <v>61</v>
       </c>
       <c r="D18">
-        <v>100</v>
+        <v>23.28</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>3.82</v>
+      </c>
+      <c r="I18">
+        <v>7.5</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -1071,16 +1086,16 @@
         <v>146</v>
       </c>
       <c r="C19">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D19">
-        <v>78.77</v>
+        <v>78.08</v>
       </c>
       <c r="E19">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F19">
-        <v>20.55</v>
+        <v>21.23</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -1089,7 +1104,7 @@
         <v>0.68</v>
       </c>
       <c r="I19">
-        <v>8.4</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1184,16 +1199,16 @@
         <v>171</v>
       </c>
       <c r="C23">
-        <v>151</v>
+        <v>21</v>
       </c>
       <c r="D23">
-        <v>88.3</v>
+        <v>12.28</v>
       </c>
       <c r="E23">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="F23">
-        <v>11.7</v>
+        <v>87.72</v>
       </c>
       <c r="G23">
         <v>0</v>
@@ -1202,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="I23">
-        <v>9.800000000000001</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1242,22 +1257,25 @@
         <v>31</v>
       </c>
       <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
         <v>31</v>
       </c>
-      <c r="D25">
-        <v>100</v>
-      </c>
-      <c r="E25">
-        <v>0</v>
-      </c>
       <c r="F25">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G25">
         <v>0</v>
       </c>
       <c r="H25">
         <v>0</v>
+      </c>
+      <c r="I25">
+        <v>8.6</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -1297,22 +1315,25 @@
         <v>139</v>
       </c>
       <c r="C27">
-        <v>139</v>
+        <v>0</v>
       </c>
       <c r="D27">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>84.89</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H27">
-        <v>0</v>
+        <v>15.11</v>
+      </c>
+      <c r="I27">
+        <v>6.4</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1381,22 +1402,25 @@
         <v>110</v>
       </c>
       <c r="C30">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="D30">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H30">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="I30">
+        <v>7.8</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -1436,10 +1460,10 @@
         <v>64</v>
       </c>
       <c r="C32">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D32">
-        <v>7.81</v>
+        <v>0</v>
       </c>
       <c r="E32">
         <v>59</v>
@@ -1448,13 +1472,13 @@
         <v>92.19</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H32">
-        <v>0</v>
+        <v>7.81</v>
       </c>
       <c r="I32">
-        <v>9.699999999999999</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -1465,22 +1489,25 @@
         <v>112</v>
       </c>
       <c r="C33">
-        <v>112</v>
+        <v>18</v>
       </c>
       <c r="D33">
-        <v>100</v>
+        <v>16.07</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>83.93000000000001</v>
       </c>
       <c r="G33">
         <v>0</v>
       </c>
       <c r="H33">
         <v>0</v>
+      </c>
+      <c r="I33">
+        <v>8.1</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -1491,25 +1518,25 @@
         <v>183</v>
       </c>
       <c r="C34">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="D34">
-        <v>37.16</v>
+        <v>0</v>
       </c>
       <c r="E34">
-        <v>86</v>
+        <v>142</v>
       </c>
       <c r="F34">
-        <v>46.99</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="G34">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="H34">
-        <v>15.85</v>
+        <v>22.4</v>
       </c>
       <c r="I34">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -1549,16 +1576,16 @@
         <v>217</v>
       </c>
       <c r="C36">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D36">
-        <v>8.289999999999999</v>
+        <v>5.07</v>
       </c>
       <c r="E36">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="F36">
-        <v>90.31999999999999</v>
+        <v>93.55</v>
       </c>
       <c r="G36">
         <v>3</v>
@@ -1578,16 +1605,16 @@
         <v>100</v>
       </c>
       <c r="C37">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="D37">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="E37">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="F37">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="G37">
         <v>0</v>
@@ -1596,7 +1623,7 @@
         <v>0</v>
       </c>
       <c r="I37">
-        <v>7</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -1607,22 +1634,25 @@
         <v>133</v>
       </c>
       <c r="C38">
-        <v>133</v>
+        <v>48</v>
       </c>
       <c r="D38">
-        <v>100</v>
+        <v>36.09</v>
       </c>
       <c r="E38">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="F38">
-        <v>0</v>
+        <v>63.91</v>
       </c>
       <c r="G38">
         <v>0</v>
       </c>
       <c r="H38">
         <v>0</v>
+      </c>
+      <c r="I38">
+        <v>7.8</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -1633,22 +1663,25 @@
         <v>101</v>
       </c>
       <c r="C39">
-        <v>101</v>
+        <v>2</v>
       </c>
       <c r="D39">
-        <v>100</v>
+        <v>1.98</v>
       </c>
       <c r="E39">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="F39">
-        <v>0</v>
+        <v>98.02</v>
       </c>
       <c r="G39">
         <v>0</v>
       </c>
       <c r="H39">
         <v>0</v>
+      </c>
+      <c r="I39">
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -1688,22 +1721,25 @@
         <v>101</v>
       </c>
       <c r="C41">
-        <v>101</v>
+        <v>0</v>
       </c>
       <c r="D41">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E41">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="F41">
-        <v>0</v>
+        <v>87.13</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H41">
-        <v>0</v>
+        <v>12.87</v>
+      </c>
+      <c r="I41">
+        <v>5.9</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -1769,22 +1805,25 @@
         <v>69</v>
       </c>
       <c r="C44">
-        <v>69</v>
+        <v>5</v>
       </c>
       <c r="D44">
-        <v>100</v>
+        <v>7.25</v>
       </c>
       <c r="E44">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="F44">
-        <v>0</v>
+        <v>69.56999999999999</v>
       </c>
       <c r="G44">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="H44">
-        <v>0</v>
+        <v>23.19</v>
+      </c>
+      <c r="I44">
+        <v>6.8</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -1824,22 +1863,25 @@
         <v>97</v>
       </c>
       <c r="C46">
-        <v>97</v>
+        <v>2</v>
       </c>
       <c r="D46">
-        <v>100</v>
+        <v>2.06</v>
       </c>
       <c r="E46">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="F46">
-        <v>0</v>
+        <v>73.2</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="H46">
-        <v>0</v>
+        <v>24.74</v>
+      </c>
+      <c r="I46">
+        <v>7.4</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -1902,22 +1944,25 @@
         <v>114</v>
       </c>
       <c r="C49">
-        <v>114</v>
+        <v>19</v>
       </c>
       <c r="D49">
-        <v>100</v>
+        <v>16.67</v>
       </c>
       <c r="E49">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F49">
-        <v>0</v>
+        <v>78.95</v>
       </c>
       <c r="G49">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H49">
-        <v>0</v>
+        <v>4.39</v>
+      </c>
+      <c r="I49">
+        <v>6.5</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -2069,10 +2114,10 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H2">
-        <v>78.89</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2147,10 +2192,10 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>78.05</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2199,10 +2244,10 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="H7">
-        <v>58.95</v>
+        <v>97.89</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2303,10 +2348,10 @@
         <v>0</v>
       </c>
       <c r="G11">
-        <v>95</v>
+        <v>124</v>
       </c>
       <c r="H11">
-        <v>64.63</v>
+        <v>84.34999999999999</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -2329,10 +2374,10 @@
         <v>0</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -2355,10 +2400,10 @@
         <v>0</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>185</v>
       </c>
       <c r="H13">
-        <v>0</v>
+        <v>98.93000000000001</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -2381,10 +2426,10 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>81.16</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -2485,10 +2530,10 @@
         <v>0</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>201</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>76.72</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -2511,10 +2556,10 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H19">
-        <v>21.23</v>
+        <v>21.92</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -2615,10 +2660,10 @@
         <v>0</v>
       </c>
       <c r="G23">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="H23">
-        <v>11.7</v>
+        <v>87.72</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -2667,10 +2712,10 @@
         <v>0</v>
       </c>
       <c r="G25">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="H25">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -2719,10 +2764,10 @@
         <v>0</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>139</v>
       </c>
       <c r="H27">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -2797,10 +2842,10 @@
         <v>0</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="H30">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -2849,10 +2894,10 @@
         <v>0</v>
       </c>
       <c r="G32">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="H32">
-        <v>92.19</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -2875,10 +2920,10 @@
         <v>0</v>
       </c>
       <c r="G33">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="H33">
-        <v>0</v>
+        <v>83.93000000000001</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -2901,10 +2946,10 @@
         <v>0</v>
       </c>
       <c r="G34">
-        <v>115</v>
+        <v>183</v>
       </c>
       <c r="H34">
-        <v>62.84</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -2953,10 +2998,10 @@
         <v>0</v>
       </c>
       <c r="G36">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="H36">
-        <v>91.70999999999999</v>
+        <v>94.93000000000001</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -2979,10 +3024,10 @@
         <v>0</v>
       </c>
       <c r="G37">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="H37">
-        <v>7</v>
+        <v>27</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -3005,10 +3050,10 @@
         <v>0</v>
       </c>
       <c r="G38">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="H38">
-        <v>0</v>
+        <v>63.91</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -3031,10 +3076,10 @@
         <v>0</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="H39">
-        <v>0</v>
+        <v>98.02</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -3083,10 +3128,10 @@
         <v>0</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="H41">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -3161,10 +3206,10 @@
         <v>0</v>
       </c>
       <c r="G44">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="H44">
-        <v>0</v>
+        <v>92.75</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -3213,10 +3258,10 @@
         <v>0</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H46">
-        <v>0</v>
+        <v>97.94</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -3291,10 +3336,10 @@
         <v>0</v>
       </c>
       <c r="G49">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H49">
-        <v>0</v>
+        <v>83.33</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -3425,16 +3470,16 @@
         <v>90</v>
       </c>
       <c r="C2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D2">
-        <v>21.11</v>
+        <v>20</v>
       </c>
       <c r="E2">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F2">
-        <v>78.89</v>
+        <v>80</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -3512,22 +3557,25 @@
         <v>123</v>
       </c>
       <c r="C5">
-        <v>123</v>
+        <v>27</v>
       </c>
       <c r="D5">
-        <v>100</v>
+        <v>21.95</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>73.98</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>4.07</v>
+      </c>
+      <c r="I5">
+        <v>7.7</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -3567,25 +3615,25 @@
         <v>95</v>
       </c>
       <c r="C7">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="D7">
-        <v>41.05</v>
+        <v>2.11</v>
       </c>
       <c r="E7">
-        <v>56</v>
+        <v>90</v>
       </c>
       <c r="F7">
-        <v>58.95</v>
+        <v>94.73999999999999</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>3.16</v>
       </c>
       <c r="I7">
-        <v>8.699999999999999</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -3680,22 +3728,22 @@
         <v>147</v>
       </c>
       <c r="C11">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="D11">
-        <v>35.37</v>
+        <v>15.65</v>
       </c>
       <c r="E11">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="F11">
-        <v>51.02</v>
+        <v>63.95</v>
       </c>
       <c r="G11">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H11">
-        <v>13.61</v>
+        <v>20.41</v>
       </c>
       <c r="I11">
         <v>7.4</v>
@@ -3709,22 +3757,25 @@
         <v>176</v>
       </c>
       <c r="C12">
-        <v>176</v>
+        <v>110</v>
       </c>
       <c r="D12">
-        <v>100</v>
+        <v>62.5</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>37.5</v>
       </c>
       <c r="G12">
         <v>0</v>
       </c>
       <c r="H12">
         <v>0</v>
+      </c>
+      <c r="I12">
+        <v>7.4</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -3735,22 +3786,25 @@
         <v>187</v>
       </c>
       <c r="C13">
-        <v>187</v>
+        <v>2</v>
       </c>
       <c r="D13">
-        <v>100</v>
+        <v>1.07</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>185</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>98.93000000000001</v>
       </c>
       <c r="G13">
         <v>0</v>
       </c>
       <c r="H13">
         <v>0</v>
+      </c>
+      <c r="I13">
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -3761,22 +3815,25 @@
         <v>69</v>
       </c>
       <c r="C14">
-        <v>69</v>
+        <v>13</v>
       </c>
       <c r="D14">
-        <v>100</v>
+        <v>18.84</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>81.16</v>
       </c>
       <c r="G14">
         <v>0</v>
       </c>
       <c r="H14">
         <v>0</v>
+      </c>
+      <c r="I14">
+        <v>7.6</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -3874,22 +3931,25 @@
         <v>262</v>
       </c>
       <c r="C18">
-        <v>262</v>
+        <v>61</v>
       </c>
       <c r="D18">
-        <v>100</v>
+        <v>23.28</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>3.82</v>
+      </c>
+      <c r="I18">
+        <v>7.5</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -3900,16 +3960,16 @@
         <v>146</v>
       </c>
       <c r="C19">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D19">
-        <v>78.77</v>
+        <v>78.08</v>
       </c>
       <c r="E19">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F19">
-        <v>20.55</v>
+        <v>21.23</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -3918,7 +3978,7 @@
         <v>0.68</v>
       </c>
       <c r="I19">
-        <v>8.4</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -4013,16 +4073,16 @@
         <v>171</v>
       </c>
       <c r="C23">
-        <v>151</v>
+        <v>21</v>
       </c>
       <c r="D23">
-        <v>88.3</v>
+        <v>12.28</v>
       </c>
       <c r="E23">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="F23">
-        <v>11.7</v>
+        <v>87.72</v>
       </c>
       <c r="G23">
         <v>0</v>
@@ -4031,7 +4091,7 @@
         <v>0</v>
       </c>
       <c r="I23">
-        <v>9.800000000000001</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -4071,22 +4131,25 @@
         <v>31</v>
       </c>
       <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
         <v>31</v>
       </c>
-      <c r="D25">
-        <v>100</v>
-      </c>
-      <c r="E25">
-        <v>0</v>
-      </c>
       <c r="F25">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G25">
         <v>0</v>
       </c>
       <c r="H25">
         <v>0</v>
+      </c>
+      <c r="I25">
+        <v>8.6</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -4126,22 +4189,25 @@
         <v>139</v>
       </c>
       <c r="C27">
-        <v>139</v>
+        <v>0</v>
       </c>
       <c r="D27">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>84.89</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H27">
-        <v>0</v>
+        <v>15.11</v>
+      </c>
+      <c r="I27">
+        <v>6.4</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -4210,22 +4276,25 @@
         <v>110</v>
       </c>
       <c r="C30">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="D30">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H30">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="I30">
+        <v>7.8</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -4265,10 +4334,10 @@
         <v>64</v>
       </c>
       <c r="C32">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D32">
-        <v>7.81</v>
+        <v>0</v>
       </c>
       <c r="E32">
         <v>59</v>
@@ -4277,13 +4346,13 @@
         <v>92.19</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H32">
-        <v>0</v>
+        <v>7.81</v>
       </c>
       <c r="I32">
-        <v>9.699999999999999</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -4294,22 +4363,25 @@
         <v>112</v>
       </c>
       <c r="C33">
-        <v>112</v>
+        <v>18</v>
       </c>
       <c r="D33">
-        <v>100</v>
+        <v>16.07</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>83.93000000000001</v>
       </c>
       <c r="G33">
         <v>0</v>
       </c>
       <c r="H33">
         <v>0</v>
+      </c>
+      <c r="I33">
+        <v>8.1</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -4320,25 +4392,25 @@
         <v>183</v>
       </c>
       <c r="C34">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="D34">
-        <v>37.16</v>
+        <v>0</v>
       </c>
       <c r="E34">
-        <v>86</v>
+        <v>142</v>
       </c>
       <c r="F34">
-        <v>46.99</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="G34">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="H34">
-        <v>15.85</v>
+        <v>22.4</v>
       </c>
       <c r="I34">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -4378,16 +4450,16 @@
         <v>217</v>
       </c>
       <c r="C36">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D36">
-        <v>8.289999999999999</v>
+        <v>5.07</v>
       </c>
       <c r="E36">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="F36">
-        <v>90.31999999999999</v>
+        <v>93.55</v>
       </c>
       <c r="G36">
         <v>3</v>
@@ -4407,16 +4479,16 @@
         <v>100</v>
       </c>
       <c r="C37">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="D37">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="E37">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="F37">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="G37">
         <v>0</v>
@@ -4425,7 +4497,7 @@
         <v>0</v>
       </c>
       <c r="I37">
-        <v>7</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -4436,22 +4508,25 @@
         <v>133</v>
       </c>
       <c r="C38">
-        <v>133</v>
+        <v>48</v>
       </c>
       <c r="D38">
-        <v>100</v>
+        <v>36.09</v>
       </c>
       <c r="E38">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="F38">
-        <v>0</v>
+        <v>63.91</v>
       </c>
       <c r="G38">
         <v>0</v>
       </c>
       <c r="H38">
         <v>0</v>
+      </c>
+      <c r="I38">
+        <v>7.8</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -4462,22 +4537,25 @@
         <v>101</v>
       </c>
       <c r="C39">
-        <v>101</v>
+        <v>2</v>
       </c>
       <c r="D39">
-        <v>100</v>
+        <v>1.98</v>
       </c>
       <c r="E39">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="F39">
-        <v>0</v>
+        <v>98.02</v>
       </c>
       <c r="G39">
         <v>0</v>
       </c>
       <c r="H39">
         <v>0</v>
+      </c>
+      <c r="I39">
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -4517,22 +4595,25 @@
         <v>101</v>
       </c>
       <c r="C41">
-        <v>101</v>
+        <v>0</v>
       </c>
       <c r="D41">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E41">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="F41">
-        <v>0</v>
+        <v>87.13</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H41">
-        <v>0</v>
+        <v>12.87</v>
+      </c>
+      <c r="I41">
+        <v>5.9</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -4598,22 +4679,25 @@
         <v>69</v>
       </c>
       <c r="C44">
-        <v>69</v>
+        <v>5</v>
       </c>
       <c r="D44">
-        <v>100</v>
+        <v>7.25</v>
       </c>
       <c r="E44">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="F44">
-        <v>0</v>
+        <v>69.56999999999999</v>
       </c>
       <c r="G44">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="H44">
-        <v>0</v>
+        <v>23.19</v>
+      </c>
+      <c r="I44">
+        <v>6.8</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -4653,22 +4737,25 @@
         <v>97</v>
       </c>
       <c r="C46">
-        <v>97</v>
+        <v>2</v>
       </c>
       <c r="D46">
-        <v>100</v>
+        <v>2.06</v>
       </c>
       <c r="E46">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="F46">
-        <v>0</v>
+        <v>73.2</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="H46">
-        <v>0</v>
+        <v>24.74</v>
+      </c>
+      <c r="I46">
+        <v>7.4</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -4731,22 +4818,25 @@
         <v>114</v>
       </c>
       <c r="C49">
-        <v>114</v>
+        <v>19</v>
       </c>
       <c r="D49">
-        <v>100</v>
+        <v>16.67</v>
       </c>
       <c r="E49">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F49">
-        <v>0</v>
+        <v>78.95</v>
       </c>
       <c r="G49">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H49">
-        <v>0</v>
+        <v>4.39</v>
+      </c>
+      <c r="I49">
+        <v>6.5</v>
       </c>
     </row>
     <row r="50" spans="1:9">

</xml_diff>

<commit_message>
Segundo Parcial 11 Mayo
</commit_message>
<xml_diff>
--- a/Totales Docentes.xlsx
+++ b/Totales Docentes.xlsx
@@ -596,16 +596,16 @@
         <v>90</v>
       </c>
       <c r="C2">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>17.78</v>
+        <v>6.67</v>
       </c>
       <c r="E2">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="F2">
-        <v>82.22</v>
+        <v>93.33</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -614,7 +614,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>9.1</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -625,16 +625,16 @@
         <v>133</v>
       </c>
       <c r="C3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>9.77</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="F3">
-        <v>90.23</v>
+        <v>100</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -643,7 +643,7 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>9.5</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -651,7 +651,7 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -660,16 +660,16 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F4">
-        <v>74.73999999999999</v>
+        <v>74.61</v>
       </c>
       <c r="G4">
         <v>49</v>
       </c>
       <c r="H4">
-        <v>25.26</v>
+        <v>25.39</v>
       </c>
       <c r="I4">
         <v>7.5</v>
@@ -680,28 +680,28 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C5">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>21.95</v>
+        <v>0</v>
       </c>
       <c r="E5">
         <v>91</v>
       </c>
       <c r="F5">
-        <v>73.98</v>
+        <v>74.59</v>
       </c>
       <c r="G5">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="H5">
-        <v>4.07</v>
+        <v>25.41</v>
       </c>
       <c r="I5">
-        <v>7.7</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -741,16 +741,16 @@
         <v>95</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>2.11</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F7">
-        <v>94.73999999999999</v>
+        <v>96.84</v>
       </c>
       <c r="G7">
         <v>3</v>
@@ -828,16 +828,16 @@
         <v>82</v>
       </c>
       <c r="C10">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="D10">
-        <v>30.49</v>
+        <v>12.2</v>
       </c>
       <c r="E10">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="F10">
-        <v>69.51000000000001</v>
+        <v>87.8</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -846,7 +846,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>7.5</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -857,16 +857,16 @@
         <v>147</v>
       </c>
       <c r="C11">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D11">
-        <v>15.65</v>
+        <v>14.29</v>
       </c>
       <c r="E11">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F11">
-        <v>63.95</v>
+        <v>65.31</v>
       </c>
       <c r="G11">
         <v>30</v>
@@ -875,7 +875,7 @@
         <v>20.41</v>
       </c>
       <c r="I11">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -886,25 +886,25 @@
         <v>176</v>
       </c>
       <c r="C12">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="D12">
-        <v>24.43</v>
+        <v>0</v>
       </c>
       <c r="E12">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="F12">
-        <v>75.56999999999999</v>
+        <v>85.23</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>14.77</v>
       </c>
       <c r="I12">
-        <v>6.7</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -912,19 +912,19 @@
         <v>20</v>
       </c>
       <c r="B13">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13">
-        <v>1.07</v>
+        <v>0.54</v>
       </c>
       <c r="E13">
         <v>185</v>
       </c>
       <c r="F13">
-        <v>98.93000000000001</v>
+        <v>99.45999999999999</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -941,19 +941,19 @@
         <v>21</v>
       </c>
       <c r="B14">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C14">
         <v>13</v>
       </c>
       <c r="D14">
-        <v>18.84</v>
+        <v>18.57</v>
       </c>
       <c r="E14">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F14">
-        <v>81.16</v>
+        <v>81.43000000000001</v>
       </c>
       <c r="G14">
         <v>0</v>
@@ -1031,16 +1031,16 @@
         <v>83</v>
       </c>
       <c r="C17">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="D17">
-        <v>22.89</v>
+        <v>8.43</v>
       </c>
       <c r="E17">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="F17">
-        <v>77.11</v>
+        <v>91.56999999999999</v>
       </c>
       <c r="G17">
         <v>0</v>
@@ -1049,7 +1049,7 @@
         <v>0</v>
       </c>
       <c r="I17">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1086,28 +1086,28 @@
         <v>26</v>
       </c>
       <c r="B19">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C19">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D19">
-        <v>14.38</v>
+        <v>10.88</v>
       </c>
       <c r="E19">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="F19">
-        <v>75.34</v>
+        <v>78.91</v>
       </c>
       <c r="G19">
         <v>15</v>
       </c>
       <c r="H19">
-        <v>10.27</v>
+        <v>10.2</v>
       </c>
       <c r="I19">
-        <v>8</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1115,19 +1115,19 @@
         <v>27</v>
       </c>
       <c r="B20">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C20">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D20">
-        <v>38.38</v>
+        <v>38.07</v>
       </c>
       <c r="E20">
         <v>122</v>
       </c>
       <c r="F20">
-        <v>61.62</v>
+        <v>61.93</v>
       </c>
       <c r="G20">
         <v>0</v>
@@ -1231,28 +1231,28 @@
         <v>31</v>
       </c>
       <c r="B24">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C24">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D24">
-        <v>9.380000000000001</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="E24">
         <v>116</v>
       </c>
       <c r="F24">
-        <v>90.63</v>
+        <v>89.92</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>1.55</v>
       </c>
       <c r="I24">
-        <v>8.199999999999999</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1292,25 +1292,25 @@
         <v>55</v>
       </c>
       <c r="C26">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D26">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E26">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="F26">
-        <v>60</v>
+        <v>74.55</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="H26">
-        <v>0</v>
+        <v>25.45</v>
       </c>
       <c r="I26">
-        <v>7.6</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1350,16 +1350,16 @@
         <v>114</v>
       </c>
       <c r="C28">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D28">
-        <v>71.05</v>
+        <v>68.42</v>
       </c>
       <c r="E28">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F28">
-        <v>28.95</v>
+        <v>31.58</v>
       </c>
       <c r="G28">
         <v>0</v>
@@ -1368,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="I28">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1437,16 +1437,16 @@
         <v>152</v>
       </c>
       <c r="C31">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D31">
-        <v>4.61</v>
+        <v>2.63</v>
       </c>
       <c r="E31">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="F31">
-        <v>95.39</v>
+        <v>97.37</v>
       </c>
       <c r="G31">
         <v>0</v>
@@ -1492,25 +1492,25 @@
         <v>40</v>
       </c>
       <c r="B33">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C33">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D33">
-        <v>16.07</v>
+        <v>14.16</v>
       </c>
       <c r="E33">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F33">
-        <v>83.93000000000001</v>
+        <v>84.95999999999999</v>
       </c>
       <c r="G33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H33">
-        <v>0</v>
+        <v>0.88</v>
       </c>
       <c r="I33">
         <v>8.1</v>
@@ -1521,7 +1521,7 @@
         <v>41</v>
       </c>
       <c r="B34">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -1530,19 +1530,19 @@
         <v>0</v>
       </c>
       <c r="E34">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F34">
-        <v>77.59999999999999</v>
+        <v>78.56999999999999</v>
       </c>
       <c r="G34">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="H34">
-        <v>22.4</v>
+        <v>21.43</v>
       </c>
       <c r="I34">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -1553,25 +1553,25 @@
         <v>182</v>
       </c>
       <c r="C35">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="D35">
-        <v>20.33</v>
+        <v>0.55</v>
       </c>
       <c r="E35">
-        <v>138</v>
+        <v>164</v>
       </c>
       <c r="F35">
-        <v>75.81999999999999</v>
+        <v>90.11</v>
       </c>
       <c r="G35">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="H35">
-        <v>3.85</v>
+        <v>9.34</v>
       </c>
       <c r="I35">
-        <v>7</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -1582,25 +1582,25 @@
         <v>217</v>
       </c>
       <c r="C36">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D36">
-        <v>3.69</v>
+        <v>0</v>
       </c>
       <c r="E36">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F36">
-        <v>94.01000000000001</v>
+        <v>94.47</v>
       </c>
       <c r="G36">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H36">
-        <v>2.3</v>
+        <v>5.53</v>
       </c>
       <c r="I36">
-        <v>7.8</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -1608,28 +1608,28 @@
         <v>44</v>
       </c>
       <c r="B37">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C37">
-        <v>73</v>
+        <v>4</v>
       </c>
       <c r="D37">
-        <v>73</v>
+        <v>3.96</v>
       </c>
       <c r="E37">
-        <v>27</v>
+        <v>67</v>
       </c>
       <c r="F37">
-        <v>27</v>
+        <v>66.34</v>
       </c>
       <c r="G37">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>29.7</v>
       </c>
       <c r="I37">
-        <v>7.1</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -1637,7 +1637,7 @@
         <v>45</v>
       </c>
       <c r="B38">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -1649,13 +1649,13 @@
         <v>121</v>
       </c>
       <c r="F38">
-        <v>90.98</v>
+        <v>91.67</v>
       </c>
       <c r="G38">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H38">
-        <v>9.02</v>
+        <v>8.33</v>
       </c>
       <c r="I38">
         <v>7.2</v>
@@ -1666,25 +1666,25 @@
         <v>46</v>
       </c>
       <c r="B39">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C39">
         <v>2</v>
       </c>
       <c r="D39">
-        <v>1.98</v>
+        <v>1.96</v>
       </c>
       <c r="E39">
         <v>99</v>
       </c>
       <c r="F39">
-        <v>98.02</v>
+        <v>97.06</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H39">
-        <v>0</v>
+        <v>0.98</v>
       </c>
       <c r="I39">
         <v>8.300000000000001</v>
@@ -1756,16 +1756,16 @@
         <v>216</v>
       </c>
       <c r="C42">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D42">
-        <v>6.48</v>
+        <v>0</v>
       </c>
       <c r="E42">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="F42">
-        <v>93.52</v>
+        <v>100</v>
       </c>
       <c r="G42">
         <v>0</v>
@@ -1774,7 +1774,7 @@
         <v>0</v>
       </c>
       <c r="I42">
-        <v>8</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -1782,7 +1782,7 @@
         <v>50</v>
       </c>
       <c r="B43">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C43">
         <v>0</v>
@@ -1794,13 +1794,13 @@
         <v>32</v>
       </c>
       <c r="F43">
-        <v>86.48999999999999</v>
+        <v>88.89</v>
       </c>
       <c r="G43">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H43">
-        <v>13.51</v>
+        <v>11.11</v>
       </c>
       <c r="I43">
         <v>7.4</v>
@@ -1843,16 +1843,16 @@
         <v>72</v>
       </c>
       <c r="C45">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D45">
-        <v>19.44</v>
+        <v>0</v>
       </c>
       <c r="E45">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="F45">
-        <v>80.56</v>
+        <v>100</v>
       </c>
       <c r="G45">
         <v>0</v>
@@ -1861,7 +1861,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>8.800000000000001</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -1898,19 +1898,19 @@
         <v>54</v>
       </c>
       <c r="B47">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C47">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D47">
-        <v>16.07</v>
+        <v>13.51</v>
       </c>
       <c r="E47">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F47">
-        <v>83.93000000000001</v>
+        <v>86.48999999999999</v>
       </c>
       <c r="G47">
         <v>0</v>
@@ -1927,19 +1927,19 @@
         <v>55</v>
       </c>
       <c r="B48">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C48">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D48">
-        <v>35.81</v>
+        <v>35.37</v>
       </c>
       <c r="E48">
         <v>95</v>
       </c>
       <c r="F48">
-        <v>64.19</v>
+        <v>64.63</v>
       </c>
       <c r="G48">
         <v>0</v>
@@ -2014,7 +2014,7 @@
         <v>58</v>
       </c>
       <c r="B51">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C51">
         <v>0</v>
@@ -2023,16 +2023,16 @@
         <v>0</v>
       </c>
       <c r="E51">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F51">
-        <v>93.62</v>
+        <v>93.56</v>
       </c>
       <c r="G51">
         <v>15</v>
       </c>
       <c r="H51">
-        <v>6.38</v>
+        <v>6.44</v>
       </c>
       <c r="I51">
         <v>8.9</v>
@@ -2043,25 +2043,25 @@
         <v>59</v>
       </c>
       <c r="B52">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D52">
-        <v>0.74</v>
+        <v>0</v>
       </c>
       <c r="E52">
         <v>123</v>
       </c>
       <c r="F52">
-        <v>90.44</v>
+        <v>91.11</v>
       </c>
       <c r="G52">
         <v>12</v>
       </c>
       <c r="H52">
-        <v>8.82</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="I52">
         <v>8.6</v>
@@ -2117,22 +2117,25 @@
         <v>90</v>
       </c>
       <c r="C2">
-        <v>90</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>100</v>
+        <v>6.67</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>93.33</v>
       </c>
       <c r="G2">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <v>82.22</v>
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2143,22 +2146,25 @@
         <v>133</v>
       </c>
       <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
         <v>133</v>
       </c>
-      <c r="D3">
+      <c r="F3">
         <v>100</v>
       </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
       <c r="G3">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="H3">
-        <v>90.23</v>
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2166,25 +2172,28 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C4">
-        <v>194</v>
+        <v>68</v>
       </c>
       <c r="D4">
-        <v>100</v>
+        <v>35.23</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>47.15</v>
       </c>
       <c r="G4">
-        <v>194</v>
+        <v>102</v>
       </c>
       <c r="H4">
-        <v>100</v>
+        <v>52.85</v>
+      </c>
+      <c r="I4">
+        <v>7.3</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2192,25 +2201,28 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C5">
-        <v>123</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>93.44</v>
       </c>
       <c r="G5">
-        <v>96</v>
+        <v>8</v>
       </c>
       <c r="H5">
-        <v>78.05</v>
+        <v>6.56</v>
+      </c>
+      <c r="I5">
+        <v>8.9</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2259,10 +2271,10 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H7">
-        <v>97.89</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2273,22 +2285,25 @@
         <v>157</v>
       </c>
       <c r="C8">
-        <v>157</v>
+        <v>123</v>
       </c>
       <c r="D8">
-        <v>100</v>
+        <v>78.34</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>21.02</v>
       </c>
       <c r="G8">
-        <v>157</v>
+        <v>124</v>
       </c>
       <c r="H8">
-        <v>100</v>
+        <v>78.98</v>
+      </c>
+      <c r="I8">
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2325,22 +2340,25 @@
         <v>82</v>
       </c>
       <c r="C10">
-        <v>82</v>
+        <v>15</v>
       </c>
       <c r="D10">
-        <v>100</v>
+        <v>18.29</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>81.70999999999999</v>
       </c>
       <c r="G10">
-        <v>57</v>
+        <v>5</v>
       </c>
       <c r="H10">
-        <v>69.51000000000001</v>
+        <v>6.1</v>
+      </c>
+      <c r="I10">
+        <v>8.1</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -2363,10 +2381,10 @@
         <v>0</v>
       </c>
       <c r="G11">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H11">
-        <v>84.34999999999999</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -2377,22 +2395,25 @@
         <v>176</v>
       </c>
       <c r="C12">
-        <v>176</v>
+        <v>9</v>
       </c>
       <c r="D12">
-        <v>100</v>
+        <v>5.11</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>47.73</v>
       </c>
       <c r="G12">
-        <v>133</v>
+        <v>92</v>
       </c>
       <c r="H12">
-        <v>75.56999999999999</v>
+        <v>52.27</v>
+      </c>
+      <c r="I12">
+        <v>6.3</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -2400,10 +2421,10 @@
         <v>20</v>
       </c>
       <c r="B13">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C13">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D13">
         <v>100</v>
@@ -2418,7 +2439,7 @@
         <v>185</v>
       </c>
       <c r="H13">
-        <v>98.93000000000001</v>
+        <v>99.45999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -2426,10 +2447,10 @@
         <v>21</v>
       </c>
       <c r="B14">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C14">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D14">
         <v>100</v>
@@ -2441,10 +2462,10 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H14">
-        <v>81.16</v>
+        <v>81.43000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -2455,22 +2476,25 @@
         <v>169</v>
       </c>
       <c r="C15">
-        <v>169</v>
+        <v>119</v>
       </c>
       <c r="D15">
-        <v>100</v>
+        <v>70.41</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>28.99</v>
       </c>
       <c r="G15">
-        <v>131</v>
+        <v>82</v>
       </c>
       <c r="H15">
-        <v>77.51000000000001</v>
+        <v>48.52</v>
+      </c>
+      <c r="I15">
+        <v>8.4</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -2499,7 +2523,7 @@
         <v>93.33</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -2507,25 +2531,28 @@
         <v>83</v>
       </c>
       <c r="C17">
-        <v>83</v>
+        <v>13</v>
       </c>
       <c r="D17">
-        <v>100</v>
+        <v>15.66</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>84.34</v>
       </c>
       <c r="G17">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="H17">
-        <v>77.11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
+        <v>7.23</v>
+      </c>
+      <c r="I17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>25</v>
       </c>
@@ -2551,15 +2578,15 @@
         <v>76.72</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
         <v>26</v>
       </c>
       <c r="B19">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C19">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D19">
         <v>100</v>
@@ -2571,21 +2598,21 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="H19">
-        <v>85.62</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
+        <v>89.12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
         <v>27</v>
       </c>
       <c r="B20">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C20">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D20">
         <v>100</v>
@@ -2600,10 +2627,10 @@
         <v>122</v>
       </c>
       <c r="H20">
-        <v>61.62</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8">
+        <v>61.93</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -2611,25 +2638,28 @@
         <v>92</v>
       </c>
       <c r="C21">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="D21">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>72.83</v>
       </c>
       <c r="G21">
-        <v>92</v>
+        <v>25</v>
       </c>
       <c r="H21">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
+        <v>27.17</v>
+      </c>
+      <c r="I21">
+        <v>6.8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -2637,25 +2667,28 @@
         <v>72</v>
       </c>
       <c r="C22">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="D22">
-        <v>100</v>
+        <v>70.83</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G22">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="H22">
-        <v>97.22</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
+        <v>72.22</v>
+      </c>
+      <c r="I22">
+        <v>7.3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -2681,33 +2714,36 @@
         <v>87.72</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:9">
       <c r="A24" t="s">
         <v>31</v>
       </c>
       <c r="B24">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C24">
-        <v>128</v>
+        <v>43</v>
       </c>
       <c r="D24">
-        <v>100</v>
+        <v>33.33</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>86</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>66.67</v>
       </c>
       <c r="G24">
-        <v>116</v>
+        <v>32</v>
       </c>
       <c r="H24">
-        <v>90.63</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8">
+        <v>24.81</v>
+      </c>
+      <c r="I24">
+        <v>8.300000000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
       <c r="A25" t="s">
         <v>32</v>
       </c>
@@ -2733,7 +2769,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:9">
       <c r="A26" t="s">
         <v>33</v>
       </c>
@@ -2753,13 +2789,13 @@
         <v>0</v>
       </c>
       <c r="G26">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="H26">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
       <c r="A27" t="s">
         <v>34</v>
       </c>
@@ -2785,7 +2821,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:9">
       <c r="A28" t="s">
         <v>35</v>
       </c>
@@ -2805,13 +2841,13 @@
         <v>0</v>
       </c>
       <c r="G28">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H28">
-        <v>28.95</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8">
+        <v>31.58</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
       <c r="A29" t="s">
         <v>36</v>
       </c>
@@ -2819,25 +2855,28 @@
         <v>114</v>
       </c>
       <c r="C29">
-        <v>114</v>
+        <v>0</v>
       </c>
       <c r="D29">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>84.20999999999999</v>
       </c>
       <c r="G29">
-        <v>114</v>
+        <v>18</v>
       </c>
       <c r="H29">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8">
+        <v>15.79</v>
+      </c>
+      <c r="I29">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
       <c r="A30" t="s">
         <v>37</v>
       </c>
@@ -2863,7 +2902,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:9">
       <c r="A31" t="s">
         <v>38</v>
       </c>
@@ -2871,25 +2910,28 @@
         <v>152</v>
       </c>
       <c r="C31">
-        <v>152</v>
+        <v>47</v>
       </c>
       <c r="D31">
-        <v>100</v>
+        <v>30.92</v>
       </c>
       <c r="E31">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="F31">
-        <v>0</v>
+        <v>68.42</v>
       </c>
       <c r="G31">
-        <v>145</v>
+        <v>44</v>
       </c>
       <c r="H31">
-        <v>95.39</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8">
+        <v>28.95</v>
+      </c>
+      <c r="I31">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
       <c r="A32" t="s">
         <v>39</v>
       </c>
@@ -2897,33 +2939,36 @@
         <v>64</v>
       </c>
       <c r="C32">
-        <v>64</v>
+        <v>27</v>
       </c>
       <c r="D32">
-        <v>100</v>
+        <v>42.19</v>
       </c>
       <c r="E32">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="F32">
-        <v>0</v>
+        <v>57.81</v>
       </c>
       <c r="G32">
-        <v>64</v>
+        <v>27</v>
       </c>
       <c r="H32">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8">
+        <v>42.19</v>
+      </c>
+      <c r="I32">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
       <c r="A33" t="s">
         <v>40</v>
       </c>
       <c r="B33">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C33">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D33">
         <v>100</v>
@@ -2935,21 +2980,21 @@
         <v>0</v>
       </c>
       <c r="G33">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H33">
-        <v>83.93000000000001</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8">
+        <v>85.84</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
       <c r="A34" t="s">
         <v>41</v>
       </c>
       <c r="B34">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C34">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D34">
         <v>100</v>
@@ -2961,13 +3006,13 @@
         <v>0</v>
       </c>
       <c r="G34">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H34">
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:9">
       <c r="A35" t="s">
         <v>42</v>
       </c>
@@ -2975,25 +3020,28 @@
         <v>182</v>
       </c>
       <c r="C35">
-        <v>182</v>
+        <v>1</v>
       </c>
       <c r="D35">
-        <v>100</v>
+        <v>0.55</v>
       </c>
       <c r="E35">
-        <v>0</v>
+        <v>129</v>
       </c>
       <c r="F35">
-        <v>0</v>
+        <v>70.88</v>
       </c>
       <c r="G35">
-        <v>145</v>
+        <v>52</v>
       </c>
       <c r="H35">
-        <v>79.67</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8">
+        <v>28.57</v>
+      </c>
+      <c r="I35">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
       <c r="A36" t="s">
         <v>43</v>
       </c>
@@ -3001,85 +3049,94 @@
         <v>217</v>
       </c>
       <c r="C36">
-        <v>217</v>
+        <v>54</v>
       </c>
       <c r="D36">
-        <v>100</v>
+        <v>24.88</v>
       </c>
       <c r="E36">
-        <v>0</v>
+        <v>158</v>
       </c>
       <c r="F36">
-        <v>0</v>
+        <v>72.81</v>
       </c>
       <c r="G36">
-        <v>209</v>
+        <v>59</v>
       </c>
       <c r="H36">
-        <v>96.31</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8">
+        <v>27.19</v>
+      </c>
+      <c r="I36">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
       <c r="A37" t="s">
         <v>44</v>
       </c>
       <c r="B37">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C37">
-        <v>100</v>
+        <v>14</v>
       </c>
       <c r="D37">
-        <v>100</v>
+        <v>13.86</v>
       </c>
       <c r="E37">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="F37">
-        <v>0</v>
+        <v>62.38</v>
       </c>
       <c r="G37">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="H37">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
+        <v>33.66</v>
+      </c>
+      <c r="I37">
+        <v>6.9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
       <c r="A38" t="s">
         <v>45</v>
       </c>
       <c r="B38">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C38">
-        <v>133</v>
+        <v>20</v>
       </c>
       <c r="D38">
-        <v>100</v>
+        <v>15.15</v>
       </c>
       <c r="E38">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="F38">
-        <v>0</v>
+        <v>82.58</v>
       </c>
       <c r="G38">
-        <v>133</v>
+        <v>23</v>
       </c>
       <c r="H38">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
+        <v>17.42</v>
+      </c>
+      <c r="I38">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
       <c r="A39" t="s">
         <v>46</v>
       </c>
       <c r="B39">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C39">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D39">
         <v>100</v>
@@ -3091,13 +3148,13 @@
         <v>0</v>
       </c>
       <c r="G39">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H39">
-        <v>98.02</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8">
+        <v>98.04000000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
       <c r="A40" t="s">
         <v>47</v>
       </c>
@@ -3105,25 +3162,28 @@
         <v>94</v>
       </c>
       <c r="C40">
-        <v>94</v>
+        <v>20</v>
       </c>
       <c r="D40">
-        <v>100</v>
+        <v>21.28</v>
       </c>
       <c r="E40">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="F40">
-        <v>0</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="G40">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="H40">
-        <v>98.94</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8">
+        <v>25.53</v>
+      </c>
+      <c r="I40">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
       <c r="A41" t="s">
         <v>48</v>
       </c>
@@ -3149,7 +3209,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:9">
       <c r="A42" t="s">
         <v>49</v>
       </c>
@@ -3157,33 +3217,36 @@
         <v>216</v>
       </c>
       <c r="C42">
+        <v>0</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
         <v>216</v>
       </c>
-      <c r="D42">
+      <c r="F42">
         <v>100</v>
       </c>
-      <c r="E42">
-        <v>0</v>
-      </c>
-      <c r="F42">
-        <v>0</v>
-      </c>
       <c r="G42">
-        <v>202</v>
+        <v>0</v>
       </c>
       <c r="H42">
-        <v>93.52</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I42">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
       <c r="A43" t="s">
         <v>50</v>
       </c>
       <c r="B43">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C43">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D43">
         <v>100</v>
@@ -3195,13 +3258,13 @@
         <v>0</v>
       </c>
       <c r="G43">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H43">
         <v>100</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:9">
       <c r="A44" t="s">
         <v>51</v>
       </c>
@@ -3227,7 +3290,7 @@
         <v>92.75</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:9">
       <c r="A45" t="s">
         <v>52</v>
       </c>
@@ -3235,25 +3298,28 @@
         <v>72</v>
       </c>
       <c r="C45">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45">
         <v>72</v>
       </c>
-      <c r="D45">
+      <c r="F45">
         <v>100</v>
       </c>
-      <c r="E45">
-        <v>0</v>
-      </c>
-      <c r="F45">
-        <v>0</v>
-      </c>
       <c r="G45">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="H45">
-        <v>80.56</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I45">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
       <c r="A46" t="s">
         <v>53</v>
       </c>
@@ -3279,41 +3345,44 @@
         <v>97.94</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:9">
       <c r="A47" t="s">
         <v>54</v>
       </c>
       <c r="B47">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C47">
-        <v>112</v>
+        <v>78</v>
       </c>
       <c r="D47">
-        <v>100</v>
+        <v>70.27</v>
       </c>
       <c r="E47">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F47">
-        <v>0</v>
+        <v>29.73</v>
       </c>
       <c r="G47">
-        <v>94</v>
+        <v>63</v>
       </c>
       <c r="H47">
-        <v>83.93000000000001</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8">
+        <v>56.76</v>
+      </c>
+      <c r="I47">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
       <c r="A48" t="s">
         <v>55</v>
       </c>
       <c r="B48">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C48">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D48">
         <v>100</v>
@@ -3328,10 +3397,10 @@
         <v>95</v>
       </c>
       <c r="H48">
-        <v>64.19</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8">
+        <v>64.63</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
       <c r="A49" t="s">
         <v>56</v>
       </c>
@@ -3357,7 +3426,7 @@
         <v>83.33</v>
       </c>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:9">
       <c r="A50" t="s">
         <v>57</v>
       </c>
@@ -3383,56 +3452,62 @@
         <v>96.97</v>
       </c>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:9">
       <c r="A51" t="s">
         <v>58</v>
       </c>
       <c r="B51">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C51">
-        <v>235</v>
+        <v>0</v>
       </c>
       <c r="D51">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E51">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="F51">
-        <v>0</v>
+        <v>98.70999999999999</v>
       </c>
       <c r="G51">
-        <v>235</v>
+        <v>3</v>
       </c>
       <c r="H51">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8">
+        <v>1.29</v>
+      </c>
+      <c r="I51">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
       <c r="A52" t="s">
         <v>59</v>
       </c>
       <c r="B52">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C52">
-        <v>136</v>
+        <v>0</v>
       </c>
       <c r="D52">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E52">
-        <v>0</v>
+        <v>124</v>
       </c>
       <c r="F52">
-        <v>0</v>
+        <v>91.84999999999999</v>
       </c>
       <c r="G52">
-        <v>135</v>
+        <v>11</v>
       </c>
       <c r="H52">
-        <v>99.26000000000001</v>
+        <v>8.15</v>
+      </c>
+      <c r="I52">
+        <v>8.199999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -3485,16 +3560,16 @@
         <v>90</v>
       </c>
       <c r="C2">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>17.78</v>
+        <v>6.67</v>
       </c>
       <c r="E2">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="F2">
-        <v>82.22</v>
+        <v>93.33</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -3514,16 +3589,16 @@
         <v>133</v>
       </c>
       <c r="C3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>9.77</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="F3">
-        <v>90.23</v>
+        <v>100</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -3532,7 +3607,7 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>9.5</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -3540,7 +3615,7 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -3549,16 +3624,16 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F4">
-        <v>74.73999999999999</v>
+        <v>76.17</v>
       </c>
       <c r="G4">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="H4">
-        <v>25.26</v>
+        <v>23.83</v>
       </c>
       <c r="I4">
         <v>7.5</v>
@@ -3569,28 +3644,28 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C5">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>21.95</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="F5">
-        <v>73.98</v>
+        <v>93.44</v>
       </c>
       <c r="G5">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H5">
-        <v>4.07</v>
+        <v>6.56</v>
       </c>
       <c r="I5">
-        <v>7.7</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -3630,16 +3705,16 @@
         <v>95</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>2.11</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F7">
-        <v>94.73999999999999</v>
+        <v>96.84</v>
       </c>
       <c r="G7">
         <v>3</v>
@@ -3665,19 +3740,19 @@
         <v>0</v>
       </c>
       <c r="E8">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F8">
-        <v>91.08</v>
+        <v>90.45</v>
       </c>
       <c r="G8">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H8">
-        <v>8.92</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="I8">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -3717,16 +3792,16 @@
         <v>82</v>
       </c>
       <c r="C10">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="D10">
-        <v>30.49</v>
+        <v>12.2</v>
       </c>
       <c r="E10">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="F10">
-        <v>69.51000000000001</v>
+        <v>87.8</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -3735,7 +3810,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -3746,16 +3821,16 @@
         <v>147</v>
       </c>
       <c r="C11">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D11">
-        <v>15.65</v>
+        <v>14.29</v>
       </c>
       <c r="E11">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F11">
-        <v>63.95</v>
+        <v>65.31</v>
       </c>
       <c r="G11">
         <v>30</v>
@@ -3764,7 +3839,7 @@
         <v>20.41</v>
       </c>
       <c r="I11">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -3775,25 +3850,25 @@
         <v>176</v>
       </c>
       <c r="C12">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="D12">
-        <v>24.43</v>
+        <v>0</v>
       </c>
       <c r="E12">
-        <v>133</v>
+        <v>92</v>
       </c>
       <c r="F12">
-        <v>75.56999999999999</v>
+        <v>52.27</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>47.73</v>
       </c>
       <c r="I12">
-        <v>6.7</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -3801,19 +3876,19 @@
         <v>20</v>
       </c>
       <c r="B13">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13">
-        <v>1.07</v>
+        <v>0.54</v>
       </c>
       <c r="E13">
         <v>185</v>
       </c>
       <c r="F13">
-        <v>98.93000000000001</v>
+        <v>99.45999999999999</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -3830,19 +3905,19 @@
         <v>21</v>
       </c>
       <c r="B14">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C14">
         <v>13</v>
       </c>
       <c r="D14">
-        <v>18.84</v>
+        <v>18.57</v>
       </c>
       <c r="E14">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F14">
-        <v>81.16</v>
+        <v>81.43000000000001</v>
       </c>
       <c r="G14">
         <v>0</v>
@@ -3868,16 +3943,16 @@
         <v>22.49</v>
       </c>
       <c r="E15">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F15">
-        <v>77.51000000000001</v>
+        <v>76.92</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>0.59</v>
       </c>
       <c r="I15">
         <v>8.199999999999999</v>
@@ -3920,16 +3995,16 @@
         <v>83</v>
       </c>
       <c r="C17">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="D17">
-        <v>22.89</v>
+        <v>8.43</v>
       </c>
       <c r="E17">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="F17">
-        <v>77.11</v>
+        <v>91.56999999999999</v>
       </c>
       <c r="G17">
         <v>0</v>
@@ -3938,7 +4013,7 @@
         <v>0</v>
       </c>
       <c r="I17">
-        <v>7.2</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -3975,28 +4050,28 @@
         <v>26</v>
       </c>
       <c r="B19">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C19">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D19">
-        <v>14.38</v>
+        <v>10.88</v>
       </c>
       <c r="E19">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="F19">
-        <v>75.34</v>
+        <v>78.91</v>
       </c>
       <c r="G19">
         <v>15</v>
       </c>
       <c r="H19">
-        <v>10.27</v>
+        <v>10.2</v>
       </c>
       <c r="I19">
-        <v>8</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -4004,19 +4079,19 @@
         <v>27</v>
       </c>
       <c r="B20">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C20">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D20">
-        <v>38.38</v>
+        <v>38.07</v>
       </c>
       <c r="E20">
         <v>122</v>
       </c>
       <c r="F20">
-        <v>61.62</v>
+        <v>61.93</v>
       </c>
       <c r="G20">
         <v>0</v>
@@ -4042,19 +4117,19 @@
         <v>0</v>
       </c>
       <c r="E21">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="F21">
-        <v>78.26000000000001</v>
+        <v>72.83</v>
       </c>
       <c r="G21">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H21">
-        <v>21.74</v>
+        <v>27.17</v>
       </c>
       <c r="I21">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -4071,19 +4146,19 @@
         <v>2.78</v>
       </c>
       <c r="E22">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F22">
-        <v>79.17</v>
+        <v>81.94</v>
       </c>
       <c r="G22">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H22">
-        <v>18.06</v>
+        <v>15.28</v>
       </c>
       <c r="I22">
-        <v>6.8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -4120,19 +4195,19 @@
         <v>31</v>
       </c>
       <c r="B24">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C24">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D24">
-        <v>9.380000000000001</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="E24">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F24">
-        <v>90.63</v>
+        <v>91.47</v>
       </c>
       <c r="G24">
         <v>0</v>
@@ -4181,25 +4256,25 @@
         <v>55</v>
       </c>
       <c r="C26">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D26">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E26">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="F26">
-        <v>60</v>
+        <v>74.55</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="H26">
-        <v>0</v>
+        <v>25.45</v>
       </c>
       <c r="I26">
-        <v>7.6</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -4239,16 +4314,16 @@
         <v>114</v>
       </c>
       <c r="C28">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D28">
-        <v>71.05</v>
+        <v>68.42</v>
       </c>
       <c r="E28">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F28">
-        <v>28.95</v>
+        <v>31.58</v>
       </c>
       <c r="G28">
         <v>0</v>
@@ -4257,7 +4332,7 @@
         <v>0</v>
       </c>
       <c r="I28">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -4274,19 +4349,19 @@
         <v>0</v>
       </c>
       <c r="E29">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="F29">
-        <v>89.47</v>
+        <v>84.20999999999999</v>
       </c>
       <c r="G29">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H29">
-        <v>10.53</v>
+        <v>15.79</v>
       </c>
       <c r="I29">
-        <v>8</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -4326,25 +4401,25 @@
         <v>152</v>
       </c>
       <c r="C31">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D31">
-        <v>4.61</v>
+        <v>2.63</v>
       </c>
       <c r="E31">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F31">
-        <v>95.39</v>
+        <v>96.70999999999999</v>
       </c>
       <c r="G31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H31">
-        <v>0</v>
+        <v>0.66</v>
       </c>
       <c r="I31">
-        <v>8.9</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -4373,7 +4448,7 @@
         <v>7.81</v>
       </c>
       <c r="I32">
-        <v>9.4</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -4381,25 +4456,25 @@
         <v>40</v>
       </c>
       <c r="B33">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C33">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D33">
-        <v>16.07</v>
+        <v>14.16</v>
       </c>
       <c r="E33">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F33">
-        <v>83.93000000000001</v>
+        <v>84.95999999999999</v>
       </c>
       <c r="G33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H33">
-        <v>0</v>
+        <v>0.88</v>
       </c>
       <c r="I33">
         <v>8.1</v>
@@ -4410,7 +4485,7 @@
         <v>41</v>
       </c>
       <c r="B34">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -4419,19 +4494,19 @@
         <v>0</v>
       </c>
       <c r="E34">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F34">
-        <v>77.59999999999999</v>
+        <v>78.56999999999999</v>
       </c>
       <c r="G34">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="H34">
-        <v>22.4</v>
+        <v>21.43</v>
       </c>
       <c r="I34">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -4442,25 +4517,25 @@
         <v>182</v>
       </c>
       <c r="C35">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="D35">
-        <v>20.33</v>
+        <v>0.55</v>
       </c>
       <c r="E35">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="F35">
-        <v>75.81999999999999</v>
+        <v>70.88</v>
       </c>
       <c r="G35">
-        <v>7</v>
+        <v>52</v>
       </c>
       <c r="H35">
-        <v>3.85</v>
+        <v>28.57</v>
       </c>
       <c r="I35">
-        <v>7</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -4471,22 +4546,22 @@
         <v>217</v>
       </c>
       <c r="C36">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D36">
-        <v>3.69</v>
+        <v>0</v>
       </c>
       <c r="E36">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F36">
-        <v>94.01000000000001</v>
+        <v>93.09</v>
       </c>
       <c r="G36">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="H36">
-        <v>2.3</v>
+        <v>6.91</v>
       </c>
       <c r="I36">
         <v>7.8</v>
@@ -4497,28 +4572,28 @@
         <v>44</v>
       </c>
       <c r="B37">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C37">
-        <v>73</v>
+        <v>4</v>
       </c>
       <c r="D37">
-        <v>73</v>
+        <v>3.96</v>
       </c>
       <c r="E37">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="F37">
-        <v>27</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="G37">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>30.69</v>
       </c>
       <c r="I37">
-        <v>7.1</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -4526,7 +4601,7 @@
         <v>45</v>
       </c>
       <c r="B38">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -4535,19 +4610,19 @@
         <v>0</v>
       </c>
       <c r="E38">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="F38">
-        <v>90.98</v>
+        <v>95.45</v>
       </c>
       <c r="G38">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H38">
-        <v>9.02</v>
+        <v>4.55</v>
       </c>
       <c r="I38">
-        <v>7.2</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -4555,25 +4630,25 @@
         <v>46</v>
       </c>
       <c r="B39">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C39">
         <v>2</v>
       </c>
       <c r="D39">
-        <v>1.98</v>
+        <v>1.96</v>
       </c>
       <c r="E39">
         <v>99</v>
       </c>
       <c r="F39">
-        <v>98.02</v>
+        <v>97.06</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H39">
-        <v>0</v>
+        <v>0.98</v>
       </c>
       <c r="I39">
         <v>8.300000000000001</v>
@@ -4593,19 +4668,19 @@
         <v>1.06</v>
       </c>
       <c r="E40">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="F40">
-        <v>78.72</v>
+        <v>86.17</v>
       </c>
       <c r="G40">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="H40">
-        <v>20.21</v>
+        <v>12.77</v>
       </c>
       <c r="I40">
-        <v>6.9</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -4645,16 +4720,16 @@
         <v>216</v>
       </c>
       <c r="C42">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D42">
-        <v>6.48</v>
+        <v>0</v>
       </c>
       <c r="E42">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="F42">
-        <v>93.52</v>
+        <v>100</v>
       </c>
       <c r="G42">
         <v>0</v>
@@ -4663,7 +4738,7 @@
         <v>0</v>
       </c>
       <c r="I42">
-        <v>8</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -4671,7 +4746,7 @@
         <v>50</v>
       </c>
       <c r="B43">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C43">
         <v>0</v>
@@ -4683,13 +4758,13 @@
         <v>32</v>
       </c>
       <c r="F43">
-        <v>86.48999999999999</v>
+        <v>88.89</v>
       </c>
       <c r="G43">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H43">
-        <v>13.51</v>
+        <v>11.11</v>
       </c>
       <c r="I43">
         <v>7.4</v>
@@ -4732,16 +4807,16 @@
         <v>72</v>
       </c>
       <c r="C45">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D45">
-        <v>19.44</v>
+        <v>0</v>
       </c>
       <c r="E45">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="F45">
-        <v>80.56</v>
+        <v>100</v>
       </c>
       <c r="G45">
         <v>0</v>
@@ -4750,7 +4825,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>8.800000000000001</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -4787,19 +4862,19 @@
         <v>54</v>
       </c>
       <c r="B47">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C47">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D47">
-        <v>16.07</v>
+        <v>13.51</v>
       </c>
       <c r="E47">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F47">
-        <v>83.93000000000001</v>
+        <v>86.48999999999999</v>
       </c>
       <c r="G47">
         <v>0</v>
@@ -4808,7 +4883,7 @@
         <v>0</v>
       </c>
       <c r="I47">
-        <v>8.699999999999999</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -4816,19 +4891,19 @@
         <v>55</v>
       </c>
       <c r="B48">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C48">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D48">
-        <v>35.81</v>
+        <v>35.37</v>
       </c>
       <c r="E48">
         <v>95</v>
       </c>
       <c r="F48">
-        <v>64.19</v>
+        <v>64.63</v>
       </c>
       <c r="G48">
         <v>0</v>
@@ -4903,7 +4978,7 @@
         <v>58</v>
       </c>
       <c r="B51">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C51">
         <v>0</v>
@@ -4912,19 +4987,19 @@
         <v>0</v>
       </c>
       <c r="E51">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="F51">
-        <v>93.62</v>
+        <v>98.70999999999999</v>
       </c>
       <c r="G51">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="H51">
-        <v>6.38</v>
+        <v>1.29</v>
       </c>
       <c r="I51">
-        <v>8.9</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -4932,25 +5007,25 @@
         <v>59</v>
       </c>
       <c r="B52">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D52">
-        <v>0.74</v>
+        <v>0</v>
       </c>
       <c r="E52">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F52">
-        <v>90.44</v>
+        <v>91.84999999999999</v>
       </c>
       <c r="G52">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H52">
-        <v>8.82</v>
+        <v>8.15</v>
       </c>
       <c r="I52">
         <v>8.6</v>

</xml_diff>

<commit_message>
Segundo Parcial 7 noviembre
</commit_message>
<xml_diff>
--- a/Totales Docentes.xlsx
+++ b/Totales Docentes.xlsx
@@ -602,25 +602,25 @@
         <v>62</v>
       </c>
       <c r="C2">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>32.26</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="F2">
-        <v>67.73999999999999</v>
+        <v>93.55</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>6.45</v>
       </c>
       <c r="I2">
-        <v>8.699999999999999</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -628,7 +628,7 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -637,7 +637,7 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F3">
         <v>100</v>
@@ -657,7 +657,7 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -669,13 +669,13 @@
         <v>183</v>
       </c>
       <c r="F4">
-        <v>85.12</v>
+        <v>85.51000000000001</v>
       </c>
       <c r="G4">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H4">
-        <v>14.88</v>
+        <v>14.49</v>
       </c>
       <c r="I4">
         <v>8.199999999999999</v>
@@ -715,25 +715,25 @@
         <v>13</v>
       </c>
       <c r="B6">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C6">
         <v>4</v>
       </c>
       <c r="D6">
-        <v>2.29</v>
+        <v>2.27</v>
       </c>
       <c r="E6">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F6">
-        <v>85.14</v>
+        <v>85.23</v>
       </c>
       <c r="G6">
         <v>22</v>
       </c>
       <c r="H6">
-        <v>12.57</v>
+        <v>12.5</v>
       </c>
       <c r="I6">
         <v>7.9</v>
@@ -747,16 +747,16 @@
         <v>18</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>5.56</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F7">
-        <v>94.44</v>
+        <v>100</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -765,7 +765,7 @@
         <v>0</v>
       </c>
       <c r="I7">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -773,25 +773,25 @@
         <v>15</v>
       </c>
       <c r="B8">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>0.6899999999999999</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F8">
-        <v>96.53</v>
+        <v>96.5</v>
       </c>
       <c r="G8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H8">
-        <v>2.78</v>
+        <v>3.5</v>
       </c>
       <c r="I8">
         <v>8.9</v>
@@ -802,28 +802,28 @@
         <v>16</v>
       </c>
       <c r="B9">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C9">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="D9">
-        <v>24.08</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>140</v>
+        <v>173</v>
       </c>
       <c r="F9">
-        <v>73.3</v>
+        <v>91.05</v>
       </c>
       <c r="G9">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="H9">
-        <v>2.62</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="I9">
-        <v>8.199999999999999</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -831,7 +831,7 @@
         <v>17</v>
       </c>
       <c r="B10">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -840,16 +840,16 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F10">
-        <v>93.55</v>
+        <v>93.48</v>
       </c>
       <c r="G10">
         <v>6</v>
       </c>
       <c r="H10">
-        <v>6.45</v>
+        <v>6.52</v>
       </c>
       <c r="I10">
         <v>8</v>
@@ -947,28 +947,28 @@
         <v>21</v>
       </c>
       <c r="B14">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D14">
-        <v>6.33</v>
+        <v>3.75</v>
       </c>
       <c r="E14">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F14">
-        <v>93.67</v>
+        <v>93.75</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="I14">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -1008,25 +1008,25 @@
         <v>87</v>
       </c>
       <c r="C16">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D16">
-        <v>14.94</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="F16">
-        <v>85.06</v>
+        <v>94.25</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H16">
-        <v>0</v>
+        <v>5.75</v>
       </c>
       <c r="I16">
-        <v>8.800000000000001</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -1043,19 +1043,19 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F17">
-        <v>88.03</v>
+        <v>88.45999999999999</v>
       </c>
       <c r="G17">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H17">
-        <v>11.97</v>
+        <v>11.54</v>
       </c>
       <c r="I17">
-        <v>7.4</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1063,28 +1063,28 @@
         <v>25</v>
       </c>
       <c r="B18">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C18">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="D18">
-        <v>24.61</v>
+        <v>0</v>
       </c>
       <c r="E18">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="F18">
-        <v>75.39</v>
+        <v>87.37</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>12.63</v>
       </c>
       <c r="I18">
-        <v>7</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -1092,25 +1092,25 @@
         <v>26</v>
       </c>
       <c r="B19">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C19">
         <v>2</v>
       </c>
       <c r="D19">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="E19">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F19">
-        <v>78.33</v>
+        <v>78.43000000000001</v>
       </c>
       <c r="G19">
         <v>42</v>
       </c>
       <c r="H19">
-        <v>20.69</v>
+        <v>20.59</v>
       </c>
       <c r="I19">
         <v>7</v>
@@ -1121,25 +1121,25 @@
         <v>27</v>
       </c>
       <c r="B20">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C20">
         <v>25</v>
       </c>
       <c r="D20">
-        <v>15.43</v>
+        <v>15.34</v>
       </c>
       <c r="E20">
         <v>136</v>
       </c>
       <c r="F20">
-        <v>83.95</v>
+        <v>83.44</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H20">
-        <v>0.62</v>
+        <v>1.23</v>
       </c>
       <c r="I20">
         <v>8.300000000000001</v>
@@ -1153,22 +1153,22 @@
         <v>140</v>
       </c>
       <c r="C21">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D21">
-        <v>10.71</v>
+        <v>0</v>
       </c>
       <c r="E21">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="F21">
-        <v>74.29000000000001</v>
+        <v>80.70999999999999</v>
       </c>
       <c r="G21">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H21">
-        <v>15</v>
+        <v>19.29</v>
       </c>
       <c r="I21">
         <v>7</v>
@@ -1211,25 +1211,25 @@
         <v>234</v>
       </c>
       <c r="C23">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="D23">
-        <v>23.93</v>
+        <v>0</v>
       </c>
       <c r="E23">
-        <v>178</v>
+        <v>203</v>
       </c>
       <c r="F23">
-        <v>76.06999999999999</v>
+        <v>86.75</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="H23">
-        <v>0</v>
+        <v>13.25</v>
       </c>
       <c r="I23">
-        <v>7.1</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1237,25 +1237,25 @@
         <v>31</v>
       </c>
       <c r="B24">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C24">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D24">
-        <v>6.37</v>
+        <v>5.91</v>
       </c>
       <c r="E24">
         <v>163</v>
       </c>
       <c r="F24">
-        <v>79.90000000000001</v>
+        <v>80.3</v>
       </c>
       <c r="G24">
         <v>28</v>
       </c>
       <c r="H24">
-        <v>13.73</v>
+        <v>13.79</v>
       </c>
       <c r="I24">
         <v>8.1</v>
@@ -1327,25 +1327,25 @@
         <v>114</v>
       </c>
       <c r="C27">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D27">
-        <v>5.26</v>
+        <v>0</v>
       </c>
       <c r="E27">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F27">
-        <v>91.23</v>
+        <v>92.98</v>
       </c>
       <c r="G27">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H27">
-        <v>3.51</v>
+        <v>7.02</v>
       </c>
       <c r="I27">
-        <v>8.9</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1356,16 +1356,16 @@
         <v>18</v>
       </c>
       <c r="C28">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D28">
-        <v>77.78</v>
+        <v>0</v>
       </c>
       <c r="E28">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="F28">
-        <v>22.22</v>
+        <v>100</v>
       </c>
       <c r="G28">
         <v>0</v>
@@ -1374,7 +1374,7 @@
         <v>0</v>
       </c>
       <c r="I28">
-        <v>9</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1382,19 +1382,19 @@
         <v>36</v>
       </c>
       <c r="B29">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C29">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D29">
-        <v>24.58</v>
+        <v>23.93</v>
       </c>
       <c r="E29">
         <v>88</v>
       </c>
       <c r="F29">
-        <v>74.58</v>
+        <v>75.20999999999999</v>
       </c>
       <c r="G29">
         <v>1</v>
@@ -1498,7 +1498,7 @@
         <v>40</v>
       </c>
       <c r="B33">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C33">
         <v>0</v>
@@ -1507,16 +1507,16 @@
         <v>0</v>
       </c>
       <c r="E33">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F33">
-        <v>94.67</v>
+        <v>94.70999999999999</v>
       </c>
       <c r="G33">
         <v>9</v>
       </c>
       <c r="H33">
-        <v>5.33</v>
+        <v>5.29</v>
       </c>
       <c r="I33">
         <v>9.300000000000001</v>
@@ -1527,28 +1527,28 @@
         <v>41</v>
       </c>
       <c r="B34">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C34">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="D34">
-        <v>25.38</v>
+        <v>0</v>
       </c>
       <c r="E34">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="F34">
-        <v>74.62</v>
+        <v>77.86</v>
       </c>
       <c r="G34">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="H34">
-        <v>0</v>
+        <v>22.14</v>
       </c>
       <c r="I34">
-        <v>7.8</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -1559,25 +1559,25 @@
         <v>305</v>
       </c>
       <c r="C35">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D35">
-        <v>4.59</v>
+        <v>0</v>
       </c>
       <c r="E35">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="F35">
-        <v>79.02</v>
+        <v>80</v>
       </c>
       <c r="G35">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="H35">
-        <v>16.39</v>
+        <v>20</v>
       </c>
       <c r="I35">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -1614,28 +1614,28 @@
         <v>44</v>
       </c>
       <c r="B37">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C37">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D37">
-        <v>3.98</v>
+        <v>1</v>
       </c>
       <c r="E37">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F37">
-        <v>96.02</v>
+        <v>97</v>
       </c>
       <c r="G37">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I37">
-        <v>7.9</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -1646,16 +1646,16 @@
         <v>165</v>
       </c>
       <c r="C38">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D38">
-        <v>64.84999999999999</v>
+        <v>62.42</v>
       </c>
       <c r="E38">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F38">
-        <v>31.52</v>
+        <v>33.94</v>
       </c>
       <c r="G38">
         <v>6</v>
@@ -1664,7 +1664,7 @@
         <v>3.64</v>
       </c>
       <c r="I38">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -1672,25 +1672,25 @@
         <v>46</v>
       </c>
       <c r="B39">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C39">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D39">
-        <v>1.39</v>
+        <v>0</v>
       </c>
       <c r="E39">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F39">
-        <v>93.75</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="G39">
         <v>7</v>
       </c>
       <c r="H39">
-        <v>4.86</v>
+        <v>4.9</v>
       </c>
       <c r="I39">
         <v>8.699999999999999</v>
@@ -1759,28 +1759,28 @@
         <v>49</v>
       </c>
       <c r="B42">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C42">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D42">
-        <v>13.89</v>
+        <v>0</v>
       </c>
       <c r="E42">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="F42">
-        <v>65.97</v>
+        <v>71.33</v>
       </c>
       <c r="G42">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="H42">
-        <v>20.14</v>
+        <v>28.67</v>
       </c>
       <c r="I42">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -1788,7 +1788,7 @@
         <v>50</v>
       </c>
       <c r="B43">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C43">
         <v>0</v>
@@ -1800,16 +1800,16 @@
         <v>187</v>
       </c>
       <c r="F43">
-        <v>98.42</v>
+        <v>97.91</v>
       </c>
       <c r="G43">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H43">
-        <v>1.58</v>
+        <v>2.09</v>
       </c>
       <c r="I43">
-        <v>7.7</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -1875,7 +1875,7 @@
         <v>53</v>
       </c>
       <c r="B46">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C46">
         <v>0</v>
@@ -1884,16 +1884,16 @@
         <v>0</v>
       </c>
       <c r="E46">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F46">
-        <v>75.38</v>
+        <v>75.76000000000001</v>
       </c>
       <c r="G46">
         <v>16</v>
       </c>
       <c r="H46">
-        <v>24.62</v>
+        <v>24.24</v>
       </c>
       <c r="I46">
         <v>6.9</v>
@@ -1962,25 +1962,25 @@
         <v>56</v>
       </c>
       <c r="B49">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D49">
-        <v>3.23</v>
+        <v>0</v>
       </c>
       <c r="E49">
         <v>23</v>
       </c>
       <c r="F49">
-        <v>74.19</v>
+        <v>76.67</v>
       </c>
       <c r="G49">
         <v>7</v>
       </c>
       <c r="H49">
-        <v>22.58</v>
+        <v>23.33</v>
       </c>
       <c r="I49">
         <v>7.8</v>
@@ -1991,28 +1991,28 @@
         <v>57</v>
       </c>
       <c r="B50">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C50">
         <v>12</v>
       </c>
       <c r="D50">
-        <v>5.5</v>
+        <v>5.56</v>
       </c>
       <c r="E50">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F50">
-        <v>85.31999999999999</v>
+        <v>85.65000000000001</v>
       </c>
       <c r="G50">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H50">
-        <v>9.17</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I50">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -2020,25 +2020,25 @@
         <v>58</v>
       </c>
       <c r="B51">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C51">
         <v>16</v>
       </c>
       <c r="D51">
-        <v>8.289999999999999</v>
+        <v>8.33</v>
       </c>
       <c r="E51">
         <v>140</v>
       </c>
       <c r="F51">
-        <v>72.54000000000001</v>
+        <v>72.92</v>
       </c>
       <c r="G51">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H51">
-        <v>19.17</v>
+        <v>18.75</v>
       </c>
       <c r="I51">
         <v>6.4</v>
@@ -2049,25 +2049,25 @@
         <v>59</v>
       </c>
       <c r="B52">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C52">
         <v>7</v>
       </c>
       <c r="D52">
-        <v>5.11</v>
+        <v>5.07</v>
       </c>
       <c r="E52">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F52">
-        <v>85.40000000000001</v>
+        <v>85.51000000000001</v>
       </c>
       <c r="G52">
         <v>13</v>
       </c>
       <c r="H52">
-        <v>9.49</v>
+        <v>9.42</v>
       </c>
       <c r="I52">
         <v>7.5</v>
@@ -2181,22 +2181,25 @@
         <v>62</v>
       </c>
       <c r="C2">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="D2">
-        <v>100</v>
+        <v>3.23</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>90.31999999999999</v>
       </c>
       <c r="G2">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="H2">
-        <v>67.73999999999999</v>
+        <v>9.68</v>
+      </c>
+      <c r="I2">
+        <v>8.4</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2204,25 +2207,28 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C3">
-        <v>93</v>
+        <v>0</v>
       </c>
       <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>92</v>
+      </c>
+      <c r="F3">
         <v>100</v>
       </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
       <c r="G3">
-        <v>93</v>
+        <v>0</v>
       </c>
       <c r="H3">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>8.1</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2230,25 +2236,28 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C4">
-        <v>215</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>192</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>89.72</v>
       </c>
       <c r="G4">
-        <v>215</v>
+        <v>22</v>
       </c>
       <c r="H4">
-        <v>100</v>
+        <v>10.28</v>
+      </c>
+      <c r="I4">
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2259,22 +2268,25 @@
         <v>86</v>
       </c>
       <c r="C5">
-        <v>86</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>100</v>
+        <v>3.49</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>88.37</v>
       </c>
       <c r="G5">
-        <v>85</v>
+        <v>9</v>
       </c>
       <c r="H5">
-        <v>98.84</v>
+        <v>10.47</v>
+      </c>
+      <c r="I5">
+        <v>7.5</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2282,25 +2294,28 @@
         <v>13</v>
       </c>
       <c r="B6">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C6">
-        <v>175</v>
+        <v>68</v>
       </c>
       <c r="D6">
-        <v>100</v>
+        <v>38.64</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>93</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>52.84</v>
       </c>
       <c r="G6">
-        <v>171</v>
+        <v>79</v>
       </c>
       <c r="H6">
-        <v>97.70999999999999</v>
+        <v>44.89</v>
+      </c>
+      <c r="I6">
+        <v>7.8</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2311,22 +2326,25 @@
         <v>18</v>
       </c>
       <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
         <v>18</v>
       </c>
-      <c r="D7">
+      <c r="F7">
         <v>100</v>
       </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
       <c r="G7">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>94.44</v>
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>9.6</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2334,10 +2352,10 @@
         <v>15</v>
       </c>
       <c r="B8">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C8">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D8">
         <v>100</v>
@@ -2352,7 +2370,7 @@
         <v>143</v>
       </c>
       <c r="H8">
-        <v>99.31</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2360,25 +2378,28 @@
         <v>16</v>
       </c>
       <c r="B9">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C9">
-        <v>191</v>
+        <v>49</v>
       </c>
       <c r="D9">
-        <v>100</v>
+        <v>25.79</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>129</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>67.89</v>
       </c>
       <c r="G9">
-        <v>145</v>
+        <v>61</v>
       </c>
       <c r="H9">
-        <v>75.92</v>
+        <v>32.11</v>
+      </c>
+      <c r="I9">
+        <v>7.6</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2386,25 +2407,28 @@
         <v>17</v>
       </c>
       <c r="B10">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C10">
-        <v>93</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>89</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>96.73999999999999</v>
       </c>
       <c r="G10">
-        <v>93</v>
+        <v>3</v>
       </c>
       <c r="H10">
-        <v>100</v>
+        <v>3.26</v>
+      </c>
+      <c r="I10">
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -2441,22 +2465,25 @@
         <v>123</v>
       </c>
       <c r="C12">
-        <v>123</v>
+        <v>80</v>
       </c>
       <c r="D12">
-        <v>100</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>25.2</v>
       </c>
       <c r="G12">
-        <v>111</v>
+        <v>80</v>
       </c>
       <c r="H12">
-        <v>90.23999999999999</v>
+        <v>65.04000000000001</v>
+      </c>
+      <c r="I12">
+        <v>7.1</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -2467,22 +2494,25 @@
         <v>186</v>
       </c>
       <c r="C13">
-        <v>186</v>
+        <v>32</v>
       </c>
       <c r="D13">
-        <v>100</v>
+        <v>17.2</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>72.58</v>
       </c>
       <c r="G13">
-        <v>160</v>
+        <v>25</v>
       </c>
       <c r="H13">
-        <v>86.02</v>
+        <v>13.44</v>
+      </c>
+      <c r="I13">
+        <v>7.9</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -2490,10 +2520,10 @@
         <v>21</v>
       </c>
       <c r="B14">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C14">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D14">
         <v>100</v>
@@ -2505,10 +2535,10 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H14">
-        <v>93.67</v>
+        <v>96.25</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -2519,22 +2549,25 @@
         <v>66</v>
       </c>
       <c r="C15">
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="D15">
-        <v>100</v>
+        <v>1.52</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>98.48</v>
       </c>
       <c r="G15">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="H15">
-        <v>98.48</v>
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>6.7</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -2545,25 +2578,28 @@
         <v>87</v>
       </c>
       <c r="C16">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="D16">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>83.91</v>
       </c>
       <c r="G16">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="H16">
-        <v>85.06</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
+        <v>16.09</v>
+      </c>
+      <c r="I16">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -2589,41 +2625,44 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>25</v>
       </c>
       <c r="B18">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C18">
-        <v>191</v>
+        <v>6</v>
       </c>
       <c r="D18">
-        <v>100</v>
+        <v>3.16</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>147</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>77.37</v>
       </c>
       <c r="G18">
-        <v>144</v>
+        <v>43</v>
       </c>
       <c r="H18">
-        <v>75.39</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
+        <v>22.63</v>
+      </c>
+      <c r="I18">
+        <v>6.7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
         <v>26</v>
       </c>
       <c r="B19">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C19">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D19">
         <v>100</v>
@@ -2635,21 +2674,21 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H19">
-        <v>99.01000000000001</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
+        <v>99.02</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
         <v>27</v>
       </c>
       <c r="B20">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C20">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D20">
         <v>100</v>
@@ -2661,13 +2700,13 @@
         <v>0</v>
       </c>
       <c r="G20">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H20">
-        <v>84.56999999999999</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8">
+        <v>84.66</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -2687,13 +2726,13 @@
         <v>0</v>
       </c>
       <c r="G21">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="H21">
-        <v>89.29000000000001</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -2701,25 +2740,28 @@
         <v>109</v>
       </c>
       <c r="C22">
-        <v>109</v>
+        <v>41</v>
       </c>
       <c r="D22">
-        <v>100</v>
+        <v>37.61</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>62.39</v>
       </c>
       <c r="G22">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>62.39</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I22">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -2727,51 +2769,57 @@
         <v>234</v>
       </c>
       <c r="C23">
-        <v>234</v>
+        <v>4</v>
       </c>
       <c r="D23">
-        <v>100</v>
+        <v>1.71</v>
       </c>
       <c r="E23">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>81.62</v>
       </c>
       <c r="G23">
-        <v>178</v>
+        <v>43</v>
       </c>
       <c r="H23">
-        <v>76.06999999999999</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
+        <v>18.38</v>
+      </c>
+      <c r="I23">
+        <v>6.9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
       <c r="A24" t="s">
         <v>31</v>
       </c>
       <c r="B24">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C24">
-        <v>204</v>
+        <v>123</v>
       </c>
       <c r="D24">
-        <v>100</v>
+        <v>60.59</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>34.98</v>
       </c>
       <c r="G24">
-        <v>191</v>
+        <v>120</v>
       </c>
       <c r="H24">
-        <v>93.63</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8">
+        <v>59.11</v>
+      </c>
+      <c r="I24">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
       <c r="A25" t="s">
         <v>32</v>
       </c>
@@ -2797,7 +2845,7 @@
         <v>87.8</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:9">
       <c r="A26" t="s">
         <v>33</v>
       </c>
@@ -2805,25 +2853,28 @@
         <v>138</v>
       </c>
       <c r="C26">
-        <v>138</v>
+        <v>0</v>
       </c>
       <c r="D26">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>134</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="G26">
-        <v>138</v>
+        <v>4</v>
       </c>
       <c r="H26">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8">
+        <v>2.9</v>
+      </c>
+      <c r="I26">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
       <c r="A27" t="s">
         <v>34</v>
       </c>
@@ -2831,25 +2882,28 @@
         <v>114</v>
       </c>
       <c r="C27">
-        <v>114</v>
+        <v>21</v>
       </c>
       <c r="D27">
-        <v>100</v>
+        <v>18.42</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>77.19</v>
       </c>
       <c r="G27">
-        <v>108</v>
+        <v>26</v>
       </c>
       <c r="H27">
-        <v>94.73999999999999</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8">
+        <v>22.81</v>
+      </c>
+      <c r="I27">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
       <c r="A28" t="s">
         <v>35</v>
       </c>
@@ -2857,51 +2911,57 @@
         <v>18</v>
       </c>
       <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
         <v>18</v>
       </c>
-      <c r="D28">
+      <c r="F28">
         <v>100</v>
       </c>
-      <c r="E28">
-        <v>0</v>
-      </c>
-      <c r="F28">
-        <v>0</v>
-      </c>
       <c r="G28">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H28">
-        <v>22.22</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I28">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
       <c r="A29" t="s">
         <v>36</v>
       </c>
       <c r="B29">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C29">
-        <v>118</v>
+        <v>36</v>
       </c>
       <c r="D29">
-        <v>100</v>
+        <v>30.77</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>66.67</v>
       </c>
       <c r="G29">
-        <v>89</v>
+        <v>11</v>
       </c>
       <c r="H29">
-        <v>75.42</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8">
+        <v>9.4</v>
+      </c>
+      <c r="I29">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
       <c r="A30" t="s">
         <v>37</v>
       </c>
@@ -2909,25 +2969,28 @@
         <v>71</v>
       </c>
       <c r="C30">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="D30">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>90.14</v>
       </c>
       <c r="G30">
-        <v>71</v>
+        <v>7</v>
       </c>
       <c r="H30">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8">
+        <v>9.859999999999999</v>
+      </c>
+      <c r="I30">
+        <v>8.699999999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
       <c r="A31" t="s">
         <v>38</v>
       </c>
@@ -2953,7 +3016,7 @@
         <v>92.31</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:9">
       <c r="A32" t="s">
         <v>39</v>
       </c>
@@ -2961,77 +3024,86 @@
         <v>184</v>
       </c>
       <c r="C32">
-        <v>184</v>
+        <v>1</v>
       </c>
       <c r="D32">
-        <v>100</v>
+        <v>0.54</v>
       </c>
       <c r="E32">
-        <v>0</v>
+        <v>174</v>
       </c>
       <c r="F32">
-        <v>0</v>
+        <v>94.56999999999999</v>
       </c>
       <c r="G32">
-        <v>183</v>
+        <v>9</v>
       </c>
       <c r="H32">
-        <v>99.45999999999999</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8">
+        <v>4.89</v>
+      </c>
+      <c r="I32">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
       <c r="A33" t="s">
         <v>40</v>
       </c>
       <c r="B33">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C33">
-        <v>169</v>
+        <v>0</v>
       </c>
       <c r="D33">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>98.23999999999999</v>
       </c>
       <c r="G33">
-        <v>169</v>
+        <v>3</v>
       </c>
       <c r="H33">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8">
+        <v>1.76</v>
+      </c>
+      <c r="I33">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
       <c r="A34" t="s">
         <v>41</v>
       </c>
       <c r="B34">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C34">
-        <v>130</v>
+        <v>0</v>
       </c>
       <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34">
         <v>100</v>
       </c>
-      <c r="E34">
-        <v>0</v>
-      </c>
       <c r="F34">
-        <v>0</v>
+        <v>76.34</v>
       </c>
       <c r="G34">
-        <v>97</v>
+        <v>31</v>
       </c>
       <c r="H34">
-        <v>74.62</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8">
+        <v>23.66</v>
+      </c>
+      <c r="I34">
+        <v>7.3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
       <c r="A35" t="s">
         <v>42</v>
       </c>
@@ -3039,25 +3111,28 @@
         <v>305</v>
       </c>
       <c r="C35">
-        <v>305</v>
+        <v>176</v>
       </c>
       <c r="D35">
-        <v>100</v>
+        <v>57.7</v>
       </c>
       <c r="E35">
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="F35">
-        <v>0</v>
+        <v>34.43</v>
       </c>
       <c r="G35">
-        <v>291</v>
+        <v>200</v>
       </c>
       <c r="H35">
-        <v>95.41</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8">
+        <v>65.56999999999999</v>
+      </c>
+      <c r="I35">
+        <v>7.3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
       <c r="A36" t="s">
         <v>43</v>
       </c>
@@ -3065,51 +3140,57 @@
         <v>186</v>
       </c>
       <c r="C36">
-        <v>186</v>
+        <v>12</v>
       </c>
       <c r="D36">
-        <v>100</v>
+        <v>6.45</v>
       </c>
       <c r="E36">
-        <v>0</v>
+        <v>151</v>
       </c>
       <c r="F36">
-        <v>0</v>
+        <v>81.18000000000001</v>
       </c>
       <c r="G36">
-        <v>174</v>
+        <v>23</v>
       </c>
       <c r="H36">
-        <v>93.55</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8">
+        <v>12.37</v>
+      </c>
+      <c r="I36">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
       <c r="A37" t="s">
         <v>44</v>
       </c>
       <c r="B37">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C37">
-        <v>201</v>
+        <v>7</v>
       </c>
       <c r="D37">
-        <v>100</v>
+        <v>3.5</v>
       </c>
       <c r="E37">
-        <v>0</v>
+        <v>184</v>
       </c>
       <c r="F37">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="G37">
-        <v>193</v>
+        <v>14</v>
       </c>
       <c r="H37">
-        <v>96.02</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
+        <v>7</v>
+      </c>
+      <c r="I37">
+        <v>8.300000000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
       <c r="A38" t="s">
         <v>45</v>
       </c>
@@ -3117,51 +3198,57 @@
         <v>165</v>
       </c>
       <c r="C38">
-        <v>165</v>
+        <v>147</v>
       </c>
       <c r="D38">
-        <v>100</v>
+        <v>89.09</v>
       </c>
       <c r="E38">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F38">
-        <v>0</v>
+        <v>9.09</v>
       </c>
       <c r="G38">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="H38">
-        <v>35.15</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
+        <v>28.48</v>
+      </c>
+      <c r="I38">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
       <c r="A39" t="s">
         <v>46</v>
       </c>
       <c r="B39">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C39">
-        <v>144</v>
+        <v>1</v>
       </c>
       <c r="D39">
-        <v>100</v>
+        <v>0.7</v>
       </c>
       <c r="E39">
-        <v>0</v>
+        <v>137</v>
       </c>
       <c r="F39">
-        <v>0</v>
+        <v>95.8</v>
       </c>
       <c r="G39">
-        <v>142</v>
+        <v>6</v>
       </c>
       <c r="H39">
-        <v>98.61</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8">
+        <v>4.2</v>
+      </c>
+      <c r="I39">
+        <v>9.199999999999999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
       <c r="A40" t="s">
         <v>47</v>
       </c>
@@ -3169,25 +3256,28 @@
         <v>66</v>
       </c>
       <c r="C40">
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="D40">
-        <v>100</v>
+        <v>1.52</v>
       </c>
       <c r="E40">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="F40">
-        <v>0</v>
+        <v>92.42</v>
       </c>
       <c r="G40">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="H40">
-        <v>98.48</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8">
+        <v>6.06</v>
+      </c>
+      <c r="I40">
+        <v>8.300000000000001</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
       <c r="A41" t="s">
         <v>48</v>
       </c>
@@ -3195,77 +3285,86 @@
         <v>63</v>
       </c>
       <c r="C41">
-        <v>63</v>
+        <v>5</v>
       </c>
       <c r="D41">
-        <v>100</v>
+        <v>7.94</v>
       </c>
       <c r="E41">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="F41">
-        <v>0</v>
+        <v>85.70999999999999</v>
       </c>
       <c r="G41">
-        <v>58</v>
+        <v>4</v>
       </c>
       <c r="H41">
-        <v>92.06</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8">
+        <v>6.35</v>
+      </c>
+      <c r="I41">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
       <c r="A42" t="s">
         <v>49</v>
       </c>
       <c r="B42">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C42">
-        <v>144</v>
+        <v>0</v>
       </c>
       <c r="D42">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E42">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="F42">
-        <v>0</v>
+        <v>59.44</v>
       </c>
       <c r="G42">
-        <v>124</v>
+        <v>58</v>
       </c>
       <c r="H42">
-        <v>86.11</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8">
+        <v>40.56</v>
+      </c>
+      <c r="I42">
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
       <c r="A43" t="s">
         <v>50</v>
       </c>
       <c r="B43">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C43">
-        <v>190</v>
+        <v>21</v>
       </c>
       <c r="D43">
-        <v>100</v>
+        <v>10.99</v>
       </c>
       <c r="E43">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="F43">
-        <v>0</v>
+        <v>87.43000000000001</v>
       </c>
       <c r="G43">
-        <v>190</v>
+        <v>24</v>
       </c>
       <c r="H43">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8">
+        <v>12.57</v>
+      </c>
+      <c r="I43">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
       <c r="A44" t="s">
         <v>51</v>
       </c>
@@ -3291,7 +3390,7 @@
         <v>56.41</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:9">
       <c r="A45" t="s">
         <v>52</v>
       </c>
@@ -3299,51 +3398,57 @@
         <v>39</v>
       </c>
       <c r="C45">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="D45">
-        <v>100</v>
+        <v>43.59</v>
       </c>
       <c r="E45">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F45">
-        <v>0</v>
+        <v>56.41</v>
       </c>
       <c r="G45">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="H45">
-        <v>71.79000000000001</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8">
+        <v>15.38</v>
+      </c>
+      <c r="I45">
+        <v>9.199999999999999</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
       <c r="A46" t="s">
         <v>53</v>
       </c>
       <c r="B46">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C46">
-        <v>65</v>
+        <v>1</v>
       </c>
       <c r="D46">
-        <v>100</v>
+        <v>1.52</v>
       </c>
       <c r="E46">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="F46">
-        <v>0</v>
+        <v>72.73</v>
       </c>
       <c r="G46">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="H46">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8">
+        <v>27.27</v>
+      </c>
+      <c r="I46">
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9">
       <c r="A47" t="s">
         <v>54</v>
       </c>
@@ -3351,25 +3456,28 @@
         <v>47</v>
       </c>
       <c r="C47">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="D47">
-        <v>100</v>
+        <v>21.28</v>
       </c>
       <c r="E47">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="F47">
-        <v>0</v>
+        <v>78.72</v>
       </c>
       <c r="G47">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="H47">
-        <v>78.72</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I47">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
       <c r="A48" t="s">
         <v>55</v>
       </c>
@@ -3377,33 +3485,36 @@
         <v>64</v>
       </c>
       <c r="C48">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="D48">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E48">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="F48">
-        <v>0</v>
+        <v>82.81</v>
       </c>
       <c r="G48">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="H48">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8">
+        <v>17.19</v>
+      </c>
+      <c r="I48">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
       <c r="A49" t="s">
         <v>56</v>
       </c>
       <c r="B49">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C49">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D49">
         <v>100</v>
@@ -3418,18 +3529,18 @@
         <v>30</v>
       </c>
       <c r="H49">
-        <v>96.77</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
       <c r="A50" t="s">
         <v>57</v>
       </c>
       <c r="B50">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C50">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="D50">
         <v>100</v>
@@ -3441,21 +3552,21 @@
         <v>0</v>
       </c>
       <c r="G50">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H50">
-        <v>94.5</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8">
+        <v>94.44</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9">
       <c r="A51" t="s">
         <v>58</v>
       </c>
       <c r="B51">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C51">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D51">
         <v>100</v>
@@ -3467,39 +3578,42 @@
         <v>0</v>
       </c>
       <c r="G51">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H51">
-        <v>91.70999999999999</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8">
+        <v>91.67</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
       <c r="A52" t="s">
         <v>59</v>
       </c>
       <c r="B52">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C52">
-        <v>137</v>
+        <v>7</v>
       </c>
       <c r="D52">
-        <v>100</v>
+        <v>5.07</v>
       </c>
       <c r="E52">
-        <v>0</v>
+        <v>124</v>
       </c>
       <c r="F52">
-        <v>0</v>
+        <v>89.86</v>
       </c>
       <c r="G52">
-        <v>130</v>
+        <v>7</v>
       </c>
       <c r="H52">
-        <v>94.89</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8">
+        <v>5.07</v>
+      </c>
+      <c r="I52">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9">
       <c r="A53" t="s">
         <v>60</v>
       </c>
@@ -3507,25 +3621,28 @@
         <v>102</v>
       </c>
       <c r="C53">
+        <v>0</v>
+      </c>
+      <c r="D53">
+        <v>0</v>
+      </c>
+      <c r="E53">
         <v>102</v>
       </c>
-      <c r="D53">
+      <c r="F53">
         <v>100</v>
       </c>
-      <c r="E53">
-        <v>0</v>
-      </c>
-      <c r="F53">
-        <v>0</v>
-      </c>
       <c r="G53">
-        <v>102</v>
+        <v>0</v>
       </c>
       <c r="H53">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I53">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9">
       <c r="A54" t="s">
         <v>61</v>
       </c>
@@ -3533,22 +3650,25 @@
         <v>118</v>
       </c>
       <c r="C54">
-        <v>118</v>
+        <v>4</v>
       </c>
       <c r="D54">
-        <v>100</v>
+        <v>3.39</v>
       </c>
       <c r="E54">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="F54">
-        <v>0</v>
+        <v>92.37</v>
       </c>
       <c r="G54">
-        <v>118</v>
+        <v>9</v>
       </c>
       <c r="H54">
-        <v>100</v>
+        <v>7.63</v>
+      </c>
+      <c r="I54">
+        <v>8.5</v>
       </c>
     </row>
   </sheetData>
@@ -3601,25 +3721,25 @@
         <v>62</v>
       </c>
       <c r="C2">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>32.26</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="F2">
-        <v>67.73999999999999</v>
+        <v>90.31999999999999</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>9.68</v>
       </c>
       <c r="I2">
-        <v>8.699999999999999</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -3627,7 +3747,7 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -3636,7 +3756,7 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F3">
         <v>100</v>
@@ -3648,7 +3768,7 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>9.800000000000001</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -3656,7 +3776,7 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -3665,19 +3785,19 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="F4">
-        <v>85.12</v>
+        <v>89.72</v>
       </c>
       <c r="G4">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="H4">
-        <v>14.88</v>
+        <v>10.28</v>
       </c>
       <c r="I4">
-        <v>8.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -3694,19 +3814,19 @@
         <v>1.16</v>
       </c>
       <c r="E5">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F5">
-        <v>96.51000000000001</v>
+        <v>90.7</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <v>2.33</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="I5">
-        <v>7.8</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -3714,28 +3834,28 @@
         <v>13</v>
       </c>
       <c r="B6">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C6">
         <v>4</v>
       </c>
       <c r="D6">
-        <v>2.29</v>
+        <v>2.27</v>
       </c>
       <c r="E6">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F6">
-        <v>85.14</v>
+        <v>83.52</v>
       </c>
       <c r="G6">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H6">
-        <v>12.57</v>
+        <v>14.2</v>
       </c>
       <c r="I6">
-        <v>7.9</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -3746,16 +3866,16 @@
         <v>18</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>5.56</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F7">
-        <v>94.44</v>
+        <v>100</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -3764,7 +3884,7 @@
         <v>0</v>
       </c>
       <c r="I7">
-        <v>8.5</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -3772,25 +3892,25 @@
         <v>15</v>
       </c>
       <c r="B8">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>0.6899999999999999</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F8">
-        <v>96.53</v>
+        <v>96.5</v>
       </c>
       <c r="G8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H8">
-        <v>2.78</v>
+        <v>3.5</v>
       </c>
       <c r="I8">
         <v>8.9</v>
@@ -3801,28 +3921,28 @@
         <v>16</v>
       </c>
       <c r="B9">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C9">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="D9">
-        <v>24.08</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>140</v>
+        <v>171</v>
       </c>
       <c r="F9">
-        <v>73.3</v>
+        <v>90</v>
       </c>
       <c r="G9">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="H9">
-        <v>2.62</v>
+        <v>10</v>
       </c>
       <c r="I9">
-        <v>8.199999999999999</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -3830,7 +3950,7 @@
         <v>17</v>
       </c>
       <c r="B10">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -3839,19 +3959,19 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F10">
-        <v>93.55</v>
+        <v>96.73999999999999</v>
       </c>
       <c r="G10">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H10">
-        <v>6.45</v>
+        <v>3.26</v>
       </c>
       <c r="I10">
-        <v>8</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -3897,19 +4017,19 @@
         <v>9.76</v>
       </c>
       <c r="E12">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="F12">
-        <v>59.35</v>
+        <v>64.23</v>
       </c>
       <c r="G12">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="H12">
-        <v>30.89</v>
+        <v>26.02</v>
       </c>
       <c r="I12">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -3926,19 +4046,19 @@
         <v>13.98</v>
       </c>
       <c r="E13">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="F13">
-        <v>68.81999999999999</v>
+        <v>75.81</v>
       </c>
       <c r="G13">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="H13">
-        <v>17.2</v>
+        <v>10.22</v>
       </c>
       <c r="I13">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -3946,28 +4066,28 @@
         <v>21</v>
       </c>
       <c r="B14">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D14">
-        <v>6.33</v>
+        <v>3.75</v>
       </c>
       <c r="E14">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F14">
-        <v>93.67</v>
+        <v>93.75</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="I14">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -3996,7 +4116,7 @@
         <v>0</v>
       </c>
       <c r="I15">
-        <v>8.300000000000001</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -4007,25 +4127,25 @@
         <v>87</v>
       </c>
       <c r="C16">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D16">
-        <v>14.94</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F16">
-        <v>85.06</v>
+        <v>83.91</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="H16">
-        <v>0</v>
+        <v>16.09</v>
       </c>
       <c r="I16">
-        <v>8.800000000000001</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -4042,19 +4162,19 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F17">
-        <v>88.03</v>
+        <v>88.45999999999999</v>
       </c>
       <c r="G17">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H17">
-        <v>11.97</v>
+        <v>11.54</v>
       </c>
       <c r="I17">
-        <v>7.4</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -4062,28 +4182,28 @@
         <v>25</v>
       </c>
       <c r="B18">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C18">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="D18">
-        <v>24.61</v>
+        <v>0</v>
       </c>
       <c r="E18">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="F18">
-        <v>75.39</v>
+        <v>79.47</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="I18">
-        <v>7</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -4091,25 +4211,25 @@
         <v>26</v>
       </c>
       <c r="B19">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C19">
         <v>2</v>
       </c>
       <c r="D19">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="E19">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F19">
-        <v>78.33</v>
+        <v>78.43000000000001</v>
       </c>
       <c r="G19">
         <v>42</v>
       </c>
       <c r="H19">
-        <v>20.69</v>
+        <v>20.59</v>
       </c>
       <c r="I19">
         <v>7</v>
@@ -4120,25 +4240,25 @@
         <v>27</v>
       </c>
       <c r="B20">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C20">
         <v>25</v>
       </c>
       <c r="D20">
-        <v>15.43</v>
+        <v>15.34</v>
       </c>
       <c r="E20">
         <v>136</v>
       </c>
       <c r="F20">
-        <v>83.95</v>
+        <v>83.44</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H20">
-        <v>0.62</v>
+        <v>1.23</v>
       </c>
       <c r="I20">
         <v>8.300000000000001</v>
@@ -4152,25 +4272,25 @@
         <v>140</v>
       </c>
       <c r="C21">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D21">
-        <v>10.71</v>
+        <v>0</v>
       </c>
       <c r="E21">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="F21">
-        <v>74.29000000000001</v>
+        <v>80.70999999999999</v>
       </c>
       <c r="G21">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H21">
-        <v>15</v>
+        <v>19.29</v>
       </c>
       <c r="I21">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -4199,7 +4319,7 @@
         <v>0</v>
       </c>
       <c r="I22">
-        <v>8.6</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -4210,25 +4330,25 @@
         <v>234</v>
       </c>
       <c r="C23">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="D23">
-        <v>23.93</v>
+        <v>0</v>
       </c>
       <c r="E23">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="F23">
-        <v>76.06999999999999</v>
+        <v>82.48</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="H23">
-        <v>0</v>
+        <v>17.52</v>
       </c>
       <c r="I23">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -4236,25 +4356,25 @@
         <v>31</v>
       </c>
       <c r="B24">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C24">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D24">
-        <v>6.37</v>
+        <v>5.91</v>
       </c>
       <c r="E24">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F24">
-        <v>79.90000000000001</v>
+        <v>81.77</v>
       </c>
       <c r="G24">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H24">
-        <v>13.73</v>
+        <v>12.32</v>
       </c>
       <c r="I24">
         <v>8.1</v>
@@ -4303,19 +4423,19 @@
         <v>0</v>
       </c>
       <c r="E26">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="F26">
-        <v>86.23</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="G26">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H26">
-        <v>13.77</v>
+        <v>2.9</v>
       </c>
       <c r="I26">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -4326,25 +4446,25 @@
         <v>114</v>
       </c>
       <c r="C27">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D27">
-        <v>5.26</v>
+        <v>0</v>
       </c>
       <c r="E27">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F27">
-        <v>91.23</v>
+        <v>92.98</v>
       </c>
       <c r="G27">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H27">
-        <v>3.51</v>
+        <v>7.02</v>
       </c>
       <c r="I27">
-        <v>8.9</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -4355,16 +4475,16 @@
         <v>18</v>
       </c>
       <c r="C28">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D28">
-        <v>77.78</v>
+        <v>0</v>
       </c>
       <c r="E28">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="F28">
-        <v>22.22</v>
+        <v>100</v>
       </c>
       <c r="G28">
         <v>0</v>
@@ -4373,7 +4493,7 @@
         <v>0</v>
       </c>
       <c r="I28">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -4381,25 +4501,25 @@
         <v>36</v>
       </c>
       <c r="B29">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C29">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D29">
-        <v>24.58</v>
+        <v>23.93</v>
       </c>
       <c r="E29">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F29">
-        <v>74.58</v>
+        <v>73.5</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H29">
-        <v>0.85</v>
+        <v>2.56</v>
       </c>
       <c r="I29">
         <v>6.9</v>
@@ -4419,16 +4539,16 @@
         <v>0</v>
       </c>
       <c r="E30">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F30">
-        <v>94.37</v>
+        <v>90.14</v>
       </c>
       <c r="G30">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H30">
-        <v>5.63</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="I30">
         <v>8.800000000000001</v>
@@ -4477,19 +4597,19 @@
         <v>0.54</v>
       </c>
       <c r="E32">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="F32">
-        <v>97.28</v>
+        <v>94.56999999999999</v>
       </c>
       <c r="G32">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H32">
-        <v>2.17</v>
+        <v>4.89</v>
       </c>
       <c r="I32">
-        <v>7.8</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -4497,7 +4617,7 @@
         <v>40</v>
       </c>
       <c r="B33">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C33">
         <v>0</v>
@@ -4506,19 +4626,19 @@
         <v>0</v>
       </c>
       <c r="E33">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="F33">
-        <v>94.67</v>
+        <v>98.23999999999999</v>
       </c>
       <c r="G33">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H33">
-        <v>5.33</v>
+        <v>1.76</v>
       </c>
       <c r="I33">
-        <v>9.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -4526,28 +4646,28 @@
         <v>41</v>
       </c>
       <c r="B34">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C34">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="D34">
-        <v>25.38</v>
+        <v>0</v>
       </c>
       <c r="E34">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F34">
-        <v>74.62</v>
+        <v>76.34</v>
       </c>
       <c r="G34">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="H34">
-        <v>0</v>
+        <v>23.66</v>
       </c>
       <c r="I34">
-        <v>7.8</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -4558,25 +4678,25 @@
         <v>305</v>
       </c>
       <c r="C35">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D35">
-        <v>4.59</v>
+        <v>0</v>
       </c>
       <c r="E35">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="F35">
-        <v>79.02</v>
+        <v>77.38</v>
       </c>
       <c r="G35">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="H35">
-        <v>16.39</v>
+        <v>22.62</v>
       </c>
       <c r="I35">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -4593,19 +4713,19 @@
         <v>6.45</v>
       </c>
       <c r="E36">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="F36">
-        <v>83.33</v>
+        <v>81.18000000000001</v>
       </c>
       <c r="G36">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="H36">
-        <v>10.22</v>
+        <v>12.37</v>
       </c>
       <c r="I36">
-        <v>6.9</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -4613,28 +4733,28 @@
         <v>44</v>
       </c>
       <c r="B37">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C37">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D37">
-        <v>3.98</v>
+        <v>1</v>
       </c>
       <c r="E37">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="F37">
-        <v>96.02</v>
+        <v>94.5</v>
       </c>
       <c r="G37">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="I37">
-        <v>7.9</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -4645,25 +4765,25 @@
         <v>165</v>
       </c>
       <c r="C38">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D38">
-        <v>64.84999999999999</v>
+        <v>62.42</v>
       </c>
       <c r="E38">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="F38">
-        <v>31.52</v>
+        <v>35.15</v>
       </c>
       <c r="G38">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H38">
-        <v>3.64</v>
+        <v>2.42</v>
       </c>
       <c r="I38">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -4671,28 +4791,28 @@
         <v>46</v>
       </c>
       <c r="B39">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C39">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D39">
-        <v>1.39</v>
+        <v>0</v>
       </c>
       <c r="E39">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F39">
-        <v>93.75</v>
+        <v>96.5</v>
       </c>
       <c r="G39">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H39">
-        <v>4.86</v>
+        <v>3.5</v>
       </c>
       <c r="I39">
-        <v>8.699999999999999</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -4709,19 +4829,19 @@
         <v>1.52</v>
       </c>
       <c r="E40">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F40">
-        <v>96.97</v>
+        <v>92.42</v>
       </c>
       <c r="G40">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H40">
-        <v>1.52</v>
+        <v>6.06</v>
       </c>
       <c r="I40">
-        <v>8.6</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -4738,19 +4858,19 @@
         <v>7.94</v>
       </c>
       <c r="E41">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F41">
-        <v>84.13</v>
+        <v>85.70999999999999</v>
       </c>
       <c r="G41">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H41">
-        <v>7.94</v>
+        <v>6.35</v>
       </c>
       <c r="I41">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -4758,28 +4878,28 @@
         <v>49</v>
       </c>
       <c r="B42">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C42">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D42">
-        <v>13.89</v>
+        <v>0</v>
       </c>
       <c r="E42">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F42">
-        <v>65.97</v>
+        <v>59.44</v>
       </c>
       <c r="G42">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="H42">
-        <v>20.14</v>
+        <v>40.56</v>
       </c>
       <c r="I42">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -4787,7 +4907,7 @@
         <v>50</v>
       </c>
       <c r="B43">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C43">
         <v>0</v>
@@ -4796,19 +4916,19 @@
         <v>0</v>
       </c>
       <c r="E43">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F43">
-        <v>98.42</v>
+        <v>97.38</v>
       </c>
       <c r="G43">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H43">
-        <v>1.58</v>
+        <v>2.62</v>
       </c>
       <c r="I43">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -4866,7 +4986,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -4874,7 +4994,7 @@
         <v>53</v>
       </c>
       <c r="B46">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C46">
         <v>0</v>
@@ -4886,16 +5006,16 @@
         <v>49</v>
       </c>
       <c r="F46">
-        <v>75.38</v>
+        <v>74.23999999999999</v>
       </c>
       <c r="G46">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H46">
-        <v>24.62</v>
+        <v>25.76</v>
       </c>
       <c r="I46">
-        <v>6.9</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -4924,7 +5044,7 @@
         <v>0</v>
       </c>
       <c r="I47">
-        <v>8.4</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -4941,19 +5061,19 @@
         <v>0</v>
       </c>
       <c r="E48">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F48">
-        <v>81.25</v>
+        <v>82.81</v>
       </c>
       <c r="G48">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H48">
-        <v>18.75</v>
+        <v>17.19</v>
       </c>
       <c r="I48">
-        <v>6.9</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -4961,25 +5081,25 @@
         <v>56</v>
       </c>
       <c r="B49">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D49">
-        <v>3.23</v>
+        <v>0</v>
       </c>
       <c r="E49">
         <v>23</v>
       </c>
       <c r="F49">
-        <v>74.19</v>
+        <v>76.67</v>
       </c>
       <c r="G49">
         <v>7</v>
       </c>
       <c r="H49">
-        <v>22.58</v>
+        <v>23.33</v>
       </c>
       <c r="I49">
         <v>7.8</v>
@@ -4990,28 +5110,28 @@
         <v>57</v>
       </c>
       <c r="B50">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C50">
         <v>12</v>
       </c>
       <c r="D50">
-        <v>5.5</v>
+        <v>5.56</v>
       </c>
       <c r="E50">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F50">
-        <v>85.31999999999999</v>
+        <v>85.65000000000001</v>
       </c>
       <c r="G50">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H50">
-        <v>9.17</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I50">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -5019,25 +5139,25 @@
         <v>58</v>
       </c>
       <c r="B51">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C51">
         <v>16</v>
       </c>
       <c r="D51">
-        <v>8.289999999999999</v>
+        <v>8.33</v>
       </c>
       <c r="E51">
         <v>140</v>
       </c>
       <c r="F51">
-        <v>72.54000000000001</v>
+        <v>72.92</v>
       </c>
       <c r="G51">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H51">
-        <v>19.17</v>
+        <v>18.75</v>
       </c>
       <c r="I51">
         <v>6.4</v>
@@ -5048,28 +5168,28 @@
         <v>59</v>
       </c>
       <c r="B52">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C52">
         <v>7</v>
       </c>
       <c r="D52">
-        <v>5.11</v>
+        <v>5.07</v>
       </c>
       <c r="E52">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="F52">
-        <v>85.40000000000001</v>
+        <v>89.86</v>
       </c>
       <c r="G52">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="H52">
-        <v>9.49</v>
+        <v>5.07</v>
       </c>
       <c r="I52">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -5098,7 +5218,7 @@
         <v>0</v>
       </c>
       <c r="I53">
-        <v>8.4</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -5115,19 +5235,19 @@
         <v>0</v>
       </c>
       <c r="E54">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F54">
-        <v>94.92</v>
+        <v>95.76000000000001</v>
       </c>
       <c r="G54">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H54">
-        <v>5.08</v>
+        <v>4.24</v>
       </c>
       <c r="I54">
-        <v>7.8</v>
+        <v>8.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Primer Parcial 15-Mar Noche
</commit_message>
<xml_diff>
--- a/Totales Docentes.xlsx
+++ b/Totales Docentes.xlsx
@@ -678,25 +678,25 @@
         <v>3561</v>
       </c>
       <c r="C7">
-        <v>1604</v>
+        <v>435</v>
       </c>
       <c r="D7">
-        <v>45.04</v>
+        <v>12.22</v>
       </c>
       <c r="E7">
-        <v>1635</v>
+        <v>2629</v>
       </c>
       <c r="F7">
-        <v>45.91</v>
+        <v>73.83</v>
       </c>
       <c r="G7">
-        <v>306</v>
+        <v>481</v>
       </c>
       <c r="H7">
-        <v>8.59</v>
+        <v>13.51</v>
       </c>
       <c r="I7">
-        <v>7.9</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -820,22 +820,25 @@
         <v>62</v>
       </c>
       <c r="C12">
-        <v>62</v>
+        <v>1</v>
       </c>
       <c r="D12">
-        <v>100</v>
+        <v>1.61</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>80.65000000000001</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>17.74</v>
+      </c>
+      <c r="I12">
+        <v>7.1</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -933,25 +936,25 @@
         <v>133</v>
       </c>
       <c r="C16">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="D16">
-        <v>50.38</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>66</v>
+        <v>125</v>
       </c>
       <c r="F16">
-        <v>49.62</v>
+        <v>93.98</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H16">
-        <v>0</v>
+        <v>6.02</v>
       </c>
       <c r="I16">
-        <v>9.300000000000001</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -991,10 +994,10 @@
         <v>104</v>
       </c>
       <c r="C18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D18">
-        <v>6.73</v>
+        <v>0</v>
       </c>
       <c r="E18">
         <v>83</v>
@@ -1003,13 +1006,13 @@
         <v>79.81</v>
       </c>
       <c r="G18">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="H18">
-        <v>13.46</v>
+        <v>20.19</v>
       </c>
       <c r="I18">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -1078,25 +1081,25 @@
         <v>180</v>
       </c>
       <c r="C21">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D21">
-        <v>11.11</v>
+        <v>0</v>
       </c>
       <c r="E21">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="F21">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G21">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H21">
-        <v>8.890000000000001</v>
+        <v>10</v>
       </c>
       <c r="I21">
-        <v>8</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -1165,22 +1168,25 @@
         <v>113</v>
       </c>
       <c r="C24">
-        <v>113</v>
+        <v>43</v>
       </c>
       <c r="D24">
-        <v>100</v>
+        <v>38.05</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>52.21</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>9.73</v>
+      </c>
+      <c r="I24">
+        <v>7.9</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1249,22 +1255,25 @@
         <v>33</v>
       </c>
       <c r="C27">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="D27">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>93.94</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H27">
-        <v>0</v>
+        <v>6.06</v>
+      </c>
+      <c r="I27">
+        <v>8.4</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1569,10 +1578,10 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <v>1941</v>
+        <v>3110</v>
       </c>
       <c r="H7">
-        <v>54.51</v>
+        <v>87.34</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1699,10 +1708,10 @@
         <v>0</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>98.39</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1803,10 +1812,10 @@
         <v>0</v>
       </c>
       <c r="G16">
-        <v>66</v>
+        <v>133</v>
       </c>
       <c r="H16">
-        <v>49.62</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1855,10 +1864,10 @@
         <v>0</v>
       </c>
       <c r="G18">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="H18">
-        <v>93.27</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1933,10 +1942,10 @@
         <v>0</v>
       </c>
       <c r="G21">
-        <v>160</v>
+        <v>180</v>
       </c>
       <c r="H21">
-        <v>88.89</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -2011,10 +2020,10 @@
         <v>0</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>61.95</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -2089,10 +2098,10 @@
         <v>0</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="H27">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -2394,25 +2403,25 @@
         <v>3561</v>
       </c>
       <c r="C7">
-        <v>1604</v>
+        <v>435</v>
       </c>
       <c r="D7">
-        <v>45.04</v>
+        <v>12.22</v>
       </c>
       <c r="E7">
-        <v>1635</v>
+        <v>2629</v>
       </c>
       <c r="F7">
-        <v>45.91</v>
+        <v>73.83</v>
       </c>
       <c r="G7">
-        <v>322</v>
+        <v>497</v>
       </c>
       <c r="H7">
-        <v>9.039999999999999</v>
+        <v>13.96</v>
       </c>
       <c r="I7">
-        <v>7.9</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2536,22 +2545,25 @@
         <v>62</v>
       </c>
       <c r="C12">
-        <v>62</v>
+        <v>1</v>
       </c>
       <c r="D12">
-        <v>100</v>
+        <v>1.61</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>80.65000000000001</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>17.74</v>
+      </c>
+      <c r="I12">
+        <v>7.1</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -2649,25 +2661,25 @@
         <v>133</v>
       </c>
       <c r="C16">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="D16">
-        <v>50.38</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>66</v>
+        <v>125</v>
       </c>
       <c r="F16">
-        <v>49.62</v>
+        <v>93.98</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H16">
-        <v>0</v>
+        <v>6.02</v>
       </c>
       <c r="I16">
-        <v>9.300000000000001</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -2707,10 +2719,10 @@
         <v>104</v>
       </c>
       <c r="C18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D18">
-        <v>6.73</v>
+        <v>0</v>
       </c>
       <c r="E18">
         <v>83</v>
@@ -2719,13 +2731,13 @@
         <v>79.81</v>
       </c>
       <c r="G18">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="H18">
-        <v>13.46</v>
+        <v>20.19</v>
       </c>
       <c r="I18">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -2794,25 +2806,25 @@
         <v>180</v>
       </c>
       <c r="C21">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D21">
-        <v>11.11</v>
+        <v>0</v>
       </c>
       <c r="E21">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="F21">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G21">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H21">
-        <v>8.890000000000001</v>
+        <v>10</v>
       </c>
       <c r="I21">
-        <v>8</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -2881,22 +2893,25 @@
         <v>113</v>
       </c>
       <c r="C24">
-        <v>113</v>
+        <v>43</v>
       </c>
       <c r="D24">
-        <v>100</v>
+        <v>38.05</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>52.21</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>9.73</v>
+      </c>
+      <c r="I24">
+        <v>7.9</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -2965,22 +2980,25 @@
         <v>33</v>
       </c>
       <c r="C27">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="D27">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>93.94</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H27">
-        <v>0</v>
+        <v>6.06</v>
+      </c>
+      <c r="I27">
+        <v>8.4</v>
       </c>
     </row>
     <row r="28" spans="1:9">

</xml_diff>

<commit_message>
Primer Parcial con Nombres
</commit_message>
<xml_diff>
--- a/Totales Docentes.xlsx
+++ b/Totales Docentes.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="60">
   <si>
     <t>Docente</t>
   </si>
@@ -48,21 +48,33 @@
     <t>Acevedo Rendón Ismael Arturo</t>
   </si>
   <si>
+    <t>Avila Coronado Julieta</t>
+  </si>
+  <si>
+    <t>Barañon Samaniego Graciela de los Ángeles</t>
+  </si>
+  <si>
+    <t>Caballero Rosas María Teresa</t>
+  </si>
+  <si>
     <t>Camacho Juárez Sergio Eduardo</t>
   </si>
   <si>
     <t>Castillo Cruz Carlos Samuel</t>
   </si>
   <si>
+    <t>Castro Vasquez Julieta</t>
+  </si>
+  <si>
     <t>Contreras Díaz Irma Ivette</t>
   </si>
   <si>
+    <t>Cruz Alejo José Armando</t>
+  </si>
+  <si>
     <t>De Jesús Orduña Sofía del Pilar</t>
   </si>
   <si>
-    <t>Desc Desc Desc</t>
-  </si>
-  <si>
     <t>Domínguez Burgos Marioscar</t>
   </si>
   <si>
@@ -72,33 +84,63 @@
     <t>Flores Ovalle Victor</t>
   </si>
   <si>
+    <t>Garcia Felix Jose Antonio</t>
+  </si>
+  <si>
+    <t>García Sánchez Magda Bexabe</t>
+  </si>
+  <si>
     <t>Gaspar Velazco Juan Francisco</t>
   </si>
   <si>
     <t>Gomez Lopez Javier</t>
   </si>
   <si>
+    <t>González Altamirano Victorino Juventino</t>
+  </si>
+  <si>
     <t>González Nuñez Veronica</t>
   </si>
   <si>
+    <t>González Sánchez Rene Aurelio</t>
+  </si>
+  <si>
+    <t>Hernández Contreras Ángel</t>
+  </si>
+  <si>
     <t>Hernández Mendoza Delfina</t>
   </si>
   <si>
     <t>Herrera Serrano Mayra Iliana</t>
   </si>
   <si>
+    <t>Jiménez Nieto Enrique</t>
+  </si>
+  <si>
     <t>Martínez Castillo Columba</t>
   </si>
   <si>
     <t>Martínez López Miguel Ángel</t>
   </si>
   <si>
+    <t>Mateos Sanchez Jorge</t>
+  </si>
+  <si>
+    <t>Medina Tolentino Elio</t>
+  </si>
+  <si>
     <t>Medina Tolentino Francisco</t>
   </si>
   <si>
+    <t>Mendoza Velazquez Laura Elena</t>
+  </si>
+  <si>
     <t>Molina Quezada Raúl</t>
   </si>
   <si>
+    <t>Moreno Aroyo Anél</t>
+  </si>
+  <si>
     <t>Muñoz Rivadeneyra Salvador</t>
   </si>
   <si>
@@ -111,12 +153,21 @@
     <t>Polanco Domínguez Rosa María</t>
   </si>
   <si>
+    <t>Rivera Cruz Ezequiel</t>
+  </si>
+  <si>
     <t>Rivera Serra Alma Lilian</t>
   </si>
   <si>
     <t>Rodriguez Roman Marisol</t>
   </si>
   <si>
+    <t>Rodríguez Román Leticia</t>
+  </si>
+  <si>
+    <t>Rosas Aguilar Claudia Leonor</t>
+  </si>
+  <si>
     <t>Santiago Hernández Mariana</t>
   </si>
   <si>
@@ -129,10 +180,22 @@
     <t>Sánchez Sánchez Miguel</t>
   </si>
   <si>
+    <t>Torres Sánchez José Luis</t>
+  </si>
+  <si>
+    <t>Vargas Olvera Francisco Eduardo</t>
+  </si>
+  <si>
+    <t>Velasco Sánchez David</t>
+  </si>
+  <si>
     <t>Villanueva Morales Luis Arturo</t>
   </si>
   <si>
     <t>Zarate Amezcua Eladio Jorge</t>
+  </si>
+  <si>
+    <t>Ángel Martínez Gerson Hermenegildo</t>
   </si>
 </sst>
 </file>
@@ -490,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="50.7109375" customWidth="1"/>
@@ -559,28 +622,28 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>130</v>
+        <v>207</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>0.77</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>119</v>
+        <v>151</v>
       </c>
       <c r="F3">
-        <v>91.54000000000001</v>
+        <v>72.95</v>
       </c>
       <c r="G3">
-        <v>10</v>
+        <v>56</v>
       </c>
       <c r="H3">
-        <v>7.69</v>
+        <v>27.05</v>
       </c>
       <c r="I3">
-        <v>8.5</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -588,7 +651,7 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -597,19 +660,19 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="F4">
-        <v>100</v>
+        <v>78.56999999999999</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="I4">
-        <v>8.6</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -617,7 +680,7 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -626,19 +689,19 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="F5">
-        <v>75</v>
+        <v>86.83</v>
       </c>
       <c r="G5">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="H5">
-        <v>25</v>
+        <v>13.17</v>
       </c>
       <c r="I5">
-        <v>6.9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -646,28 +709,28 @@
         <v>13</v>
       </c>
       <c r="B6">
-        <v>94</v>
+        <v>130</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="E6">
-        <v>77</v>
+        <v>119</v>
       </c>
       <c r="F6">
-        <v>81.91</v>
+        <v>91.54000000000001</v>
       </c>
       <c r="G6">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="H6">
-        <v>18.09</v>
+        <v>7.69</v>
       </c>
       <c r="I6">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -675,28 +738,28 @@
         <v>14</v>
       </c>
       <c r="B7">
-        <v>3563</v>
+        <v>19</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>3026</v>
+        <v>19</v>
       </c>
       <c r="F7">
-        <v>84.93000000000001</v>
+        <v>100</v>
       </c>
       <c r="G7">
-        <v>519</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>14.57</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>7.6</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -704,28 +767,28 @@
         <v>15</v>
       </c>
       <c r="B8">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>85</v>
+        <v>110</v>
       </c>
       <c r="F8">
-        <v>71.43000000000001</v>
+        <v>96.48999999999999</v>
       </c>
       <c r="G8">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="H8">
-        <v>27.73</v>
+        <v>3.51</v>
       </c>
       <c r="I8">
-        <v>6.9</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -733,7 +796,7 @@
         <v>16</v>
       </c>
       <c r="B9">
-        <v>36</v>
+        <v>168</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -742,19 +805,19 @@
         <v>0</v>
       </c>
       <c r="E9">
-        <v>18</v>
+        <v>126</v>
       </c>
       <c r="F9">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="G9">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="H9">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="I9">
-        <v>6</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -762,7 +825,7 @@
         <v>17</v>
       </c>
       <c r="B10">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -771,19 +834,19 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="F10">
-        <v>75.36</v>
+        <v>100</v>
       </c>
       <c r="G10">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>24.64</v>
+        <v>0</v>
       </c>
       <c r="I10">
-        <v>7</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -800,19 +863,19 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="F11">
-        <v>56.38</v>
+        <v>81.91</v>
       </c>
       <c r="G11">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="H11">
-        <v>43.62</v>
+        <v>18.09</v>
       </c>
       <c r="I11">
-        <v>5.9</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -820,28 +883,28 @@
         <v>19</v>
       </c>
       <c r="B12">
-        <v>64</v>
+        <v>119</v>
       </c>
       <c r="C12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12">
-        <v>3.13</v>
+        <v>0.84</v>
       </c>
       <c r="E12">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="F12">
-        <v>78.13</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="G12">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="H12">
-        <v>18.75</v>
+        <v>27.73</v>
       </c>
       <c r="I12">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -849,28 +912,28 @@
         <v>20</v>
       </c>
       <c r="B13">
-        <v>163</v>
+        <v>135</v>
       </c>
       <c r="C13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D13">
-        <v>1.23</v>
+        <v>0</v>
       </c>
       <c r="E13">
-        <v>131</v>
+        <v>57</v>
       </c>
       <c r="F13">
-        <v>80.37</v>
+        <v>42.22</v>
       </c>
       <c r="G13">
-        <v>23</v>
+        <v>78</v>
       </c>
       <c r="H13">
-        <v>14.11</v>
+        <v>57.78</v>
       </c>
       <c r="I13">
-        <v>7.3</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -878,7 +941,7 @@
         <v>21</v>
       </c>
       <c r="B14">
-        <v>129</v>
+        <v>69</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -887,19 +950,19 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>96</v>
+        <v>52</v>
       </c>
       <c r="F14">
-        <v>74.42</v>
+        <v>75.36</v>
       </c>
       <c r="G14">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="H14">
-        <v>25.58</v>
+        <v>24.64</v>
       </c>
       <c r="I14">
-        <v>7.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -907,7 +970,7 @@
         <v>22</v>
       </c>
       <c r="B15">
-        <v>87</v>
+        <v>166</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -916,19 +979,19 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>68</v>
+        <v>133</v>
       </c>
       <c r="F15">
-        <v>78.16</v>
+        <v>80.12</v>
       </c>
       <c r="G15">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H15">
-        <v>21.84</v>
+        <v>18.67</v>
       </c>
       <c r="I15">
-        <v>7</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -936,7 +999,7 @@
         <v>23</v>
       </c>
       <c r="B16">
-        <v>133</v>
+        <v>277</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -945,19 +1008,19 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>125</v>
+        <v>247</v>
       </c>
       <c r="F16">
-        <v>93.98</v>
+        <v>89.17</v>
       </c>
       <c r="G16">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="H16">
-        <v>6.02</v>
+        <v>10.83</v>
       </c>
       <c r="I16">
-        <v>8.699999999999999</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -965,7 +1028,7 @@
         <v>24</v>
       </c>
       <c r="B17">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -974,19 +1037,19 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F17">
-        <v>85.25</v>
+        <v>56.38</v>
       </c>
       <c r="G17">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="H17">
-        <v>14.75</v>
+        <v>43.62</v>
       </c>
       <c r="I17">
-        <v>7.6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -994,25 +1057,25 @@
         <v>25</v>
       </c>
       <c r="B18">
-        <v>104</v>
+        <v>64</v>
       </c>
       <c r="C18">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>3.13</v>
       </c>
       <c r="E18">
-        <v>83</v>
+        <v>50</v>
       </c>
       <c r="F18">
-        <v>79.81</v>
+        <v>78.13</v>
       </c>
       <c r="G18">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="H18">
-        <v>20.19</v>
+        <v>18.75</v>
       </c>
       <c r="I18">
         <v>7.1</v>
@@ -1023,7 +1086,7 @@
         <v>26</v>
       </c>
       <c r="B19">
-        <v>132</v>
+        <v>248</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -1032,19 +1095,19 @@
         <v>0</v>
       </c>
       <c r="E19">
-        <v>132</v>
+        <v>167</v>
       </c>
       <c r="F19">
-        <v>100</v>
+        <v>67.34</v>
       </c>
       <c r="G19">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="H19">
-        <v>0</v>
+        <v>32.66</v>
       </c>
       <c r="I19">
-        <v>8.800000000000001</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1052,28 +1115,28 @@
         <v>27</v>
       </c>
       <c r="B20">
-        <v>114</v>
+        <v>163</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20">
-        <v>0.88</v>
+        <v>1.23</v>
       </c>
       <c r="E20">
-        <v>89</v>
+        <v>131</v>
       </c>
       <c r="F20">
-        <v>78.06999999999999</v>
+        <v>80.37</v>
       </c>
       <c r="G20">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H20">
-        <v>19.3</v>
+        <v>14.11</v>
       </c>
       <c r="I20">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -1081,28 +1144,28 @@
         <v>28</v>
       </c>
       <c r="B21">
-        <v>180</v>
+        <v>208</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>0.48</v>
       </c>
       <c r="E21">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="F21">
-        <v>90</v>
+        <v>86.06</v>
       </c>
       <c r="G21">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H21">
-        <v>10</v>
+        <v>13.46</v>
       </c>
       <c r="I21">
-        <v>7.9</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -1110,7 +1173,7 @@
         <v>29</v>
       </c>
       <c r="B22">
-        <v>226</v>
+        <v>62</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -1119,19 +1182,19 @@
         <v>0</v>
       </c>
       <c r="E22">
-        <v>194</v>
+        <v>59</v>
       </c>
       <c r="F22">
-        <v>85.84</v>
+        <v>95.16</v>
       </c>
       <c r="G22">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="H22">
-        <v>14.16</v>
+        <v>4.84</v>
       </c>
       <c r="I22">
-        <v>7</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -1139,28 +1202,28 @@
         <v>30</v>
       </c>
       <c r="B23">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="C23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D23">
-        <v>0.72</v>
+        <v>0</v>
       </c>
       <c r="E23">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="F23">
-        <v>65.22</v>
+        <v>63.71</v>
       </c>
       <c r="G23">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H23">
-        <v>34.06</v>
+        <v>36.29</v>
       </c>
       <c r="I23">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1168,28 +1231,28 @@
         <v>31</v>
       </c>
       <c r="B24">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="C24">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D24">
-        <v>1.74</v>
+        <v>0</v>
       </c>
       <c r="E24">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="F24">
-        <v>77.39</v>
+        <v>78.16</v>
       </c>
       <c r="G24">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="H24">
-        <v>20.87</v>
+        <v>21.84</v>
       </c>
       <c r="I24">
-        <v>7.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1197,7 +1260,7 @@
         <v>32</v>
       </c>
       <c r="B25">
-        <v>115</v>
+        <v>180</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -1206,19 +1269,19 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>100</v>
+        <v>152</v>
       </c>
       <c r="F25">
-        <v>86.95999999999999</v>
+        <v>84.44</v>
       </c>
       <c r="G25">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H25">
-        <v>13.04</v>
+        <v>15.56</v>
       </c>
       <c r="I25">
-        <v>8</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -1226,7 +1289,7 @@
         <v>33</v>
       </c>
       <c r="B26">
-        <v>17</v>
+        <v>133</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -1235,19 +1298,19 @@
         <v>0</v>
       </c>
       <c r="E26">
-        <v>17</v>
+        <v>125</v>
       </c>
       <c r="F26">
-        <v>100</v>
+        <v>93.98</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H26">
-        <v>0</v>
+        <v>6.02</v>
       </c>
       <c r="I26">
-        <v>9.199999999999999</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1255,7 +1318,7 @@
         <v>34</v>
       </c>
       <c r="B27">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -1264,19 +1327,19 @@
         <v>0</v>
       </c>
       <c r="E27">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="F27">
-        <v>93.94</v>
+        <v>85.25</v>
       </c>
       <c r="G27">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H27">
-        <v>6.06</v>
+        <v>14.75</v>
       </c>
       <c r="I27">
-        <v>8.4</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1284,28 +1347,28 @@
         <v>35</v>
       </c>
       <c r="B28">
-        <v>77</v>
+        <v>186</v>
       </c>
       <c r="C28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28">
-        <v>0</v>
+        <v>0.54</v>
       </c>
       <c r="E28">
-        <v>58</v>
+        <v>163</v>
       </c>
       <c r="F28">
-        <v>75.31999999999999</v>
+        <v>87.63</v>
       </c>
       <c r="G28">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="H28">
-        <v>24.68</v>
+        <v>4.3</v>
       </c>
       <c r="I28">
-        <v>6.4</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1313,7 +1376,7 @@
         <v>36</v>
       </c>
       <c r="B29">
-        <v>63</v>
+        <v>177</v>
       </c>
       <c r="C29">
         <v>0</v>
@@ -1322,19 +1385,19 @@
         <v>0</v>
       </c>
       <c r="E29">
-        <v>62</v>
+        <v>177</v>
       </c>
       <c r="F29">
-        <v>98.41</v>
+        <v>100</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29">
-        <v>1.59</v>
+        <v>0</v>
       </c>
       <c r="I29">
-        <v>8.199999999999999</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -1342,7 +1405,7 @@
         <v>37</v>
       </c>
       <c r="B30">
-        <v>151</v>
+        <v>104</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -1351,19 +1414,19 @@
         <v>0</v>
       </c>
       <c r="E30">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="F30">
-        <v>45.7</v>
+        <v>79.81</v>
       </c>
       <c r="G30">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="H30">
-        <v>53.64</v>
+        <v>20.19</v>
       </c>
       <c r="I30">
-        <v>5.7</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -1371,28 +1434,637 @@
         <v>38</v>
       </c>
       <c r="B31">
+        <v>111</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>96</v>
+      </c>
+      <c r="F31">
+        <v>86.48999999999999</v>
+      </c>
+      <c r="G31">
+        <v>15</v>
+      </c>
+      <c r="H31">
+        <v>13.51</v>
+      </c>
+      <c r="I31">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32">
+        <v>132</v>
+      </c>
+      <c r="C32">
+        <v>0</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32">
+        <v>132</v>
+      </c>
+      <c r="F32">
+        <v>100</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
+      </c>
+      <c r="I32">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33">
+        <v>159</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33">
+        <v>140</v>
+      </c>
+      <c r="F33">
+        <v>88.05</v>
+      </c>
+      <c r="G33">
+        <v>19</v>
+      </c>
+      <c r="H33">
+        <v>11.95</v>
+      </c>
+      <c r="I33">
+        <v>8.300000000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" t="s">
+        <v>41</v>
+      </c>
+      <c r="B34">
+        <v>114</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="D34">
+        <v>0.88</v>
+      </c>
+      <c r="E34">
+        <v>89</v>
+      </c>
+      <c r="F34">
+        <v>78.06999999999999</v>
+      </c>
+      <c r="G34">
+        <v>22</v>
+      </c>
+      <c r="H34">
+        <v>19.3</v>
+      </c>
+      <c r="I34">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" t="s">
+        <v>42</v>
+      </c>
+      <c r="B35">
+        <v>180</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>162</v>
+      </c>
+      <c r="F35">
+        <v>90</v>
+      </c>
+      <c r="G35">
+        <v>18</v>
+      </c>
+      <c r="H35">
+        <v>10</v>
+      </c>
+      <c r="I35">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" t="s">
+        <v>43</v>
+      </c>
+      <c r="B36">
+        <v>226</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36">
+        <v>194</v>
+      </c>
+      <c r="F36">
+        <v>85.84</v>
+      </c>
+      <c r="G36">
+        <v>32</v>
+      </c>
+      <c r="H36">
+        <v>14.16</v>
+      </c>
+      <c r="I36">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" t="s">
+        <v>44</v>
+      </c>
+      <c r="B37">
+        <v>138</v>
+      </c>
+      <c r="C37">
+        <v>1</v>
+      </c>
+      <c r="D37">
+        <v>0.72</v>
+      </c>
+      <c r="E37">
+        <v>90</v>
+      </c>
+      <c r="F37">
+        <v>65.22</v>
+      </c>
+      <c r="G37">
+        <v>47</v>
+      </c>
+      <c r="H37">
+        <v>34.06</v>
+      </c>
+      <c r="I37">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" t="s">
+        <v>45</v>
+      </c>
+      <c r="B38">
+        <v>125</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>110</v>
+      </c>
+      <c r="F38">
+        <v>88</v>
+      </c>
+      <c r="G38">
+        <v>15</v>
+      </c>
+      <c r="H38">
+        <v>12</v>
+      </c>
+      <c r="I38">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" t="s">
+        <v>46</v>
+      </c>
+      <c r="B39">
+        <v>115</v>
+      </c>
+      <c r="C39">
+        <v>2</v>
+      </c>
+      <c r="D39">
+        <v>1.74</v>
+      </c>
+      <c r="E39">
+        <v>89</v>
+      </c>
+      <c r="F39">
+        <v>77.39</v>
+      </c>
+      <c r="G39">
+        <v>24</v>
+      </c>
+      <c r="H39">
+        <v>20.87</v>
+      </c>
+      <c r="I39">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" t="s">
+        <v>47</v>
+      </c>
+      <c r="B40">
+        <v>115</v>
+      </c>
+      <c r="C40">
+        <v>0</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40">
+        <v>100</v>
+      </c>
+      <c r="F40">
+        <v>86.95999999999999</v>
+      </c>
+      <c r="G40">
+        <v>15</v>
+      </c>
+      <c r="H40">
+        <v>13.04</v>
+      </c>
+      <c r="I40">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" t="s">
+        <v>48</v>
+      </c>
+      <c r="B41">
+        <v>158</v>
+      </c>
+      <c r="C41">
+        <v>0</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>134</v>
+      </c>
+      <c r="F41">
+        <v>84.81</v>
+      </c>
+      <c r="G41">
+        <v>24</v>
+      </c>
+      <c r="H41">
+        <v>15.19</v>
+      </c>
+      <c r="I41">
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" t="s">
+        <v>49</v>
+      </c>
+      <c r="B42">
+        <v>234</v>
+      </c>
+      <c r="C42">
+        <v>0</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>220</v>
+      </c>
+      <c r="F42">
+        <v>94.02</v>
+      </c>
+      <c r="G42">
+        <v>14</v>
+      </c>
+      <c r="H42">
+        <v>5.98</v>
+      </c>
+      <c r="I42">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" t="s">
+        <v>50</v>
+      </c>
+      <c r="B43">
+        <v>17</v>
+      </c>
+      <c r="C43">
+        <v>0</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="E43">
+        <v>17</v>
+      </c>
+      <c r="F43">
+        <v>100</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+      <c r="H43">
+        <v>0</v>
+      </c>
+      <c r="I43">
+        <v>9.199999999999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" t="s">
+        <v>51</v>
+      </c>
+      <c r="B44">
+        <v>33</v>
+      </c>
+      <c r="C44">
+        <v>0</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>31</v>
+      </c>
+      <c r="F44">
+        <v>93.94</v>
+      </c>
+      <c r="G44">
+        <v>2</v>
+      </c>
+      <c r="H44">
+        <v>6.06</v>
+      </c>
+      <c r="I44">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" t="s">
+        <v>52</v>
+      </c>
+      <c r="B45">
+        <v>77</v>
+      </c>
+      <c r="C45">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45">
+        <v>58</v>
+      </c>
+      <c r="F45">
+        <v>75.31999999999999</v>
+      </c>
+      <c r="G45">
+        <v>19</v>
+      </c>
+      <c r="H45">
+        <v>24.68</v>
+      </c>
+      <c r="I45">
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" t="s">
+        <v>53</v>
+      </c>
+      <c r="B46">
+        <v>63</v>
+      </c>
+      <c r="C46">
+        <v>0</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46">
+        <v>62</v>
+      </c>
+      <c r="F46">
+        <v>98.41</v>
+      </c>
+      <c r="G46">
+        <v>1</v>
+      </c>
+      <c r="H46">
+        <v>1.59</v>
+      </c>
+      <c r="I46">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" t="s">
+        <v>54</v>
+      </c>
+      <c r="B47">
+        <v>91</v>
+      </c>
+      <c r="C47">
+        <v>0</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47">
+        <v>78</v>
+      </c>
+      <c r="F47">
+        <v>85.70999999999999</v>
+      </c>
+      <c r="G47">
+        <v>13</v>
+      </c>
+      <c r="H47">
+        <v>14.29</v>
+      </c>
+      <c r="I47">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" t="s">
+        <v>55</v>
+      </c>
+      <c r="B48">
+        <v>123</v>
+      </c>
+      <c r="C48">
+        <v>0</v>
+      </c>
+      <c r="D48">
+        <v>0</v>
+      </c>
+      <c r="E48">
+        <v>113</v>
+      </c>
+      <c r="F48">
+        <v>91.87</v>
+      </c>
+      <c r="G48">
+        <v>10</v>
+      </c>
+      <c r="H48">
+        <v>8.130000000000001</v>
+      </c>
+      <c r="I48">
+        <v>8.699999999999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" t="s">
+        <v>56</v>
+      </c>
+      <c r="B49">
+        <v>172</v>
+      </c>
+      <c r="C49">
+        <v>0</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+      <c r="E49">
+        <v>141</v>
+      </c>
+      <c r="F49">
+        <v>81.98</v>
+      </c>
+      <c r="G49">
+        <v>31</v>
+      </c>
+      <c r="H49">
+        <v>18.02</v>
+      </c>
+      <c r="I49">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" t="s">
+        <v>57</v>
+      </c>
+      <c r="B50">
+        <v>151</v>
+      </c>
+      <c r="C50">
+        <v>0</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50">
+        <v>69</v>
+      </c>
+      <c r="F50">
+        <v>45.7</v>
+      </c>
+      <c r="G50">
+        <v>81</v>
+      </c>
+      <c r="H50">
+        <v>53.64</v>
+      </c>
+      <c r="I50">
+        <v>5.7</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9">
+      <c r="A51" t="s">
+        <v>58</v>
+      </c>
+      <c r="B51">
         <v>103</v>
       </c>
-      <c r="C31">
-        <v>0</v>
-      </c>
-      <c r="D31">
-        <v>0</v>
-      </c>
-      <c r="E31">
+      <c r="C51">
+        <v>0</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51">
         <v>66</v>
       </c>
-      <c r="F31">
+      <c r="F51">
         <v>64.08</v>
       </c>
-      <c r="G31">
+      <c r="G51">
         <v>37</v>
       </c>
-      <c r="H31">
+      <c r="H51">
         <v>35.92</v>
       </c>
-      <c r="I31">
+      <c r="I51">
         <v>6.8</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52">
+        <v>174</v>
+      </c>
+      <c r="C52">
+        <v>0</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52">
+        <v>174</v>
+      </c>
+      <c r="F52">
+        <v>100</v>
+      </c>
+      <c r="G52">
+        <v>0</v>
+      </c>
+      <c r="H52">
+        <v>0</v>
+      </c>
+      <c r="I52">
+        <v>9.1</v>
       </c>
     </row>
   </sheetData>
@@ -1402,7 +2074,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="50.7109375" customWidth="1"/>
@@ -1468,10 +2140,10 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>130</v>
+        <v>207</v>
       </c>
       <c r="C3">
-        <v>130</v>
+        <v>207</v>
       </c>
       <c r="D3">
         <v>100</v>
@@ -1483,10 +2155,10 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>129</v>
+        <v>207</v>
       </c>
       <c r="H3">
-        <v>99.23</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1494,10 +2166,10 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="C4">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="D4">
         <v>100</v>
@@ -1509,7 +2181,7 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="H4">
         <v>100</v>
@@ -1520,10 +2192,10 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C5">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D5">
         <v>100</v>
@@ -1535,7 +2207,7 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H5">
         <v>100</v>
@@ -1546,10 +2218,10 @@
         <v>13</v>
       </c>
       <c r="B6">
-        <v>94</v>
+        <v>130</v>
       </c>
       <c r="C6">
-        <v>94</v>
+        <v>130</v>
       </c>
       <c r="D6">
         <v>100</v>
@@ -1561,10 +2233,10 @@
         <v>0</v>
       </c>
       <c r="G6">
-        <v>94</v>
+        <v>129</v>
       </c>
       <c r="H6">
-        <v>100</v>
+        <v>99.23</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1572,10 +2244,10 @@
         <v>14</v>
       </c>
       <c r="B7">
-        <v>3563</v>
+        <v>19</v>
       </c>
       <c r="C7">
-        <v>3563</v>
+        <v>19</v>
       </c>
       <c r="D7">
         <v>100</v>
@@ -1587,10 +2259,10 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <v>3545</v>
+        <v>19</v>
       </c>
       <c r="H7">
-        <v>99.48999999999999</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1598,10 +2270,10 @@
         <v>15</v>
       </c>
       <c r="B8">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C8">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D8">
         <v>100</v>
@@ -1613,10 +2285,10 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="H8">
-        <v>99.16</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -1624,10 +2296,10 @@
         <v>16</v>
       </c>
       <c r="B9">
-        <v>36</v>
+        <v>168</v>
       </c>
       <c r="C9">
-        <v>36</v>
+        <v>168</v>
       </c>
       <c r="D9">
         <v>100</v>
@@ -1639,7 +2311,7 @@
         <v>0</v>
       </c>
       <c r="G9">
-        <v>36</v>
+        <v>168</v>
       </c>
       <c r="H9">
         <v>100</v>
@@ -1650,10 +2322,10 @@
         <v>17</v>
       </c>
       <c r="B10">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="C10">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="D10">
         <v>100</v>
@@ -1665,7 +2337,7 @@
         <v>0</v>
       </c>
       <c r="G10">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="H10">
         <v>100</v>
@@ -1702,10 +2374,10 @@
         <v>19</v>
       </c>
       <c r="B12">
-        <v>64</v>
+        <v>119</v>
       </c>
       <c r="C12">
-        <v>64</v>
+        <v>119</v>
       </c>
       <c r="D12">
         <v>100</v>
@@ -1717,10 +2389,10 @@
         <v>0</v>
       </c>
       <c r="G12">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="H12">
-        <v>96.88</v>
+        <v>99.16</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1728,10 +2400,10 @@
         <v>20</v>
       </c>
       <c r="B13">
-        <v>163</v>
+        <v>135</v>
       </c>
       <c r="C13">
-        <v>163</v>
+        <v>135</v>
       </c>
       <c r="D13">
         <v>100</v>
@@ -1743,10 +2415,10 @@
         <v>0</v>
       </c>
       <c r="G13">
-        <v>154</v>
+        <v>135</v>
       </c>
       <c r="H13">
-        <v>94.48</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -1754,10 +2426,10 @@
         <v>21</v>
       </c>
       <c r="B14">
-        <v>129</v>
+        <v>69</v>
       </c>
       <c r="C14">
-        <v>129</v>
+        <v>69</v>
       </c>
       <c r="D14">
         <v>100</v>
@@ -1769,7 +2441,7 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <v>129</v>
+        <v>69</v>
       </c>
       <c r="H14">
         <v>100</v>
@@ -1780,10 +2452,10 @@
         <v>22</v>
       </c>
       <c r="B15">
-        <v>87</v>
+        <v>166</v>
       </c>
       <c r="C15">
-        <v>87</v>
+        <v>166</v>
       </c>
       <c r="D15">
         <v>100</v>
@@ -1795,10 +2467,10 @@
         <v>0</v>
       </c>
       <c r="G15">
-        <v>87</v>
+        <v>164</v>
       </c>
       <c r="H15">
-        <v>100</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -1806,10 +2478,10 @@
         <v>23</v>
       </c>
       <c r="B16">
-        <v>133</v>
+        <v>277</v>
       </c>
       <c r="C16">
-        <v>133</v>
+        <v>277</v>
       </c>
       <c r="D16">
         <v>100</v>
@@ -1821,7 +2493,7 @@
         <v>0</v>
       </c>
       <c r="G16">
-        <v>133</v>
+        <v>277</v>
       </c>
       <c r="H16">
         <v>100</v>
@@ -1832,10 +2504,10 @@
         <v>24</v>
       </c>
       <c r="B17">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="C17">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="D17">
         <v>100</v>
@@ -1847,7 +2519,7 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="H17">
         <v>100</v>
@@ -1858,10 +2530,10 @@
         <v>25</v>
       </c>
       <c r="B18">
-        <v>104</v>
+        <v>64</v>
       </c>
       <c r="C18">
-        <v>104</v>
+        <v>64</v>
       </c>
       <c r="D18">
         <v>100</v>
@@ -1873,10 +2545,10 @@
         <v>0</v>
       </c>
       <c r="G18">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="H18">
-        <v>100</v>
+        <v>96.88</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1884,10 +2556,10 @@
         <v>26</v>
       </c>
       <c r="B19">
-        <v>132</v>
+        <v>248</v>
       </c>
       <c r="C19">
-        <v>132</v>
+        <v>248</v>
       </c>
       <c r="D19">
         <v>100</v>
@@ -1899,7 +2571,7 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>132</v>
+        <v>248</v>
       </c>
       <c r="H19">
         <v>100</v>
@@ -1910,10 +2582,10 @@
         <v>27</v>
       </c>
       <c r="B20">
-        <v>114</v>
+        <v>163</v>
       </c>
       <c r="C20">
-        <v>114</v>
+        <v>163</v>
       </c>
       <c r="D20">
         <v>100</v>
@@ -1925,10 +2597,10 @@
         <v>0</v>
       </c>
       <c r="G20">
-        <v>111</v>
+        <v>154</v>
       </c>
       <c r="H20">
-        <v>97.37</v>
+        <v>94.48</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1936,10 +2608,10 @@
         <v>28</v>
       </c>
       <c r="B21">
-        <v>180</v>
+        <v>208</v>
       </c>
       <c r="C21">
-        <v>180</v>
+        <v>208</v>
       </c>
       <c r="D21">
         <v>100</v>
@@ -1951,10 +2623,10 @@
         <v>0</v>
       </c>
       <c r="G21">
-        <v>180</v>
+        <v>207</v>
       </c>
       <c r="H21">
-        <v>100</v>
+        <v>99.52</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1962,10 +2634,10 @@
         <v>29</v>
       </c>
       <c r="B22">
-        <v>226</v>
+        <v>62</v>
       </c>
       <c r="C22">
-        <v>226</v>
+        <v>62</v>
       </c>
       <c r="D22">
         <v>100</v>
@@ -1977,7 +2649,7 @@
         <v>0</v>
       </c>
       <c r="G22">
-        <v>226</v>
+        <v>62</v>
       </c>
       <c r="H22">
         <v>100</v>
@@ -1988,10 +2660,10 @@
         <v>30</v>
       </c>
       <c r="B23">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="C23">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="D23">
         <v>100</v>
@@ -2003,10 +2675,10 @@
         <v>0</v>
       </c>
       <c r="G23">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="H23">
-        <v>99.28</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -2014,10 +2686,10 @@
         <v>31</v>
       </c>
       <c r="B24">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="C24">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="D24">
         <v>100</v>
@@ -2029,10 +2701,10 @@
         <v>0</v>
       </c>
       <c r="G24">
-        <v>113</v>
+        <v>87</v>
       </c>
       <c r="H24">
-        <v>98.26000000000001</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -2040,10 +2712,10 @@
         <v>32</v>
       </c>
       <c r="B25">
-        <v>115</v>
+        <v>180</v>
       </c>
       <c r="C25">
-        <v>115</v>
+        <v>180</v>
       </c>
       <c r="D25">
         <v>100</v>
@@ -2055,7 +2727,7 @@
         <v>0</v>
       </c>
       <c r="G25">
-        <v>115</v>
+        <v>180</v>
       </c>
       <c r="H25">
         <v>100</v>
@@ -2066,10 +2738,10 @@
         <v>33</v>
       </c>
       <c r="B26">
-        <v>17</v>
+        <v>133</v>
       </c>
       <c r="C26">
-        <v>17</v>
+        <v>133</v>
       </c>
       <c r="D26">
         <v>100</v>
@@ -2081,7 +2753,7 @@
         <v>0</v>
       </c>
       <c r="G26">
-        <v>17</v>
+        <v>133</v>
       </c>
       <c r="H26">
         <v>100</v>
@@ -2092,10 +2764,10 @@
         <v>34</v>
       </c>
       <c r="B27">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="C27">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="D27">
         <v>100</v>
@@ -2107,7 +2779,7 @@
         <v>0</v>
       </c>
       <c r="G27">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="H27">
         <v>100</v>
@@ -2118,10 +2790,10 @@
         <v>35</v>
       </c>
       <c r="B28">
-        <v>77</v>
+        <v>186</v>
       </c>
       <c r="C28">
-        <v>77</v>
+        <v>186</v>
       </c>
       <c r="D28">
         <v>100</v>
@@ -2133,10 +2805,10 @@
         <v>0</v>
       </c>
       <c r="G28">
-        <v>77</v>
+        <v>171</v>
       </c>
       <c r="H28">
-        <v>100</v>
+        <v>91.94</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -2144,10 +2816,10 @@
         <v>36</v>
       </c>
       <c r="B29">
-        <v>63</v>
+        <v>177</v>
       </c>
       <c r="C29">
-        <v>63</v>
+        <v>177</v>
       </c>
       <c r="D29">
         <v>100</v>
@@ -2159,7 +2831,7 @@
         <v>0</v>
       </c>
       <c r="G29">
-        <v>63</v>
+        <v>177</v>
       </c>
       <c r="H29">
         <v>100</v>
@@ -2170,10 +2842,10 @@
         <v>37</v>
       </c>
       <c r="B30">
-        <v>151</v>
+        <v>104</v>
       </c>
       <c r="C30">
-        <v>151</v>
+        <v>104</v>
       </c>
       <c r="D30">
         <v>100</v>
@@ -2185,10 +2857,10 @@
         <v>0</v>
       </c>
       <c r="G30">
-        <v>150</v>
+        <v>104</v>
       </c>
       <c r="H30">
-        <v>99.34</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -2196,24 +2868,570 @@
         <v>38</v>
       </c>
       <c r="B31">
+        <v>111</v>
+      </c>
+      <c r="C31">
+        <v>111</v>
+      </c>
+      <c r="D31">
+        <v>100</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31">
+        <v>111</v>
+      </c>
+      <c r="H31">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32">
+        <v>132</v>
+      </c>
+      <c r="C32">
+        <v>132</v>
+      </c>
+      <c r="D32">
+        <v>100</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="G32">
+        <v>132</v>
+      </c>
+      <c r="H32">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33">
+        <v>159</v>
+      </c>
+      <c r="C33">
+        <v>159</v>
+      </c>
+      <c r="D33">
+        <v>100</v>
+      </c>
+      <c r="E33">
+        <v>0</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>159</v>
+      </c>
+      <c r="H33">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" t="s">
+        <v>41</v>
+      </c>
+      <c r="B34">
+        <v>114</v>
+      </c>
+      <c r="C34">
+        <v>114</v>
+      </c>
+      <c r="D34">
+        <v>100</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="G34">
+        <v>111</v>
+      </c>
+      <c r="H34">
+        <v>97.37</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35" t="s">
+        <v>42</v>
+      </c>
+      <c r="B35">
+        <v>180</v>
+      </c>
+      <c r="C35">
+        <v>180</v>
+      </c>
+      <c r="D35">
+        <v>100</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="G35">
+        <v>180</v>
+      </c>
+      <c r="H35">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" t="s">
+        <v>43</v>
+      </c>
+      <c r="B36">
+        <v>226</v>
+      </c>
+      <c r="C36">
+        <v>226</v>
+      </c>
+      <c r="D36">
+        <v>100</v>
+      </c>
+      <c r="E36">
+        <v>0</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
+      </c>
+      <c r="G36">
+        <v>226</v>
+      </c>
+      <c r="H36">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" t="s">
+        <v>44</v>
+      </c>
+      <c r="B37">
+        <v>138</v>
+      </c>
+      <c r="C37">
+        <v>138</v>
+      </c>
+      <c r="D37">
+        <v>100</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+      <c r="G37">
+        <v>137</v>
+      </c>
+      <c r="H37">
+        <v>99.28</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" t="s">
+        <v>45</v>
+      </c>
+      <c r="B38">
+        <v>125</v>
+      </c>
+      <c r="C38">
+        <v>125</v>
+      </c>
+      <c r="D38">
+        <v>100</v>
+      </c>
+      <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38">
+        <v>0</v>
+      </c>
+      <c r="G38">
+        <v>125</v>
+      </c>
+      <c r="H38">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" t="s">
+        <v>46</v>
+      </c>
+      <c r="B39">
+        <v>115</v>
+      </c>
+      <c r="C39">
+        <v>115</v>
+      </c>
+      <c r="D39">
+        <v>100</v>
+      </c>
+      <c r="E39">
+        <v>0</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="G39">
+        <v>113</v>
+      </c>
+      <c r="H39">
+        <v>98.26000000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" t="s">
+        <v>47</v>
+      </c>
+      <c r="B40">
+        <v>115</v>
+      </c>
+      <c r="C40">
+        <v>115</v>
+      </c>
+      <c r="D40">
+        <v>100</v>
+      </c>
+      <c r="E40">
+        <v>0</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40">
+        <v>115</v>
+      </c>
+      <c r="H40">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" t="s">
+        <v>48</v>
+      </c>
+      <c r="B41">
+        <v>158</v>
+      </c>
+      <c r="C41">
+        <v>158</v>
+      </c>
+      <c r="D41">
+        <v>100</v>
+      </c>
+      <c r="E41">
+        <v>0</v>
+      </c>
+      <c r="F41">
+        <v>0</v>
+      </c>
+      <c r="G41">
+        <v>158</v>
+      </c>
+      <c r="H41">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" t="s">
+        <v>49</v>
+      </c>
+      <c r="B42">
+        <v>234</v>
+      </c>
+      <c r="C42">
+        <v>234</v>
+      </c>
+      <c r="D42">
+        <v>100</v>
+      </c>
+      <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42">
+        <v>234</v>
+      </c>
+      <c r="H42">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43" t="s">
+        <v>50</v>
+      </c>
+      <c r="B43">
+        <v>17</v>
+      </c>
+      <c r="C43">
+        <v>17</v>
+      </c>
+      <c r="D43">
+        <v>100</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43">
+        <v>17</v>
+      </c>
+      <c r="H43">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44" t="s">
+        <v>51</v>
+      </c>
+      <c r="B44">
+        <v>33</v>
+      </c>
+      <c r="C44">
+        <v>33</v>
+      </c>
+      <c r="D44">
+        <v>100</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44">
+        <v>33</v>
+      </c>
+      <c r="H44">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" t="s">
+        <v>52</v>
+      </c>
+      <c r="B45">
+        <v>77</v>
+      </c>
+      <c r="C45">
+        <v>77</v>
+      </c>
+      <c r="D45">
+        <v>100</v>
+      </c>
+      <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <v>77</v>
+      </c>
+      <c r="H45">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46" t="s">
+        <v>53</v>
+      </c>
+      <c r="B46">
+        <v>63</v>
+      </c>
+      <c r="C46">
+        <v>63</v>
+      </c>
+      <c r="D46">
+        <v>100</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46">
+        <v>63</v>
+      </c>
+      <c r="H46">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47" t="s">
+        <v>54</v>
+      </c>
+      <c r="B47">
+        <v>91</v>
+      </c>
+      <c r="C47">
+        <v>91</v>
+      </c>
+      <c r="D47">
+        <v>100</v>
+      </c>
+      <c r="E47">
+        <v>0</v>
+      </c>
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47">
+        <v>91</v>
+      </c>
+      <c r="H47">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48" t="s">
+        <v>55</v>
+      </c>
+      <c r="B48">
+        <v>123</v>
+      </c>
+      <c r="C48">
+        <v>123</v>
+      </c>
+      <c r="D48">
+        <v>100</v>
+      </c>
+      <c r="E48">
+        <v>0</v>
+      </c>
+      <c r="F48">
+        <v>0</v>
+      </c>
+      <c r="G48">
+        <v>123</v>
+      </c>
+      <c r="H48">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49" t="s">
+        <v>56</v>
+      </c>
+      <c r="B49">
+        <v>172</v>
+      </c>
+      <c r="C49">
+        <v>172</v>
+      </c>
+      <c r="D49">
+        <v>100</v>
+      </c>
+      <c r="E49">
+        <v>0</v>
+      </c>
+      <c r="F49">
+        <v>0</v>
+      </c>
+      <c r="G49">
+        <v>172</v>
+      </c>
+      <c r="H49">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50" t="s">
+        <v>57</v>
+      </c>
+      <c r="B50">
+        <v>151</v>
+      </c>
+      <c r="C50">
+        <v>151</v>
+      </c>
+      <c r="D50">
+        <v>100</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+      <c r="F50">
+        <v>0</v>
+      </c>
+      <c r="G50">
+        <v>150</v>
+      </c>
+      <c r="H50">
+        <v>99.34</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" t="s">
+        <v>58</v>
+      </c>
+      <c r="B51">
         <v>103</v>
       </c>
-      <c r="C31">
+      <c r="C51">
         <v>103</v>
       </c>
-      <c r="D31">
-        <v>100</v>
-      </c>
-      <c r="E31">
-        <v>0</v>
-      </c>
-      <c r="F31">
-        <v>0</v>
-      </c>
-      <c r="G31">
+      <c r="D51">
+        <v>100</v>
+      </c>
+      <c r="E51">
+        <v>0</v>
+      </c>
+      <c r="F51">
+        <v>0</v>
+      </c>
+      <c r="G51">
         <v>103</v>
       </c>
-      <c r="H31">
+      <c r="H51">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52">
+        <v>174</v>
+      </c>
+      <c r="C52">
+        <v>174</v>
+      </c>
+      <c r="D52">
+        <v>100</v>
+      </c>
+      <c r="E52">
+        <v>0</v>
+      </c>
+      <c r="F52">
+        <v>0</v>
+      </c>
+      <c r="G52">
+        <v>174</v>
+      </c>
+      <c r="H52">
         <v>100</v>
       </c>
     </row>
@@ -2224,7 +3442,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="50.7109375" customWidth="1"/>
@@ -2293,28 +3511,28 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>130</v>
+        <v>207</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>0.77</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>119</v>
+        <v>151</v>
       </c>
       <c r="F3">
-        <v>91.54000000000001</v>
+        <v>72.95</v>
       </c>
       <c r="G3">
-        <v>10</v>
+        <v>56</v>
       </c>
       <c r="H3">
-        <v>7.69</v>
+        <v>27.05</v>
       </c>
       <c r="I3">
-        <v>8.5</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2322,7 +3540,7 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -2331,19 +3549,19 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="F4">
-        <v>100</v>
+        <v>78.56999999999999</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="I4">
-        <v>8.6</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2351,7 +3569,7 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -2360,19 +3578,19 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="F5">
-        <v>75</v>
+        <v>86.83</v>
       </c>
       <c r="G5">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="H5">
-        <v>25</v>
+        <v>13.17</v>
       </c>
       <c r="I5">
-        <v>6.9</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2380,28 +3598,28 @@
         <v>13</v>
       </c>
       <c r="B6">
-        <v>94</v>
+        <v>130</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="E6">
-        <v>77</v>
+        <v>119</v>
       </c>
       <c r="F6">
-        <v>81.91</v>
+        <v>91.54000000000001</v>
       </c>
       <c r="G6">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="H6">
-        <v>18.09</v>
+        <v>7.69</v>
       </c>
       <c r="I6">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2409,28 +3627,28 @@
         <v>14</v>
       </c>
       <c r="B7">
-        <v>3563</v>
+        <v>19</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>3026</v>
+        <v>19</v>
       </c>
       <c r="F7">
-        <v>84.93000000000001</v>
+        <v>100</v>
       </c>
       <c r="G7">
-        <v>535</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>15.02</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>7.7</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2438,28 +3656,28 @@
         <v>15</v>
       </c>
       <c r="B8">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>85</v>
+        <v>110</v>
       </c>
       <c r="F8">
-        <v>71.43000000000001</v>
+        <v>96.48999999999999</v>
       </c>
       <c r="G8">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="H8">
-        <v>27.73</v>
+        <v>3.51</v>
       </c>
       <c r="I8">
-        <v>6.9</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2467,7 +3685,7 @@
         <v>16</v>
       </c>
       <c r="B9">
-        <v>36</v>
+        <v>168</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -2476,19 +3694,19 @@
         <v>0</v>
       </c>
       <c r="E9">
-        <v>18</v>
+        <v>126</v>
       </c>
       <c r="F9">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="G9">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="H9">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="I9">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2496,7 +3714,7 @@
         <v>17</v>
       </c>
       <c r="B10">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -2505,19 +3723,19 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="F10">
-        <v>75.36</v>
+        <v>100</v>
       </c>
       <c r="G10">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>24.64</v>
+        <v>0</v>
       </c>
       <c r="I10">
-        <v>7</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -2534,19 +3752,19 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="F11">
-        <v>56.38</v>
+        <v>81.91</v>
       </c>
       <c r="G11">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="H11">
-        <v>43.62</v>
+        <v>18.09</v>
       </c>
       <c r="I11">
-        <v>6.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -2554,28 +3772,28 @@
         <v>19</v>
       </c>
       <c r="B12">
-        <v>64</v>
+        <v>119</v>
       </c>
       <c r="C12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12">
-        <v>3.13</v>
+        <v>0.84</v>
       </c>
       <c r="E12">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="F12">
-        <v>78.13</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="G12">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="H12">
-        <v>18.75</v>
+        <v>27.73</v>
       </c>
       <c r="I12">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -2583,28 +3801,28 @@
         <v>20</v>
       </c>
       <c r="B13">
-        <v>163</v>
+        <v>135</v>
       </c>
       <c r="C13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D13">
-        <v>1.23</v>
+        <v>0</v>
       </c>
       <c r="E13">
-        <v>131</v>
+        <v>57</v>
       </c>
       <c r="F13">
-        <v>80.37</v>
+        <v>42.22</v>
       </c>
       <c r="G13">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="H13">
-        <v>18.4</v>
+        <v>57.78</v>
       </c>
       <c r="I13">
-        <v>7.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -2612,7 +3830,7 @@
         <v>21</v>
       </c>
       <c r="B14">
-        <v>129</v>
+        <v>69</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -2621,19 +3839,19 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>96</v>
+        <v>52</v>
       </c>
       <c r="F14">
-        <v>74.42</v>
+        <v>75.36</v>
       </c>
       <c r="G14">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="H14">
-        <v>25.58</v>
+        <v>24.64</v>
       </c>
       <c r="I14">
-        <v>7.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -2641,7 +3859,7 @@
         <v>22</v>
       </c>
       <c r="B15">
-        <v>87</v>
+        <v>166</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -2650,19 +3868,19 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>68</v>
+        <v>133</v>
       </c>
       <c r="F15">
-        <v>78.16</v>
+        <v>80.12</v>
       </c>
       <c r="G15">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="H15">
-        <v>21.84</v>
+        <v>19.88</v>
       </c>
       <c r="I15">
-        <v>7</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -2670,7 +3888,7 @@
         <v>23</v>
       </c>
       <c r="B16">
-        <v>133</v>
+        <v>277</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -2679,19 +3897,19 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>125</v>
+        <v>247</v>
       </c>
       <c r="F16">
-        <v>93.98</v>
+        <v>89.17</v>
       </c>
       <c r="G16">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="H16">
-        <v>6.02</v>
+        <v>10.83</v>
       </c>
       <c r="I16">
-        <v>8.699999999999999</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -2699,7 +3917,7 @@
         <v>24</v>
       </c>
       <c r="B17">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -2708,19 +3926,19 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F17">
-        <v>85.25</v>
+        <v>56.38</v>
       </c>
       <c r="G17">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="H17">
-        <v>14.75</v>
+        <v>43.62</v>
       </c>
       <c r="I17">
-        <v>7.6</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -2728,25 +3946,25 @@
         <v>25</v>
       </c>
       <c r="B18">
-        <v>104</v>
+        <v>64</v>
       </c>
       <c r="C18">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>3.13</v>
       </c>
       <c r="E18">
-        <v>83</v>
+        <v>50</v>
       </c>
       <c r="F18">
-        <v>79.81</v>
+        <v>78.13</v>
       </c>
       <c r="G18">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="H18">
-        <v>20.19</v>
+        <v>18.75</v>
       </c>
       <c r="I18">
         <v>7.1</v>
@@ -2757,7 +3975,7 @@
         <v>26</v>
       </c>
       <c r="B19">
-        <v>132</v>
+        <v>248</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -2766,19 +3984,19 @@
         <v>0</v>
       </c>
       <c r="E19">
-        <v>132</v>
+        <v>167</v>
       </c>
       <c r="F19">
-        <v>100</v>
+        <v>67.34</v>
       </c>
       <c r="G19">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="H19">
-        <v>0</v>
+        <v>32.66</v>
       </c>
       <c r="I19">
-        <v>8.800000000000001</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -2786,25 +4004,25 @@
         <v>27</v>
       </c>
       <c r="B20">
-        <v>114</v>
+        <v>163</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20">
-        <v>0.88</v>
+        <v>1.23</v>
       </c>
       <c r="E20">
-        <v>89</v>
+        <v>131</v>
       </c>
       <c r="F20">
-        <v>78.06999999999999</v>
+        <v>80.37</v>
       </c>
       <c r="G20">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="H20">
-        <v>21.05</v>
+        <v>18.4</v>
       </c>
       <c r="I20">
         <v>7.2</v>
@@ -2815,28 +4033,28 @@
         <v>28</v>
       </c>
       <c r="B21">
-        <v>180</v>
+        <v>208</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>0.48</v>
       </c>
       <c r="E21">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="F21">
-        <v>90</v>
+        <v>86.06</v>
       </c>
       <c r="G21">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H21">
-        <v>10</v>
+        <v>13.46</v>
       </c>
       <c r="I21">
-        <v>7.9</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -2844,7 +4062,7 @@
         <v>29</v>
       </c>
       <c r="B22">
-        <v>226</v>
+        <v>62</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -2853,19 +4071,19 @@
         <v>0</v>
       </c>
       <c r="E22">
-        <v>194</v>
+        <v>59</v>
       </c>
       <c r="F22">
-        <v>85.84</v>
+        <v>95.16</v>
       </c>
       <c r="G22">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="H22">
-        <v>14.16</v>
+        <v>4.84</v>
       </c>
       <c r="I22">
-        <v>7</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -2873,28 +4091,28 @@
         <v>30</v>
       </c>
       <c r="B23">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="C23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D23">
-        <v>0.72</v>
+        <v>0</v>
       </c>
       <c r="E23">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="F23">
-        <v>65.22</v>
+        <v>63.71</v>
       </c>
       <c r="G23">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H23">
-        <v>34.06</v>
+        <v>36.29</v>
       </c>
       <c r="I23">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -2902,28 +4120,28 @@
         <v>31</v>
       </c>
       <c r="B24">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="C24">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D24">
-        <v>1.74</v>
+        <v>0</v>
       </c>
       <c r="E24">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="F24">
-        <v>77.39</v>
+        <v>78.16</v>
       </c>
       <c r="G24">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="H24">
-        <v>20.87</v>
+        <v>21.84</v>
       </c>
       <c r="I24">
-        <v>7.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -2931,7 +4149,7 @@
         <v>32</v>
       </c>
       <c r="B25">
-        <v>115</v>
+        <v>180</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -2940,19 +4158,19 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>100</v>
+        <v>152</v>
       </c>
       <c r="F25">
-        <v>86.95999999999999</v>
+        <v>84.44</v>
       </c>
       <c r="G25">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H25">
-        <v>13.04</v>
+        <v>15.56</v>
       </c>
       <c r="I25">
-        <v>8</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -2960,7 +4178,7 @@
         <v>33</v>
       </c>
       <c r="B26">
-        <v>17</v>
+        <v>133</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -2969,19 +4187,19 @@
         <v>0</v>
       </c>
       <c r="E26">
-        <v>17</v>
+        <v>125</v>
       </c>
       <c r="F26">
-        <v>100</v>
+        <v>93.98</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H26">
-        <v>0</v>
+        <v>6.02</v>
       </c>
       <c r="I26">
-        <v>9.199999999999999</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -2989,7 +4207,7 @@
         <v>34</v>
       </c>
       <c r="B27">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -2998,19 +4216,19 @@
         <v>0</v>
       </c>
       <c r="E27">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="F27">
-        <v>93.94</v>
+        <v>85.25</v>
       </c>
       <c r="G27">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H27">
-        <v>6.06</v>
+        <v>14.75</v>
       </c>
       <c r="I27">
-        <v>8.4</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -3018,28 +4236,28 @@
         <v>35</v>
       </c>
       <c r="B28">
-        <v>77</v>
+        <v>186</v>
       </c>
       <c r="C28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28">
-        <v>0</v>
+        <v>0.54</v>
       </c>
       <c r="E28">
-        <v>58</v>
+        <v>163</v>
       </c>
       <c r="F28">
-        <v>75.31999999999999</v>
+        <v>87.63</v>
       </c>
       <c r="G28">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="H28">
-        <v>24.68</v>
+        <v>11.83</v>
       </c>
       <c r="I28">
-        <v>6.4</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -3047,7 +4265,7 @@
         <v>36</v>
       </c>
       <c r="B29">
-        <v>63</v>
+        <v>177</v>
       </c>
       <c r="C29">
         <v>0</v>
@@ -3056,19 +4274,19 @@
         <v>0</v>
       </c>
       <c r="E29">
-        <v>62</v>
+        <v>177</v>
       </c>
       <c r="F29">
-        <v>98.41</v>
+        <v>100</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29">
-        <v>1.59</v>
+        <v>0</v>
       </c>
       <c r="I29">
-        <v>8.199999999999999</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -3076,7 +4294,7 @@
         <v>37</v>
       </c>
       <c r="B30">
-        <v>151</v>
+        <v>104</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -3085,19 +4303,19 @@
         <v>0</v>
       </c>
       <c r="E30">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="F30">
-        <v>45.7</v>
+        <v>79.81</v>
       </c>
       <c r="G30">
-        <v>82</v>
+        <v>21</v>
       </c>
       <c r="H30">
-        <v>54.3</v>
+        <v>20.19</v>
       </c>
       <c r="I30">
-        <v>6</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -3105,28 +4323,637 @@
         <v>38</v>
       </c>
       <c r="B31">
+        <v>111</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>96</v>
+      </c>
+      <c r="F31">
+        <v>86.48999999999999</v>
+      </c>
+      <c r="G31">
+        <v>15</v>
+      </c>
+      <c r="H31">
+        <v>13.51</v>
+      </c>
+      <c r="I31">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32">
+        <v>132</v>
+      </c>
+      <c r="C32">
+        <v>0</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32">
+        <v>132</v>
+      </c>
+      <c r="F32">
+        <v>100</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
+      </c>
+      <c r="I32">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33">
+        <v>159</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33">
+        <v>140</v>
+      </c>
+      <c r="F33">
+        <v>88.05</v>
+      </c>
+      <c r="G33">
+        <v>19</v>
+      </c>
+      <c r="H33">
+        <v>11.95</v>
+      </c>
+      <c r="I33">
+        <v>8.300000000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" t="s">
+        <v>41</v>
+      </c>
+      <c r="B34">
+        <v>114</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="D34">
+        <v>0.88</v>
+      </c>
+      <c r="E34">
+        <v>89</v>
+      </c>
+      <c r="F34">
+        <v>78.06999999999999</v>
+      </c>
+      <c r="G34">
+        <v>24</v>
+      </c>
+      <c r="H34">
+        <v>21.05</v>
+      </c>
+      <c r="I34">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" t="s">
+        <v>42</v>
+      </c>
+      <c r="B35">
+        <v>180</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>162</v>
+      </c>
+      <c r="F35">
+        <v>90</v>
+      </c>
+      <c r="G35">
+        <v>18</v>
+      </c>
+      <c r="H35">
+        <v>10</v>
+      </c>
+      <c r="I35">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" t="s">
+        <v>43</v>
+      </c>
+      <c r="B36">
+        <v>226</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36">
+        <v>194</v>
+      </c>
+      <c r="F36">
+        <v>85.84</v>
+      </c>
+      <c r="G36">
+        <v>32</v>
+      </c>
+      <c r="H36">
+        <v>14.16</v>
+      </c>
+      <c r="I36">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" t="s">
+        <v>44</v>
+      </c>
+      <c r="B37">
+        <v>138</v>
+      </c>
+      <c r="C37">
+        <v>1</v>
+      </c>
+      <c r="D37">
+        <v>0.72</v>
+      </c>
+      <c r="E37">
+        <v>90</v>
+      </c>
+      <c r="F37">
+        <v>65.22</v>
+      </c>
+      <c r="G37">
+        <v>47</v>
+      </c>
+      <c r="H37">
+        <v>34.06</v>
+      </c>
+      <c r="I37">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" t="s">
+        <v>45</v>
+      </c>
+      <c r="B38">
+        <v>125</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>110</v>
+      </c>
+      <c r="F38">
+        <v>88</v>
+      </c>
+      <c r="G38">
+        <v>15</v>
+      </c>
+      <c r="H38">
+        <v>12</v>
+      </c>
+      <c r="I38">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" t="s">
+        <v>46</v>
+      </c>
+      <c r="B39">
+        <v>115</v>
+      </c>
+      <c r="C39">
+        <v>2</v>
+      </c>
+      <c r="D39">
+        <v>1.74</v>
+      </c>
+      <c r="E39">
+        <v>89</v>
+      </c>
+      <c r="F39">
+        <v>77.39</v>
+      </c>
+      <c r="G39">
+        <v>24</v>
+      </c>
+      <c r="H39">
+        <v>20.87</v>
+      </c>
+      <c r="I39">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" t="s">
+        <v>47</v>
+      </c>
+      <c r="B40">
+        <v>115</v>
+      </c>
+      <c r="C40">
+        <v>0</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40">
+        <v>100</v>
+      </c>
+      <c r="F40">
+        <v>86.95999999999999</v>
+      </c>
+      <c r="G40">
+        <v>15</v>
+      </c>
+      <c r="H40">
+        <v>13.04</v>
+      </c>
+      <c r="I40">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" t="s">
+        <v>48</v>
+      </c>
+      <c r="B41">
+        <v>158</v>
+      </c>
+      <c r="C41">
+        <v>0</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>134</v>
+      </c>
+      <c r="F41">
+        <v>84.81</v>
+      </c>
+      <c r="G41">
+        <v>24</v>
+      </c>
+      <c r="H41">
+        <v>15.19</v>
+      </c>
+      <c r="I41">
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" t="s">
+        <v>49</v>
+      </c>
+      <c r="B42">
+        <v>234</v>
+      </c>
+      <c r="C42">
+        <v>0</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>220</v>
+      </c>
+      <c r="F42">
+        <v>94.02</v>
+      </c>
+      <c r="G42">
+        <v>14</v>
+      </c>
+      <c r="H42">
+        <v>5.98</v>
+      </c>
+      <c r="I42">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" t="s">
+        <v>50</v>
+      </c>
+      <c r="B43">
+        <v>17</v>
+      </c>
+      <c r="C43">
+        <v>0</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="E43">
+        <v>17</v>
+      </c>
+      <c r="F43">
+        <v>100</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+      <c r="H43">
+        <v>0</v>
+      </c>
+      <c r="I43">
+        <v>9.199999999999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" t="s">
+        <v>51</v>
+      </c>
+      <c r="B44">
+        <v>33</v>
+      </c>
+      <c r="C44">
+        <v>0</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>31</v>
+      </c>
+      <c r="F44">
+        <v>93.94</v>
+      </c>
+      <c r="G44">
+        <v>2</v>
+      </c>
+      <c r="H44">
+        <v>6.06</v>
+      </c>
+      <c r="I44">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" t="s">
+        <v>52</v>
+      </c>
+      <c r="B45">
+        <v>77</v>
+      </c>
+      <c r="C45">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45">
+        <v>58</v>
+      </c>
+      <c r="F45">
+        <v>75.31999999999999</v>
+      </c>
+      <c r="G45">
+        <v>19</v>
+      </c>
+      <c r="H45">
+        <v>24.68</v>
+      </c>
+      <c r="I45">
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" t="s">
+        <v>53</v>
+      </c>
+      <c r="B46">
+        <v>63</v>
+      </c>
+      <c r="C46">
+        <v>0</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46">
+        <v>62</v>
+      </c>
+      <c r="F46">
+        <v>98.41</v>
+      </c>
+      <c r="G46">
+        <v>1</v>
+      </c>
+      <c r="H46">
+        <v>1.59</v>
+      </c>
+      <c r="I46">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" t="s">
+        <v>54</v>
+      </c>
+      <c r="B47">
+        <v>91</v>
+      </c>
+      <c r="C47">
+        <v>0</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47">
+        <v>78</v>
+      </c>
+      <c r="F47">
+        <v>85.70999999999999</v>
+      </c>
+      <c r="G47">
+        <v>13</v>
+      </c>
+      <c r="H47">
+        <v>14.29</v>
+      </c>
+      <c r="I47">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" t="s">
+        <v>55</v>
+      </c>
+      <c r="B48">
+        <v>123</v>
+      </c>
+      <c r="C48">
+        <v>0</v>
+      </c>
+      <c r="D48">
+        <v>0</v>
+      </c>
+      <c r="E48">
+        <v>113</v>
+      </c>
+      <c r="F48">
+        <v>91.87</v>
+      </c>
+      <c r="G48">
+        <v>10</v>
+      </c>
+      <c r="H48">
+        <v>8.130000000000001</v>
+      </c>
+      <c r="I48">
+        <v>8.699999999999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" t="s">
+        <v>56</v>
+      </c>
+      <c r="B49">
+        <v>172</v>
+      </c>
+      <c r="C49">
+        <v>0</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+      <c r="E49">
+        <v>141</v>
+      </c>
+      <c r="F49">
+        <v>81.98</v>
+      </c>
+      <c r="G49">
+        <v>31</v>
+      </c>
+      <c r="H49">
+        <v>18.02</v>
+      </c>
+      <c r="I49">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" t="s">
+        <v>57</v>
+      </c>
+      <c r="B50">
+        <v>151</v>
+      </c>
+      <c r="C50">
+        <v>0</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50">
+        <v>69</v>
+      </c>
+      <c r="F50">
+        <v>45.7</v>
+      </c>
+      <c r="G50">
+        <v>82</v>
+      </c>
+      <c r="H50">
+        <v>54.3</v>
+      </c>
+      <c r="I50">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9">
+      <c r="A51" t="s">
+        <v>58</v>
+      </c>
+      <c r="B51">
         <v>103</v>
       </c>
-      <c r="C31">
-        <v>0</v>
-      </c>
-      <c r="D31">
-        <v>0</v>
-      </c>
-      <c r="E31">
+      <c r="C51">
+        <v>0</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51">
         <v>66</v>
       </c>
-      <c r="F31">
+      <c r="F51">
         <v>64.08</v>
       </c>
-      <c r="G31">
+      <c r="G51">
         <v>37</v>
       </c>
-      <c r="H31">
+      <c r="H51">
         <v>35.92</v>
       </c>
-      <c r="I31">
+      <c r="I51">
         <v>6.8</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52">
+        <v>174</v>
+      </c>
+      <c r="C52">
+        <v>0</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52">
+        <v>174</v>
+      </c>
+      <c r="F52">
+        <v>100</v>
+      </c>
+      <c r="G52">
+        <v>0</v>
+      </c>
+      <c r="H52">
+        <v>0</v>
+      </c>
+      <c r="I52">
+        <v>9.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>